<commit_message>
Levantamiento de Observaciones Incidentes 12/06/2020
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/Incidentes/Investigacion/JU-MAP-STD-001.F02_Investigación final de incidente ambiental_V00.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/Incidentes/Investigacion/JU-MAP-STD-001.F02_Investigación final de incidente ambiental_V00.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Tablas Maestras\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\Incidentes\Investigacion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\PruebaMerge3y4\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\Incidentes\Investigacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C4C6B20-8637-4700-B5B4-D9E5706F9269}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB28612F-D37B-4E3A-89D6-27B188EC3D13}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3793,12 +3793,6 @@
     <t>Zorro costeño</t>
   </si>
   <si>
-    <t>Área de suelo afectada:</t>
-  </si>
-  <si>
-    <t>Cantidad de suelo impactado:</t>
-  </si>
-  <si>
     <t>Cancha de volatización</t>
   </si>
   <si>
@@ -3835,12 +3829,6 @@
     <t>Empresa</t>
   </si>
   <si>
-    <t>Cantidad de Residuos Sólidos Generados</t>
-  </si>
-  <si>
-    <t>Volumen de residuos generdos:</t>
-  </si>
-  <si>
     <t>3.4 Impactos Ambientales o daños derivados del incidente</t>
   </si>
   <si>
@@ -3911,6 +3899,18 @@
   </si>
   <si>
     <t>Cantidad de producto no recuperado</t>
+  </si>
+  <si>
+    <t>Área afectada:</t>
+  </si>
+  <si>
+    <t>Cantidad de tierra impregnada:</t>
+  </si>
+  <si>
+    <t>Cantidad Total de Residuos Sólidos Generados:</t>
+  </si>
+  <si>
+    <t>Cantidad Total de Residuos Líquidos Generados:</t>
   </si>
 </sst>
 </file>
@@ -4878,9 +4878,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -4889,6 +4886,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -7242,7 +7242,7 @@
       <c r="K12" s="199"/>
       <c r="L12" s="199"/>
       <c r="M12" s="199"/>
-      <c r="N12" s="171" t="s">
+      <c r="N12" s="170" t="s">
         <v>441</v>
       </c>
       <c r="O12" s="199"/>
@@ -7362,7 +7362,7 @@
       <c r="K15" s="199"/>
       <c r="L15" s="199"/>
       <c r="M15" s="199"/>
-      <c r="N15" s="171" t="s">
+      <c r="N15" s="170" t="s">
         <v>441</v>
       </c>
       <c r="O15" s="199"/>
@@ -8914,7 +8914,7 @@
     <row r="25" spans="1:271" ht="23.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="194" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="C25" s="194"/>
       <c r="D25" s="194"/>
@@ -9179,9 +9179,9 @@
       <c r="JG25" s="2"/>
       <c r="JH25" s="2"/>
     </row>
-    <row r="26" spans="1:271" ht="34.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:271" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
-      <c r="B26" s="170" t="s">
+      <c r="B26" s="169" t="s">
         <v>662</v>
       </c>
       <c r="C26" s="199"/>
@@ -9450,10 +9450,10 @@
     <row r="27" spans="1:271" ht="34.35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
       <c r="B27" s="167" t="s">
-        <v>713</v>
+        <v>709</v>
       </c>
       <c r="C27" s="209" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
       <c r="D27" s="209"/>
       <c r="E27" s="209"/>
@@ -9469,7 +9469,7 @@
       <c r="O27" s="209"/>
       <c r="P27" s="209"/>
       <c r="Q27" s="207" t="s">
-        <v>715</v>
+        <v>711</v>
       </c>
       <c r="R27" s="207"/>
       <c r="S27" s="207"/>
@@ -9488,7 +9488,7 @@
       <c r="AB27" s="208"/>
       <c r="AC27" s="208"/>
       <c r="AD27" s="173" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="AE27" s="173"/>
       <c r="AF27" s="173"/>
@@ -9728,7 +9728,7 @@
     <row r="28" spans="1:271" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
       <c r="B28" s="194" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="C28" s="194"/>
       <c r="D28" s="194"/>
@@ -9993,10 +9993,10 @@
       <c r="JG28" s="2"/>
       <c r="JH28" s="2"/>
     </row>
-    <row r="29" spans="1:271" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:271" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1"/>
-      <c r="B29" s="168" t="s">
-        <v>716</v>
+      <c r="B29" s="171" t="s">
+        <v>712</v>
       </c>
       <c r="C29" s="206" t="s">
         <v>474</v>
@@ -10007,30 +10007,30 @@
       <c r="G29" s="206"/>
       <c r="H29" s="206"/>
       <c r="I29" s="206" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
       <c r="J29" s="206"/>
       <c r="K29" s="206"/>
       <c r="L29" s="206"/>
       <c r="M29" s="206" t="s">
-        <v>718</v>
+        <v>714</v>
       </c>
       <c r="N29" s="206"/>
       <c r="O29" s="206"/>
       <c r="P29" s="206" t="s">
-        <v>719</v>
+        <v>715</v>
       </c>
       <c r="Q29" s="206"/>
       <c r="R29" s="206"/>
       <c r="S29" s="206"/>
       <c r="T29" s="206" t="s">
-        <v>701</v>
+        <v>697</v>
       </c>
       <c r="U29" s="206"/>
       <c r="V29" s="206"/>
       <c r="W29" s="206"/>
       <c r="X29" s="206" t="s">
-        <v>720</v>
+        <v>716</v>
       </c>
       <c r="Y29" s="206"/>
       <c r="Z29" s="206"/>
@@ -10038,7 +10038,7 @@
       <c r="AB29" s="206"/>
       <c r="AC29" s="206"/>
       <c r="AD29" s="206" t="s">
-        <v>721</v>
+        <v>717</v>
       </c>
       <c r="AE29" s="206"/>
       <c r="AF29" s="206"/>
@@ -10278,7 +10278,7 @@
     <row r="30" spans="1:271" ht="22.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1"/>
       <c r="B30" s="194" t="s">
-        <v>698</v>
+        <v>694</v>
       </c>
       <c r="C30" s="194"/>
       <c r="D30" s="194"/>
@@ -10545,7 +10545,7 @@
     </row>
     <row r="31" spans="1:271" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1"/>
-      <c r="B31" s="169" t="s">
+      <c r="B31" s="168" t="s">
         <v>1</v>
       </c>
       <c r="C31" s="196" t="s">
@@ -10557,7 +10557,7 @@
       <c r="G31" s="174"/>
       <c r="H31" s="174"/>
       <c r="I31" s="180" t="s">
-        <v>682</v>
+        <v>718</v>
       </c>
       <c r="J31" s="180"/>
       <c r="K31" s="180"/>
@@ -10567,7 +10567,7 @@
       <c r="O31" s="181"/>
       <c r="P31" s="181"/>
       <c r="Q31" s="180" t="s">
-        <v>683</v>
+        <v>719</v>
       </c>
       <c r="R31" s="180"/>
       <c r="S31" s="180"/>
@@ -10821,7 +10821,7 @@
     </row>
     <row r="32" spans="1:271" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1"/>
-      <c r="B32" s="169" t="s">
+      <c r="B32" s="168" t="s">
         <v>3</v>
       </c>
       <c r="C32" s="180" t="s">
@@ -10833,7 +10833,7 @@
       <c r="G32" s="174"/>
       <c r="H32" s="174"/>
       <c r="I32" s="197" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="J32" s="197"/>
       <c r="K32" s="197"/>
@@ -11097,7 +11097,7 @@
     </row>
     <row r="33" spans="1:268" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1"/>
-      <c r="B33" s="169" t="s">
+      <c r="B33" s="168" t="s">
         <v>4</v>
       </c>
       <c r="C33" s="180" t="s">
@@ -11385,7 +11385,7 @@
       <c r="G34" s="174"/>
       <c r="H34" s="174"/>
       <c r="I34" s="180" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="J34" s="180"/>
       <c r="K34" s="180"/>
@@ -11649,8 +11649,8 @@
     </row>
     <row r="35" spans="1:268" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1"/>
-      <c r="B35" s="169" t="s">
-        <v>691</v>
+      <c r="B35" s="168" t="s">
+        <v>689</v>
       </c>
       <c r="C35" s="175"/>
       <c r="D35" s="175"/>
@@ -11659,7 +11659,7 @@
       <c r="G35" s="175"/>
       <c r="H35" s="175"/>
       <c r="I35" s="180" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="J35" s="180"/>
       <c r="K35" s="180"/>
@@ -11925,7 +11925,7 @@
     </row>
     <row r="36" spans="1:268" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1"/>
-      <c r="B36" s="169" t="s">
+      <c r="B36" s="168" t="s">
         <v>567</v>
       </c>
       <c r="C36" s="180" t="s">
@@ -12195,10 +12195,10 @@
       <c r="JG36" s="2"/>
       <c r="JH36" s="2"/>
     </row>
-    <row r="37" spans="1:268" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:268" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A37" s="1"/>
       <c r="B37" s="150" t="s">
-        <v>696</v>
+        <v>720</v>
       </c>
       <c r="C37" s="203"/>
       <c r="D37" s="203"/>
@@ -12211,7 +12211,7 @@
       <c r="K37" s="204"/>
       <c r="L37" s="204"/>
       <c r="M37" s="205" t="s">
-        <v>697</v>
+        <v>721</v>
       </c>
       <c r="N37" s="205"/>
       <c r="O37" s="205"/>
@@ -12224,7 +12224,7 @@
       <c r="V37" s="201"/>
       <c r="W37" s="201"/>
       <c r="X37" s="202" t="s">
-        <v>700</v>
+        <v>696</v>
       </c>
       <c r="Y37" s="202"/>
       <c r="Z37" s="202"/>
@@ -12783,13 +12783,13 @@
       <c r="T46" s="173"/>
       <c r="U46" s="173"/>
       <c r="V46" s="176" t="s">
-        <v>712</v>
+        <v>708</v>
       </c>
       <c r="W46" s="177"/>
       <c r="X46" s="177"/>
       <c r="Y46" s="178"/>
       <c r="Z46" s="176" t="s">
-        <v>706</v>
+        <v>702</v>
       </c>
       <c r="AA46" s="177"/>
       <c r="AB46" s="177"/>
@@ -12863,13 +12863,13 @@
       <c r="T48" s="173"/>
       <c r="U48" s="173"/>
       <c r="V48" s="176" t="s">
-        <v>712</v>
+        <v>708</v>
       </c>
       <c r="W48" s="177"/>
       <c r="X48" s="177"/>
       <c r="Y48" s="178"/>
       <c r="Z48" s="176" t="s">
-        <v>706</v>
+        <v>702</v>
       </c>
       <c r="AA48" s="177"/>
       <c r="AB48" s="177"/>
@@ -12883,7 +12883,7 @@
     </row>
     <row r="49" spans="2:33" x14ac:dyDescent="0.2">
       <c r="B49" s="191" t="s">
-        <v>708</v>
+        <v>704</v>
       </c>
       <c r="C49" s="192"/>
       <c r="D49" s="192"/>
@@ -13023,7 +13023,7 @@
     </row>
     <row r="53" spans="2:33" x14ac:dyDescent="0.2">
       <c r="B53" s="198" t="s">
-        <v>707</v>
+        <v>703</v>
       </c>
       <c r="C53" s="198"/>
       <c r="D53" s="198"/>
@@ -13411,7 +13411,7 @@
       </c>
       <c r="G3" s="67"/>
       <c r="H3" s="67" t="s">
-        <v>704</v>
+        <v>700</v>
       </c>
       <c r="J3" s="69">
         <v>1</v>
@@ -13497,10 +13497,10 @@
       <c r="P4" s="93"/>
       <c r="Q4" s="93"/>
       <c r="R4" s="156" t="s">
-        <v>709</v>
+        <v>705</v>
       </c>
       <c r="S4" s="162" t="s">
-        <v>710</v>
+        <v>706</v>
       </c>
       <c r="T4" s="165" t="str">
         <f>_xlfn.CONCAT($R$4,H4,CHAR(39),$S$4)</f>
@@ -14495,7 +14495,7 @@
         <v>47</v>
       </c>
       <c r="X21" s="106" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="Z21" s="113" t="s">
         <v>606</v>
@@ -14550,7 +14550,7 @@
         <v>93</v>
       </c>
       <c r="X22" s="106" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="Y22" s="101"/>
       <c r="AA22" s="101"/>
@@ -15332,7 +15332,7 @@
         <v>511</v>
       </c>
       <c r="AB37" s="55" t="s">
-        <v>699</v>
+        <v>695</v>
       </c>
     </row>
     <row r="38" spans="1:28" x14ac:dyDescent="0.25">
@@ -15824,7 +15824,7 @@
       </c>
       <c r="U48" s="119"/>
       <c r="X48" s="64" t="s">
-        <v>701</v>
+        <v>697</v>
       </c>
       <c r="Z48" s="123" t="s">
         <v>522</v>
@@ -15878,7 +15878,7 @@
       </c>
       <c r="U49" s="119"/>
       <c r="X49" s="122" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="Z49" s="123" t="s">
         <v>523</v>
@@ -15920,7 +15920,7 @@
       </c>
       <c r="U50" s="119"/>
       <c r="X50" s="122" t="s">
-        <v>703</v>
+        <v>699</v>
       </c>
       <c r="Z50" s="123" t="s">
         <v>524</v>
@@ -16161,7 +16161,7 @@
         <v>530</v>
       </c>
       <c r="AB56" s="64" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
     </row>
     <row r="57" spans="3:28" x14ac:dyDescent="0.25">
@@ -16200,7 +16200,7 @@
         <v>531</v>
       </c>
       <c r="AB57" s="109" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
     </row>
     <row r="58" spans="3:28" x14ac:dyDescent="0.25">
@@ -16239,7 +16239,7 @@
         <v>532</v>
       </c>
       <c r="AB58" s="106" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
     </row>
     <row r="59" spans="3:28" x14ac:dyDescent="0.25">
@@ -16928,7 +16928,7 @@
       </c>
       <c r="G78" s="126"/>
       <c r="H78" s="127" t="s">
-        <v>705</v>
+        <v>701</v>
       </c>
       <c r="I78" s="97"/>
       <c r="J78" s="97"/>
@@ -16937,10 +16937,10 @@
       </c>
       <c r="L78" s="118"/>
       <c r="R78" s="156" t="s">
-        <v>709</v>
+        <v>705</v>
       </c>
       <c r="S78" s="162" t="s">
-        <v>711</v>
+        <v>707</v>
       </c>
       <c r="U78" s="119"/>
     </row>

</xml_diff>

<commit_message>
Levantamiento de observaciones 17/06/2020. Listo para publicación
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/Incidentes/Investigacion/JU-MAP-STD-001.F02_Investigación final de incidente ambiental_V00.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/Incidentes/Investigacion/JU-MAP-STD-001.F02_Investigación final de incidente ambiental_V00.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\PruebaMerge3y4\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\Incidentes\Investigacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB28612F-D37B-4E3A-89D6-27B188EC3D13}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB6EA616-C00A-4CE0-A304-CEFF8B0C8526}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IFIA" sheetId="3" r:id="rId1"/>
-    <sheet name="Tablas" sheetId="2" r:id="rId2"/>
-    <sheet name="Causas" sheetId="4" r:id="rId3"/>
+    <sheet name="Tablas" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="Causas" sheetId="4" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">IFIA!$B$2:$AG$52</definedName>
@@ -4890,17 +4890,185 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4911,178 +5079,10 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -5652,40 +5652,40 @@
     <row r="1" spans="1:271" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="1:271" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
-      <c r="B2" s="224"/>
-      <c r="C2" s="227" t="s">
+      <c r="B2" s="202"/>
+      <c r="C2" s="205" t="s">
         <v>604</v>
       </c>
-      <c r="D2" s="228"/>
-      <c r="E2" s="228"/>
-      <c r="F2" s="228"/>
-      <c r="G2" s="228"/>
-      <c r="H2" s="228"/>
-      <c r="I2" s="228"/>
-      <c r="J2" s="228"/>
-      <c r="K2" s="228"/>
-      <c r="L2" s="228"/>
-      <c r="M2" s="228"/>
-      <c r="N2" s="228"/>
-      <c r="O2" s="228"/>
-      <c r="P2" s="228"/>
-      <c r="Q2" s="228"/>
-      <c r="R2" s="228"/>
-      <c r="S2" s="228"/>
-      <c r="T2" s="228"/>
-      <c r="U2" s="228"/>
-      <c r="V2" s="228"/>
-      <c r="W2" s="228"/>
-      <c r="X2" s="228"/>
-      <c r="Y2" s="228"/>
-      <c r="Z2" s="228"/>
-      <c r="AA2" s="228"/>
-      <c r="AB2" s="228"/>
-      <c r="AC2" s="231"/>
-      <c r="AD2" s="231"/>
-      <c r="AE2" s="231"/>
-      <c r="AF2" s="231"/>
-      <c r="AG2" s="231"/>
+      <c r="D2" s="206"/>
+      <c r="E2" s="206"/>
+      <c r="F2" s="206"/>
+      <c r="G2" s="206"/>
+      <c r="H2" s="206"/>
+      <c r="I2" s="206"/>
+      <c r="J2" s="206"/>
+      <c r="K2" s="206"/>
+      <c r="L2" s="206"/>
+      <c r="M2" s="206"/>
+      <c r="N2" s="206"/>
+      <c r="O2" s="206"/>
+      <c r="P2" s="206"/>
+      <c r="Q2" s="206"/>
+      <c r="R2" s="206"/>
+      <c r="S2" s="206"/>
+      <c r="T2" s="206"/>
+      <c r="U2" s="206"/>
+      <c r="V2" s="206"/>
+      <c r="W2" s="206"/>
+      <c r="X2" s="206"/>
+      <c r="Y2" s="206"/>
+      <c r="Z2" s="206"/>
+      <c r="AA2" s="206"/>
+      <c r="AB2" s="206"/>
+      <c r="AC2" s="209"/>
+      <c r="AD2" s="209"/>
+      <c r="AE2" s="209"/>
+      <c r="AF2" s="209"/>
+      <c r="AG2" s="209"/>
       <c r="AH2" s="2"/>
       <c r="AI2" s="2"/>
       <c r="AJ2" s="2"/>
@@ -5923,50 +5923,50 @@
     </row>
     <row r="3" spans="1:271" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
-      <c r="B3" s="224"/>
-      <c r="C3" s="221" t="s">
+      <c r="B3" s="202"/>
+      <c r="C3" s="199" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="222"/>
-      <c r="E3" s="222"/>
-      <c r="F3" s="229" t="s">
+      <c r="D3" s="200"/>
+      <c r="E3" s="200"/>
+      <c r="F3" s="207" t="s">
         <v>607</v>
       </c>
-      <c r="G3" s="229"/>
-      <c r="H3" s="229"/>
-      <c r="I3" s="229"/>
-      <c r="J3" s="229"/>
-      <c r="K3" s="229"/>
-      <c r="L3" s="230"/>
-      <c r="M3" s="210" t="s">
+      <c r="G3" s="207"/>
+      <c r="H3" s="207"/>
+      <c r="I3" s="207"/>
+      <c r="J3" s="207"/>
+      <c r="K3" s="207"/>
+      <c r="L3" s="208"/>
+      <c r="M3" s="188" t="s">
         <v>10</v>
       </c>
-      <c r="N3" s="211"/>
-      <c r="O3" s="211"/>
-      <c r="P3" s="212">
+      <c r="N3" s="189"/>
+      <c r="O3" s="189"/>
+      <c r="P3" s="191">
         <v>43831</v>
       </c>
-      <c r="Q3" s="213"/>
-      <c r="R3" s="213"/>
-      <c r="S3" s="214"/>
+      <c r="Q3" s="192"/>
+      <c r="R3" s="192"/>
+      <c r="S3" s="193"/>
       <c r="T3" s="3" t="s">
         <v>9</v>
       </c>
       <c r="U3" s="37"/>
-      <c r="V3" s="211">
+      <c r="V3" s="189">
         <v>0</v>
       </c>
-      <c r="W3" s="211"/>
-      <c r="X3" s="211"/>
-      <c r="Y3" s="211"/>
-      <c r="Z3" s="211"/>
-      <c r="AA3" s="211"/>
-      <c r="AB3" s="211"/>
-      <c r="AC3" s="231"/>
-      <c r="AD3" s="231"/>
-      <c r="AE3" s="231"/>
-      <c r="AF3" s="231"/>
-      <c r="AG3" s="231"/>
+      <c r="W3" s="189"/>
+      <c r="X3" s="189"/>
+      <c r="Y3" s="189"/>
+      <c r="Z3" s="189"/>
+      <c r="AA3" s="189"/>
+      <c r="AB3" s="189"/>
+      <c r="AC3" s="209"/>
+      <c r="AD3" s="209"/>
+      <c r="AE3" s="209"/>
+      <c r="AF3" s="209"/>
+      <c r="AG3" s="209"/>
       <c r="AI3" s="2"/>
       <c r="AK3" s="2"/>
       <c r="AL3" s="2"/>
@@ -6202,50 +6202,50 @@
     </row>
     <row r="4" spans="1:271" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
-      <c r="B4" s="224"/>
-      <c r="C4" s="221" t="s">
+      <c r="B4" s="202"/>
+      <c r="C4" s="199" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="222"/>
-      <c r="E4" s="222" t="s">
+      <c r="D4" s="200"/>
+      <c r="E4" s="200" t="s">
         <v>376</v>
       </c>
-      <c r="F4" s="222"/>
-      <c r="G4" s="222"/>
-      <c r="H4" s="222"/>
-      <c r="I4" s="222"/>
-      <c r="J4" s="222"/>
-      <c r="K4" s="222"/>
-      <c r="L4" s="223"/>
-      <c r="M4" s="210" t="s">
+      <c r="F4" s="200"/>
+      <c r="G4" s="200"/>
+      <c r="H4" s="200"/>
+      <c r="I4" s="200"/>
+      <c r="J4" s="200"/>
+      <c r="K4" s="200"/>
+      <c r="L4" s="201"/>
+      <c r="M4" s="188" t="s">
         <v>0</v>
       </c>
-      <c r="N4" s="211"/>
-      <c r="O4" s="211">
+      <c r="N4" s="189"/>
+      <c r="O4" s="189">
         <v>1</v>
       </c>
-      <c r="P4" s="211"/>
-      <c r="Q4" s="211"/>
-      <c r="R4" s="211"/>
-      <c r="S4" s="215"/>
-      <c r="T4" s="219" t="s">
+      <c r="P4" s="189"/>
+      <c r="Q4" s="189"/>
+      <c r="R4" s="189"/>
+      <c r="S4" s="194"/>
+      <c r="T4" s="197" t="s">
         <v>11</v>
       </c>
-      <c r="U4" s="220"/>
-      <c r="V4" s="220"/>
-      <c r="W4" s="220"/>
-      <c r="X4" s="220"/>
-      <c r="Y4" s="225">
+      <c r="U4" s="198"/>
+      <c r="V4" s="198"/>
+      <c r="W4" s="198"/>
+      <c r="X4" s="198"/>
+      <c r="Y4" s="203">
         <v>43818</v>
       </c>
-      <c r="Z4" s="226"/>
-      <c r="AA4" s="226"/>
-      <c r="AB4" s="226"/>
-      <c r="AC4" s="231"/>
-      <c r="AD4" s="231"/>
-      <c r="AE4" s="231"/>
-      <c r="AF4" s="231"/>
-      <c r="AG4" s="231"/>
+      <c r="Z4" s="204"/>
+      <c r="AA4" s="204"/>
+      <c r="AB4" s="204"/>
+      <c r="AC4" s="209"/>
+      <c r="AD4" s="209"/>
+      <c r="AE4" s="209"/>
+      <c r="AF4" s="209"/>
+      <c r="AG4" s="209"/>
       <c r="AI4" s="2"/>
       <c r="AK4" s="2"/>
       <c r="AL4" s="2"/>
@@ -6747,40 +6747,40 @@
       <c r="JK5" s="2"/>
     </row>
     <row r="6" spans="1:271" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="218" t="s">
+      <c r="B6" s="196" t="s">
         <v>470</v>
       </c>
-      <c r="C6" s="218"/>
-      <c r="D6" s="218"/>
-      <c r="E6" s="218"/>
-      <c r="F6" s="218"/>
-      <c r="G6" s="218"/>
-      <c r="H6" s="218"/>
-      <c r="I6" s="218"/>
-      <c r="J6" s="218"/>
-      <c r="K6" s="218"/>
-      <c r="L6" s="218"/>
-      <c r="M6" s="218"/>
-      <c r="N6" s="218"/>
-      <c r="O6" s="218"/>
-      <c r="P6" s="218"/>
-      <c r="Q6" s="218"/>
-      <c r="R6" s="218"/>
-      <c r="S6" s="218"/>
-      <c r="T6" s="218"/>
-      <c r="U6" s="218"/>
-      <c r="V6" s="218"/>
-      <c r="W6" s="218"/>
-      <c r="X6" s="218"/>
-      <c r="Y6" s="218"/>
-      <c r="Z6" s="218"/>
-      <c r="AA6" s="218"/>
-      <c r="AB6" s="218"/>
-      <c r="AC6" s="218"/>
-      <c r="AD6" s="218"/>
-      <c r="AE6" s="218"/>
-      <c r="AF6" s="218"/>
-      <c r="AG6" s="218"/>
+      <c r="C6" s="196"/>
+      <c r="D6" s="196"/>
+      <c r="E6" s="196"/>
+      <c r="F6" s="196"/>
+      <c r="G6" s="196"/>
+      <c r="H6" s="196"/>
+      <c r="I6" s="196"/>
+      <c r="J6" s="196"/>
+      <c r="K6" s="196"/>
+      <c r="L6" s="196"/>
+      <c r="M6" s="196"/>
+      <c r="N6" s="196"/>
+      <c r="O6" s="196"/>
+      <c r="P6" s="196"/>
+      <c r="Q6" s="196"/>
+      <c r="R6" s="196"/>
+      <c r="S6" s="196"/>
+      <c r="T6" s="196"/>
+      <c r="U6" s="196"/>
+      <c r="V6" s="196"/>
+      <c r="W6" s="196"/>
+      <c r="X6" s="196"/>
+      <c r="Y6" s="196"/>
+      <c r="Z6" s="196"/>
+      <c r="AA6" s="196"/>
+      <c r="AB6" s="196"/>
+      <c r="AC6" s="196"/>
+      <c r="AD6" s="196"/>
+      <c r="AE6" s="196"/>
+      <c r="AF6" s="196"/>
+      <c r="AG6" s="196"/>
       <c r="AH6" s="2"/>
       <c r="AI6" s="2"/>
       <c r="AK6" s="2"/>
@@ -6789,51 +6789,51 @@
       <c r="B7" s="139" t="s">
         <v>440</v>
       </c>
-      <c r="C7" s="199" t="s">
+      <c r="C7" s="174" t="s">
         <v>609</v>
       </c>
-      <c r="D7" s="199"/>
-      <c r="E7" s="199"/>
-      <c r="F7" s="199"/>
-      <c r="G7" s="199"/>
-      <c r="H7" s="199"/>
-      <c r="I7" s="199"/>
-      <c r="J7" s="199"/>
-      <c r="K7" s="172" t="s">
+      <c r="D7" s="174"/>
+      <c r="E7" s="174"/>
+      <c r="F7" s="174"/>
+      <c r="G7" s="174"/>
+      <c r="H7" s="174"/>
+      <c r="I7" s="174"/>
+      <c r="J7" s="174"/>
+      <c r="K7" s="183" t="s">
         <v>443</v>
       </c>
-      <c r="L7" s="172"/>
-      <c r="M7" s="172"/>
-      <c r="N7" s="217" t="s">
+      <c r="L7" s="183"/>
+      <c r="M7" s="183"/>
+      <c r="N7" s="177" t="s">
         <v>384</v>
       </c>
-      <c r="O7" s="217"/>
-      <c r="P7" s="217"/>
-      <c r="Q7" s="217"/>
+      <c r="O7" s="177"/>
+      <c r="P7" s="177"/>
+      <c r="Q7" s="177"/>
       <c r="R7" s="139" t="s">
         <v>441</v>
       </c>
       <c r="S7" s="139"/>
-      <c r="T7" s="199">
+      <c r="T7" s="174">
         <v>20508972734</v>
       </c>
-      <c r="U7" s="199"/>
-      <c r="V7" s="199"/>
-      <c r="W7" s="199"/>
-      <c r="X7" s="199"/>
-      <c r="Y7" s="216" t="s">
+      <c r="U7" s="174"/>
+      <c r="V7" s="174"/>
+      <c r="W7" s="174"/>
+      <c r="X7" s="174"/>
+      <c r="Y7" s="173" t="s">
         <v>444</v>
       </c>
-      <c r="Z7" s="216"/>
-      <c r="AA7" s="216"/>
-      <c r="AB7" s="216"/>
-      <c r="AC7" s="199" t="s">
+      <c r="Z7" s="173"/>
+      <c r="AA7" s="173"/>
+      <c r="AB7" s="173"/>
+      <c r="AC7" s="174" t="s">
         <v>608</v>
       </c>
-      <c r="AD7" s="199"/>
-      <c r="AE7" s="199"/>
-      <c r="AF7" s="199"/>
-      <c r="AG7" s="199"/>
+      <c r="AD7" s="174"/>
+      <c r="AE7" s="174"/>
+      <c r="AF7" s="174"/>
+      <c r="AG7" s="174"/>
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
       <c r="AK7" s="2"/>
@@ -6842,41 +6842,41 @@
       <c r="B8" s="150" t="s">
         <v>442</v>
       </c>
-      <c r="C8" s="232" t="s">
+      <c r="C8" s="185" t="s">
         <v>610</v>
       </c>
-      <c r="D8" s="232"/>
-      <c r="E8" s="232"/>
-      <c r="F8" s="232"/>
-      <c r="G8" s="232"/>
-      <c r="H8" s="232"/>
-      <c r="I8" s="232"/>
-      <c r="J8" s="232"/>
-      <c r="K8" s="232"/>
-      <c r="L8" s="232"/>
-      <c r="M8" s="232"/>
-      <c r="N8" s="232"/>
-      <c r="O8" s="232"/>
-      <c r="P8" s="232"/>
-      <c r="Q8" s="232"/>
-      <c r="R8" s="202" t="s">
+      <c r="D8" s="185"/>
+      <c r="E8" s="185"/>
+      <c r="F8" s="185"/>
+      <c r="G8" s="185"/>
+      <c r="H8" s="185"/>
+      <c r="I8" s="185"/>
+      <c r="J8" s="185"/>
+      <c r="K8" s="185"/>
+      <c r="L8" s="185"/>
+      <c r="M8" s="185"/>
+      <c r="N8" s="185"/>
+      <c r="O8" s="185"/>
+      <c r="P8" s="185"/>
+      <c r="Q8" s="185"/>
+      <c r="R8" s="187" t="s">
         <v>611</v>
       </c>
-      <c r="S8" s="202"/>
-      <c r="T8" s="202"/>
-      <c r="U8" s="202"/>
-      <c r="V8" s="202"/>
-      <c r="W8" s="202"/>
-      <c r="X8" s="202"/>
-      <c r="Y8" s="232"/>
-      <c r="Z8" s="232"/>
-      <c r="AA8" s="232"/>
-      <c r="AB8" s="232"/>
-      <c r="AC8" s="232"/>
-      <c r="AD8" s="232"/>
-      <c r="AE8" s="232"/>
-      <c r="AF8" s="232"/>
-      <c r="AG8" s="232"/>
+      <c r="S8" s="187"/>
+      <c r="T8" s="187"/>
+      <c r="U8" s="187"/>
+      <c r="V8" s="187"/>
+      <c r="W8" s="187"/>
+      <c r="X8" s="187"/>
+      <c r="Y8" s="185"/>
+      <c r="Z8" s="185"/>
+      <c r="AA8" s="185"/>
+      <c r="AB8" s="185"/>
+      <c r="AC8" s="185"/>
+      <c r="AD8" s="185"/>
+      <c r="AE8" s="185"/>
+      <c r="AF8" s="185"/>
+      <c r="AG8" s="185"/>
       <c r="AH8" s="2"/>
       <c r="AI8" s="2"/>
       <c r="AK8" s="2"/>
@@ -7150,79 +7150,79 @@
       <c r="JK9" s="2"/>
     </row>
     <row r="10" spans="1:271" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="236" t="s">
+      <c r="B10" s="172" t="s">
         <v>471</v>
       </c>
-      <c r="C10" s="236"/>
-      <c r="D10" s="236"/>
-      <c r="E10" s="236"/>
-      <c r="F10" s="236"/>
-      <c r="G10" s="236"/>
-      <c r="H10" s="236"/>
-      <c r="I10" s="236"/>
-      <c r="J10" s="236"/>
-      <c r="K10" s="236"/>
-      <c r="L10" s="236"/>
-      <c r="M10" s="236"/>
-      <c r="N10" s="236"/>
-      <c r="O10" s="236"/>
-      <c r="P10" s="236"/>
-      <c r="Q10" s="236"/>
-      <c r="R10" s="236"/>
-      <c r="S10" s="236"/>
-      <c r="T10" s="236"/>
-      <c r="U10" s="236"/>
-      <c r="V10" s="236"/>
-      <c r="W10" s="236"/>
-      <c r="X10" s="236"/>
-      <c r="Y10" s="236"/>
-      <c r="Z10" s="236"/>
-      <c r="AA10" s="236"/>
-      <c r="AB10" s="236"/>
-      <c r="AC10" s="236"/>
-      <c r="AD10" s="236"/>
-      <c r="AE10" s="236"/>
-      <c r="AF10" s="236"/>
-      <c r="AG10" s="236"/>
+      <c r="C10" s="172"/>
+      <c r="D10" s="172"/>
+      <c r="E10" s="172"/>
+      <c r="F10" s="172"/>
+      <c r="G10" s="172"/>
+      <c r="H10" s="172"/>
+      <c r="I10" s="172"/>
+      <c r="J10" s="172"/>
+      <c r="K10" s="172"/>
+      <c r="L10" s="172"/>
+      <c r="M10" s="172"/>
+      <c r="N10" s="172"/>
+      <c r="O10" s="172"/>
+      <c r="P10" s="172"/>
+      <c r="Q10" s="172"/>
+      <c r="R10" s="172"/>
+      <c r="S10" s="172"/>
+      <c r="T10" s="172"/>
+      <c r="U10" s="172"/>
+      <c r="V10" s="172"/>
+      <c r="W10" s="172"/>
+      <c r="X10" s="172"/>
+      <c r="Y10" s="172"/>
+      <c r="Z10" s="172"/>
+      <c r="AA10" s="172"/>
+      <c r="AB10" s="172"/>
+      <c r="AC10" s="172"/>
+      <c r="AD10" s="172"/>
+      <c r="AE10" s="172"/>
+      <c r="AF10" s="172"/>
+      <c r="AG10" s="172"/>
       <c r="AH10" s="2"/>
       <c r="AI10" s="2"/>
       <c r="AK10" s="2"/>
     </row>
     <row r="11" spans="1:271" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="194" t="s">
+      <c r="B11" s="175" t="s">
         <v>612</v>
       </c>
-      <c r="C11" s="194"/>
-      <c r="D11" s="194"/>
-      <c r="E11" s="194"/>
-      <c r="F11" s="194"/>
-      <c r="G11" s="194"/>
-      <c r="H11" s="194"/>
-      <c r="I11" s="194"/>
-      <c r="J11" s="194"/>
-      <c r="K11" s="194"/>
-      <c r="L11" s="194"/>
-      <c r="M11" s="194"/>
-      <c r="N11" s="194"/>
-      <c r="O11" s="194"/>
-      <c r="P11" s="194"/>
-      <c r="Q11" s="194"/>
-      <c r="R11" s="194"/>
-      <c r="S11" s="194"/>
-      <c r="T11" s="194"/>
-      <c r="U11" s="194"/>
-      <c r="V11" s="194"/>
-      <c r="W11" s="194"/>
-      <c r="X11" s="194"/>
-      <c r="Y11" s="194"/>
-      <c r="Z11" s="194"/>
-      <c r="AA11" s="194"/>
-      <c r="AB11" s="194"/>
-      <c r="AC11" s="194"/>
-      <c r="AD11" s="194"/>
-      <c r="AE11" s="194"/>
-      <c r="AF11" s="194"/>
-      <c r="AG11" s="194"/>
+      <c r="C11" s="175"/>
+      <c r="D11" s="175"/>
+      <c r="E11" s="175"/>
+      <c r="F11" s="175"/>
+      <c r="G11" s="175"/>
+      <c r="H11" s="175"/>
+      <c r="I11" s="175"/>
+      <c r="J11" s="175"/>
+      <c r="K11" s="175"/>
+      <c r="L11" s="175"/>
+      <c r="M11" s="175"/>
+      <c r="N11" s="175"/>
+      <c r="O11" s="175"/>
+      <c r="P11" s="175"/>
+      <c r="Q11" s="175"/>
+      <c r="R11" s="175"/>
+      <c r="S11" s="175"/>
+      <c r="T11" s="175"/>
+      <c r="U11" s="175"/>
+      <c r="V11" s="175"/>
+      <c r="W11" s="175"/>
+      <c r="X11" s="175"/>
+      <c r="Y11" s="175"/>
+      <c r="Z11" s="175"/>
+      <c r="AA11" s="175"/>
+      <c r="AB11" s="175"/>
+      <c r="AC11" s="175"/>
+      <c r="AD11" s="175"/>
+      <c r="AE11" s="175"/>
+      <c r="AF11" s="175"/>
+      <c r="AG11" s="175"/>
       <c r="AH11" s="2"/>
       <c r="AI11" s="2"/>
       <c r="AK11" s="2"/>
@@ -7231,118 +7231,118 @@
       <c r="B12" s="139" t="s">
         <v>440</v>
       </c>
-      <c r="C12" s="199"/>
-      <c r="D12" s="199"/>
-      <c r="E12" s="199"/>
-      <c r="F12" s="199"/>
-      <c r="G12" s="199"/>
-      <c r="H12" s="199"/>
-      <c r="I12" s="199"/>
-      <c r="J12" s="199"/>
-      <c r="K12" s="199"/>
-      <c r="L12" s="199"/>
-      <c r="M12" s="199"/>
+      <c r="C12" s="174"/>
+      <c r="D12" s="174"/>
+      <c r="E12" s="174"/>
+      <c r="F12" s="174"/>
+      <c r="G12" s="174"/>
+      <c r="H12" s="174"/>
+      <c r="I12" s="174"/>
+      <c r="J12" s="174"/>
+      <c r="K12" s="174"/>
+      <c r="L12" s="174"/>
+      <c r="M12" s="174"/>
       <c r="N12" s="170" t="s">
         <v>441</v>
       </c>
-      <c r="O12" s="199"/>
-      <c r="P12" s="199"/>
-      <c r="Q12" s="199"/>
-      <c r="R12" s="199"/>
-      <c r="S12" s="199"/>
-      <c r="T12" s="199"/>
-      <c r="U12" s="216" t="s">
+      <c r="O12" s="174"/>
+      <c r="P12" s="174"/>
+      <c r="Q12" s="174"/>
+      <c r="R12" s="174"/>
+      <c r="S12" s="174"/>
+      <c r="T12" s="174"/>
+      <c r="U12" s="173" t="s">
         <v>444</v>
       </c>
-      <c r="V12" s="216"/>
-      <c r="W12" s="216"/>
-      <c r="X12" s="216"/>
-      <c r="Y12" s="199"/>
-      <c r="Z12" s="199"/>
-      <c r="AA12" s="199"/>
-      <c r="AB12" s="199"/>
-      <c r="AC12" s="199"/>
-      <c r="AD12" s="199"/>
-      <c r="AE12" s="199"/>
-      <c r="AF12" s="199"/>
-      <c r="AG12" s="199"/>
+      <c r="V12" s="173"/>
+      <c r="W12" s="173"/>
+      <c r="X12" s="173"/>
+      <c r="Y12" s="174"/>
+      <c r="Z12" s="174"/>
+      <c r="AA12" s="174"/>
+      <c r="AB12" s="174"/>
+      <c r="AC12" s="174"/>
+      <c r="AD12" s="174"/>
+      <c r="AE12" s="174"/>
+      <c r="AF12" s="174"/>
+      <c r="AG12" s="174"/>
     </row>
     <row r="13" spans="1:271" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="138" t="s">
         <v>442</v>
       </c>
-      <c r="C13" s="217"/>
-      <c r="D13" s="217"/>
-      <c r="E13" s="217"/>
-      <c r="F13" s="217"/>
-      <c r="G13" s="217"/>
-      <c r="H13" s="217"/>
-      <c r="I13" s="217"/>
-      <c r="J13" s="217"/>
-      <c r="K13" s="217"/>
-      <c r="L13" s="217"/>
-      <c r="M13" s="217"/>
-      <c r="N13" s="217"/>
-      <c r="O13" s="217"/>
-      <c r="P13" s="217"/>
-      <c r="Q13" s="217"/>
-      <c r="R13" s="173" t="s">
+      <c r="C13" s="177"/>
+      <c r="D13" s="177"/>
+      <c r="E13" s="177"/>
+      <c r="F13" s="177"/>
+      <c r="G13" s="177"/>
+      <c r="H13" s="177"/>
+      <c r="I13" s="177"/>
+      <c r="J13" s="177"/>
+      <c r="K13" s="177"/>
+      <c r="L13" s="177"/>
+      <c r="M13" s="177"/>
+      <c r="N13" s="177"/>
+      <c r="O13" s="177"/>
+      <c r="P13" s="177"/>
+      <c r="Q13" s="177"/>
+      <c r="R13" s="176" t="s">
         <v>611</v>
       </c>
-      <c r="S13" s="173"/>
-      <c r="T13" s="173"/>
-      <c r="U13" s="173"/>
-      <c r="V13" s="173"/>
-      <c r="W13" s="173"/>
-      <c r="X13" s="173"/>
-      <c r="Y13" s="217"/>
-      <c r="Z13" s="217"/>
-      <c r="AA13" s="217"/>
-      <c r="AB13" s="217"/>
-      <c r="AC13" s="217"/>
-      <c r="AD13" s="217"/>
-      <c r="AE13" s="217"/>
-      <c r="AF13" s="217"/>
-      <c r="AG13" s="217"/>
+      <c r="S13" s="176"/>
+      <c r="T13" s="176"/>
+      <c r="U13" s="176"/>
+      <c r="V13" s="176"/>
+      <c r="W13" s="176"/>
+      <c r="X13" s="176"/>
+      <c r="Y13" s="177"/>
+      <c r="Z13" s="177"/>
+      <c r="AA13" s="177"/>
+      <c r="AB13" s="177"/>
+      <c r="AC13" s="177"/>
+      <c r="AD13" s="177"/>
+      <c r="AE13" s="177"/>
+      <c r="AF13" s="177"/>
+      <c r="AG13" s="177"/>
       <c r="AH13" s="2"/>
       <c r="AI13" s="2"/>
       <c r="AK13" s="2"/>
     </row>
     <row r="14" spans="1:271" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="194" t="s">
+      <c r="B14" s="175" t="s">
         <v>472</v>
       </c>
-      <c r="C14" s="194"/>
-      <c r="D14" s="194"/>
-      <c r="E14" s="194"/>
-      <c r="F14" s="194"/>
-      <c r="G14" s="194"/>
-      <c r="H14" s="194"/>
-      <c r="I14" s="194"/>
-      <c r="J14" s="194"/>
-      <c r="K14" s="194"/>
-      <c r="L14" s="194"/>
-      <c r="M14" s="194"/>
-      <c r="N14" s="194"/>
-      <c r="O14" s="194"/>
-      <c r="P14" s="194"/>
-      <c r="Q14" s="194"/>
-      <c r="R14" s="194"/>
-      <c r="S14" s="194"/>
-      <c r="T14" s="194"/>
-      <c r="U14" s="194"/>
-      <c r="V14" s="194"/>
-      <c r="W14" s="194"/>
-      <c r="X14" s="194"/>
-      <c r="Y14" s="194"/>
-      <c r="Z14" s="194"/>
-      <c r="AA14" s="194"/>
-      <c r="AB14" s="194"/>
-      <c r="AC14" s="194"/>
-      <c r="AD14" s="194"/>
-      <c r="AE14" s="194"/>
-      <c r="AF14" s="194"/>
-      <c r="AG14" s="194"/>
+      <c r="C14" s="175"/>
+      <c r="D14" s="175"/>
+      <c r="E14" s="175"/>
+      <c r="F14" s="175"/>
+      <c r="G14" s="175"/>
+      <c r="H14" s="175"/>
+      <c r="I14" s="175"/>
+      <c r="J14" s="175"/>
+      <c r="K14" s="175"/>
+      <c r="L14" s="175"/>
+      <c r="M14" s="175"/>
+      <c r="N14" s="175"/>
+      <c r="O14" s="175"/>
+      <c r="P14" s="175"/>
+      <c r="Q14" s="175"/>
+      <c r="R14" s="175"/>
+      <c r="S14" s="175"/>
+      <c r="T14" s="175"/>
+      <c r="U14" s="175"/>
+      <c r="V14" s="175"/>
+      <c r="W14" s="175"/>
+      <c r="X14" s="175"/>
+      <c r="Y14" s="175"/>
+      <c r="Z14" s="175"/>
+      <c r="AA14" s="175"/>
+      <c r="AB14" s="175"/>
+      <c r="AC14" s="175"/>
+      <c r="AD14" s="175"/>
+      <c r="AE14" s="175"/>
+      <c r="AF14" s="175"/>
+      <c r="AG14" s="175"/>
       <c r="AH14" s="2"/>
       <c r="AI14" s="2"/>
       <c r="AK14" s="2"/>
@@ -7351,79 +7351,79 @@
       <c r="B15" s="139" t="s">
         <v>440</v>
       </c>
-      <c r="C15" s="199"/>
-      <c r="D15" s="199"/>
-      <c r="E15" s="199"/>
-      <c r="F15" s="199"/>
-      <c r="G15" s="199"/>
-      <c r="H15" s="199"/>
-      <c r="I15" s="199"/>
-      <c r="J15" s="199"/>
-      <c r="K15" s="199"/>
-      <c r="L15" s="199"/>
-      <c r="M15" s="199"/>
+      <c r="C15" s="174"/>
+      <c r="D15" s="174"/>
+      <c r="E15" s="174"/>
+      <c r="F15" s="174"/>
+      <c r="G15" s="174"/>
+      <c r="H15" s="174"/>
+      <c r="I15" s="174"/>
+      <c r="J15" s="174"/>
+      <c r="K15" s="174"/>
+      <c r="L15" s="174"/>
+      <c r="M15" s="174"/>
       <c r="N15" s="170" t="s">
         <v>441</v>
       </c>
-      <c r="O15" s="199"/>
-      <c r="P15" s="199"/>
-      <c r="Q15" s="199"/>
-      <c r="R15" s="199"/>
-      <c r="S15" s="199"/>
-      <c r="T15" s="199"/>
-      <c r="U15" s="216" t="s">
+      <c r="O15" s="174"/>
+      <c r="P15" s="174"/>
+      <c r="Q15" s="174"/>
+      <c r="R15" s="174"/>
+      <c r="S15" s="174"/>
+      <c r="T15" s="174"/>
+      <c r="U15" s="173" t="s">
         <v>444</v>
       </c>
-      <c r="V15" s="216"/>
-      <c r="W15" s="216"/>
-      <c r="X15" s="216"/>
-      <c r="Y15" s="199"/>
-      <c r="Z15" s="199"/>
-      <c r="AA15" s="199"/>
-      <c r="AB15" s="199"/>
-      <c r="AC15" s="199"/>
-      <c r="AD15" s="199"/>
-      <c r="AE15" s="199"/>
-      <c r="AF15" s="199"/>
-      <c r="AG15" s="199"/>
+      <c r="V15" s="173"/>
+      <c r="W15" s="173"/>
+      <c r="X15" s="173"/>
+      <c r="Y15" s="174"/>
+      <c r="Z15" s="174"/>
+      <c r="AA15" s="174"/>
+      <c r="AB15" s="174"/>
+      <c r="AC15" s="174"/>
+      <c r="AD15" s="174"/>
+      <c r="AE15" s="174"/>
+      <c r="AF15" s="174"/>
+      <c r="AG15" s="174"/>
     </row>
     <row r="16" spans="1:271" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="150" t="s">
         <v>442</v>
       </c>
-      <c r="C16" s="232"/>
-      <c r="D16" s="232"/>
-      <c r="E16" s="232"/>
-      <c r="F16" s="232"/>
-      <c r="G16" s="232"/>
-      <c r="H16" s="232"/>
-      <c r="I16" s="232"/>
-      <c r="J16" s="232"/>
-      <c r="K16" s="232"/>
-      <c r="L16" s="232"/>
-      <c r="M16" s="232"/>
-      <c r="N16" s="232"/>
-      <c r="O16" s="232"/>
-      <c r="P16" s="232"/>
-      <c r="Q16" s="232"/>
-      <c r="R16" s="202" t="s">
+      <c r="C16" s="185"/>
+      <c r="D16" s="185"/>
+      <c r="E16" s="185"/>
+      <c r="F16" s="185"/>
+      <c r="G16" s="185"/>
+      <c r="H16" s="185"/>
+      <c r="I16" s="185"/>
+      <c r="J16" s="185"/>
+      <c r="K16" s="185"/>
+      <c r="L16" s="185"/>
+      <c r="M16" s="185"/>
+      <c r="N16" s="185"/>
+      <c r="O16" s="185"/>
+      <c r="P16" s="185"/>
+      <c r="Q16" s="185"/>
+      <c r="R16" s="187" t="s">
         <v>611</v>
       </c>
-      <c r="S16" s="202"/>
-      <c r="T16" s="202"/>
-      <c r="U16" s="202"/>
-      <c r="V16" s="202"/>
-      <c r="W16" s="202"/>
-      <c r="X16" s="202"/>
-      <c r="Y16" s="232"/>
-      <c r="Z16" s="232"/>
-      <c r="AA16" s="232"/>
-      <c r="AB16" s="232"/>
-      <c r="AC16" s="232"/>
-      <c r="AD16" s="232"/>
-      <c r="AE16" s="232"/>
-      <c r="AF16" s="232"/>
-      <c r="AG16" s="232"/>
+      <c r="S16" s="187"/>
+      <c r="T16" s="187"/>
+      <c r="U16" s="187"/>
+      <c r="V16" s="187"/>
+      <c r="W16" s="187"/>
+      <c r="X16" s="187"/>
+      <c r="Y16" s="185"/>
+      <c r="Z16" s="185"/>
+      <c r="AA16" s="185"/>
+      <c r="AB16" s="185"/>
+      <c r="AC16" s="185"/>
+      <c r="AD16" s="185"/>
+      <c r="AE16" s="185"/>
+      <c r="AF16" s="185"/>
+      <c r="AG16" s="185"/>
       <c r="AH16" s="2"/>
       <c r="AI16" s="2"/>
       <c r="AK16" s="2"/>
@@ -7466,79 +7466,79 @@
       <c r="AK17" s="2"/>
     </row>
     <row r="18" spans="1:271" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="234" t="s">
+      <c r="B18" s="184" t="s">
         <v>473</v>
       </c>
-      <c r="C18" s="234"/>
-      <c r="D18" s="234"/>
-      <c r="E18" s="234"/>
-      <c r="F18" s="234"/>
-      <c r="G18" s="234"/>
-      <c r="H18" s="234"/>
-      <c r="I18" s="234"/>
-      <c r="J18" s="234"/>
-      <c r="K18" s="234"/>
-      <c r="L18" s="234"/>
-      <c r="M18" s="234"/>
-      <c r="N18" s="234"/>
-      <c r="O18" s="234"/>
-      <c r="P18" s="234"/>
-      <c r="Q18" s="234"/>
-      <c r="R18" s="234"/>
-      <c r="S18" s="234"/>
-      <c r="T18" s="234"/>
-      <c r="U18" s="234"/>
-      <c r="V18" s="234"/>
-      <c r="W18" s="234"/>
-      <c r="X18" s="234"/>
-      <c r="Y18" s="234"/>
-      <c r="Z18" s="234"/>
-      <c r="AA18" s="234"/>
-      <c r="AB18" s="234"/>
-      <c r="AC18" s="234"/>
-      <c r="AD18" s="234"/>
-      <c r="AE18" s="234"/>
-      <c r="AF18" s="234"/>
-      <c r="AG18" s="234"/>
+      <c r="C18" s="184"/>
+      <c r="D18" s="184"/>
+      <c r="E18" s="184"/>
+      <c r="F18" s="184"/>
+      <c r="G18" s="184"/>
+      <c r="H18" s="184"/>
+      <c r="I18" s="184"/>
+      <c r="J18" s="184"/>
+      <c r="K18" s="184"/>
+      <c r="L18" s="184"/>
+      <c r="M18" s="184"/>
+      <c r="N18" s="184"/>
+      <c r="O18" s="184"/>
+      <c r="P18" s="184"/>
+      <c r="Q18" s="184"/>
+      <c r="R18" s="184"/>
+      <c r="S18" s="184"/>
+      <c r="T18" s="184"/>
+      <c r="U18" s="184"/>
+      <c r="V18" s="184"/>
+      <c r="W18" s="184"/>
+      <c r="X18" s="184"/>
+      <c r="Y18" s="184"/>
+      <c r="Z18" s="184"/>
+      <c r="AA18" s="184"/>
+      <c r="AB18" s="184"/>
+      <c r="AC18" s="184"/>
+      <c r="AD18" s="184"/>
+      <c r="AE18" s="184"/>
+      <c r="AF18" s="184"/>
+      <c r="AG18" s="184"/>
       <c r="AH18" s="2"/>
       <c r="AI18" s="2"/>
       <c r="AK18" s="2"/>
     </row>
     <row r="19" spans="1:271" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="194" t="s">
+      <c r="B19" s="175" t="s">
         <v>561</v>
       </c>
-      <c r="C19" s="194"/>
-      <c r="D19" s="194"/>
-      <c r="E19" s="194"/>
-      <c r="F19" s="194"/>
-      <c r="G19" s="194"/>
-      <c r="H19" s="194"/>
-      <c r="I19" s="194"/>
-      <c r="J19" s="194"/>
-      <c r="K19" s="194"/>
-      <c r="L19" s="194"/>
-      <c r="M19" s="194"/>
-      <c r="N19" s="194"/>
-      <c r="O19" s="194"/>
-      <c r="P19" s="194"/>
-      <c r="Q19" s="194"/>
-      <c r="R19" s="194"/>
-      <c r="S19" s="194"/>
-      <c r="T19" s="194"/>
-      <c r="U19" s="194"/>
-      <c r="V19" s="194"/>
-      <c r="W19" s="194"/>
-      <c r="X19" s="194"/>
-      <c r="Y19" s="194"/>
-      <c r="Z19" s="194"/>
-      <c r="AA19" s="194"/>
-      <c r="AB19" s="194"/>
-      <c r="AC19" s="194"/>
-      <c r="AD19" s="194"/>
-      <c r="AE19" s="194"/>
-      <c r="AF19" s="194"/>
-      <c r="AG19" s="194"/>
+      <c r="C19" s="175"/>
+      <c r="D19" s="175"/>
+      <c r="E19" s="175"/>
+      <c r="F19" s="175"/>
+      <c r="G19" s="175"/>
+      <c r="H19" s="175"/>
+      <c r="I19" s="175"/>
+      <c r="J19" s="175"/>
+      <c r="K19" s="175"/>
+      <c r="L19" s="175"/>
+      <c r="M19" s="175"/>
+      <c r="N19" s="175"/>
+      <c r="O19" s="175"/>
+      <c r="P19" s="175"/>
+      <c r="Q19" s="175"/>
+      <c r="R19" s="175"/>
+      <c r="S19" s="175"/>
+      <c r="T19" s="175"/>
+      <c r="U19" s="175"/>
+      <c r="V19" s="175"/>
+      <c r="W19" s="175"/>
+      <c r="X19" s="175"/>
+      <c r="Y19" s="175"/>
+      <c r="Z19" s="175"/>
+      <c r="AA19" s="175"/>
+      <c r="AB19" s="175"/>
+      <c r="AC19" s="175"/>
+      <c r="AD19" s="175"/>
+      <c r="AE19" s="175"/>
+      <c r="AF19" s="175"/>
+      <c r="AG19" s="175"/>
       <c r="AH19" s="2"/>
       <c r="AI19" s="2"/>
       <c r="AK19" s="2"/>
@@ -7548,39 +7548,39 @@
       <c r="B20" s="137" t="s">
         <v>447</v>
       </c>
-      <c r="C20" s="217"/>
-      <c r="D20" s="217"/>
-      <c r="E20" s="217"/>
-      <c r="F20" s="217"/>
-      <c r="G20" s="217"/>
-      <c r="H20" s="217"/>
-      <c r="I20" s="217"/>
-      <c r="J20" s="217"/>
-      <c r="K20" s="217"/>
-      <c r="L20" s="217"/>
-      <c r="M20" s="217"/>
-      <c r="N20" s="217"/>
-      <c r="O20" s="217"/>
-      <c r="P20" s="217"/>
-      <c r="Q20" s="172" t="s">
+      <c r="C20" s="177"/>
+      <c r="D20" s="177"/>
+      <c r="E20" s="177"/>
+      <c r="F20" s="177"/>
+      <c r="G20" s="177"/>
+      <c r="H20" s="177"/>
+      <c r="I20" s="177"/>
+      <c r="J20" s="177"/>
+      <c r="K20" s="177"/>
+      <c r="L20" s="177"/>
+      <c r="M20" s="177"/>
+      <c r="N20" s="177"/>
+      <c r="O20" s="177"/>
+      <c r="P20" s="177"/>
+      <c r="Q20" s="183" t="s">
         <v>448</v>
       </c>
-      <c r="R20" s="172"/>
-      <c r="S20" s="172"/>
-      <c r="T20" s="172"/>
-      <c r="U20" s="172"/>
-      <c r="V20" s="172"/>
-      <c r="W20" s="172"/>
-      <c r="X20" s="217"/>
-      <c r="Y20" s="217"/>
-      <c r="Z20" s="217"/>
-      <c r="AA20" s="217"/>
-      <c r="AB20" s="217"/>
-      <c r="AC20" s="217"/>
-      <c r="AD20" s="217"/>
-      <c r="AE20" s="217"/>
-      <c r="AF20" s="217"/>
-      <c r="AG20" s="217"/>
+      <c r="R20" s="183"/>
+      <c r="S20" s="183"/>
+      <c r="T20" s="183"/>
+      <c r="U20" s="183"/>
+      <c r="V20" s="183"/>
+      <c r="W20" s="183"/>
+      <c r="X20" s="177"/>
+      <c r="Y20" s="177"/>
+      <c r="Z20" s="177"/>
+      <c r="AA20" s="177"/>
+      <c r="AB20" s="177"/>
+      <c r="AC20" s="177"/>
+      <c r="AD20" s="177"/>
+      <c r="AE20" s="177"/>
+      <c r="AF20" s="177"/>
+      <c r="AG20" s="177"/>
       <c r="AH20" s="2"/>
       <c r="AI20" s="2"/>
       <c r="AK20" s="2"/>
@@ -7820,43 +7820,43 @@
       <c r="B21" s="138" t="s">
         <v>450</v>
       </c>
-      <c r="C21" s="217"/>
-      <c r="D21" s="217"/>
-      <c r="E21" s="217"/>
-      <c r="F21" s="217"/>
-      <c r="G21" s="217"/>
-      <c r="H21" s="217"/>
-      <c r="I21" s="217"/>
-      <c r="J21" s="217"/>
-      <c r="K21" s="217"/>
-      <c r="L21" s="235" t="s">
+      <c r="C21" s="177"/>
+      <c r="D21" s="177"/>
+      <c r="E21" s="177"/>
+      <c r="F21" s="177"/>
+      <c r="G21" s="177"/>
+      <c r="H21" s="177"/>
+      <c r="I21" s="177"/>
+      <c r="J21" s="177"/>
+      <c r="K21" s="177"/>
+      <c r="L21" s="186" t="s">
         <v>660</v>
       </c>
-      <c r="M21" s="235"/>
-      <c r="N21" s="235"/>
-      <c r="O21" s="235"/>
-      <c r="P21" s="235"/>
-      <c r="Q21" s="173" t="s">
+      <c r="M21" s="186"/>
+      <c r="N21" s="186"/>
+      <c r="O21" s="186"/>
+      <c r="P21" s="186"/>
+      <c r="Q21" s="176" t="s">
         <v>455</v>
       </c>
-      <c r="R21" s="173"/>
-      <c r="S21" s="173"/>
-      <c r="T21" s="199"/>
-      <c r="U21" s="199"/>
-      <c r="V21" s="199"/>
-      <c r="W21" s="199"/>
-      <c r="X21" s="173" t="s">
+      <c r="R21" s="176"/>
+      <c r="S21" s="176"/>
+      <c r="T21" s="174"/>
+      <c r="U21" s="174"/>
+      <c r="V21" s="174"/>
+      <c r="W21" s="174"/>
+      <c r="X21" s="176" t="s">
         <v>456</v>
       </c>
-      <c r="Y21" s="173"/>
-      <c r="Z21" s="173"/>
-      <c r="AA21" s="173"/>
-      <c r="AB21" s="217"/>
-      <c r="AC21" s="217"/>
-      <c r="AD21" s="217"/>
-      <c r="AE21" s="217"/>
-      <c r="AF21" s="217"/>
-      <c r="AG21" s="217"/>
+      <c r="Y21" s="176"/>
+      <c r="Z21" s="176"/>
+      <c r="AA21" s="176"/>
+      <c r="AB21" s="177"/>
+      <c r="AC21" s="177"/>
+      <c r="AD21" s="177"/>
+      <c r="AE21" s="177"/>
+      <c r="AF21" s="177"/>
+      <c r="AG21" s="177"/>
       <c r="AH21" s="2"/>
       <c r="AI21" s="2"/>
       <c r="AK21" s="2"/>
@@ -8096,43 +8096,43 @@
       <c r="B22" s="139" t="s">
         <v>661</v>
       </c>
-      <c r="C22" s="217"/>
-      <c r="D22" s="217"/>
-      <c r="E22" s="217"/>
-      <c r="F22" s="217"/>
-      <c r="G22" s="217"/>
-      <c r="H22" s="217"/>
-      <c r="I22" s="217"/>
-      <c r="J22" s="217"/>
-      <c r="K22" s="217"/>
-      <c r="L22" s="173" t="s">
+      <c r="C22" s="177"/>
+      <c r="D22" s="177"/>
+      <c r="E22" s="177"/>
+      <c r="F22" s="177"/>
+      <c r="G22" s="177"/>
+      <c r="H22" s="177"/>
+      <c r="I22" s="177"/>
+      <c r="J22" s="177"/>
+      <c r="K22" s="177"/>
+      <c r="L22" s="176" t="s">
         <v>445</v>
       </c>
-      <c r="M22" s="173"/>
-      <c r="N22" s="173"/>
-      <c r="O22" s="173"/>
-      <c r="P22" s="173"/>
-      <c r="Q22" s="217"/>
-      <c r="R22" s="217"/>
-      <c r="S22" s="217"/>
-      <c r="T22" s="173" t="s">
+      <c r="M22" s="176"/>
+      <c r="N22" s="176"/>
+      <c r="O22" s="176"/>
+      <c r="P22" s="176"/>
+      <c r="Q22" s="177"/>
+      <c r="R22" s="177"/>
+      <c r="S22" s="177"/>
+      <c r="T22" s="176" t="s">
         <v>446</v>
       </c>
-      <c r="U22" s="173"/>
-      <c r="V22" s="173"/>
-      <c r="W22" s="173"/>
-      <c r="X22" s="217"/>
-      <c r="Y22" s="217"/>
-      <c r="Z22" s="217"/>
-      <c r="AA22" s="217"/>
-      <c r="AB22" s="173" t="s">
+      <c r="U22" s="176"/>
+      <c r="V22" s="176"/>
+      <c r="W22" s="176"/>
+      <c r="X22" s="177"/>
+      <c r="Y22" s="177"/>
+      <c r="Z22" s="177"/>
+      <c r="AA22" s="177"/>
+      <c r="AB22" s="176" t="s">
         <v>449</v>
       </c>
-      <c r="AC22" s="173"/>
-      <c r="AD22" s="173"/>
-      <c r="AE22" s="175"/>
-      <c r="AF22" s="175"/>
-      <c r="AG22" s="175"/>
+      <c r="AC22" s="176"/>
+      <c r="AD22" s="176"/>
+      <c r="AE22" s="195"/>
+      <c r="AF22" s="195"/>
+      <c r="AG22" s="195"/>
       <c r="AH22" s="2"/>
       <c r="AI22" s="2"/>
       <c r="AK22" s="2"/>
@@ -8372,43 +8372,43 @@
       <c r="B23" s="138" t="s">
         <v>658</v>
       </c>
-      <c r="C23" s="217"/>
-      <c r="D23" s="217"/>
-      <c r="E23" s="217"/>
-      <c r="F23" s="217"/>
-      <c r="G23" s="217"/>
-      <c r="H23" s="217"/>
-      <c r="I23" s="217"/>
-      <c r="J23" s="217"/>
-      <c r="K23" s="217"/>
-      <c r="L23" s="173" t="s">
+      <c r="C23" s="177"/>
+      <c r="D23" s="177"/>
+      <c r="E23" s="177"/>
+      <c r="F23" s="177"/>
+      <c r="G23" s="177"/>
+      <c r="H23" s="177"/>
+      <c r="I23" s="177"/>
+      <c r="J23" s="177"/>
+      <c r="K23" s="177"/>
+      <c r="L23" s="176" t="s">
         <v>659</v>
       </c>
-      <c r="M23" s="173"/>
-      <c r="N23" s="173"/>
-      <c r="O23" s="173"/>
-      <c r="P23" s="173"/>
-      <c r="Q23" s="175"/>
-      <c r="R23" s="175"/>
-      <c r="S23" s="175"/>
-      <c r="T23" s="173" t="s">
+      <c r="M23" s="176"/>
+      <c r="N23" s="176"/>
+      <c r="O23" s="176"/>
+      <c r="P23" s="176"/>
+      <c r="Q23" s="195"/>
+      <c r="R23" s="195"/>
+      <c r="S23" s="195"/>
+      <c r="T23" s="176" t="s">
         <v>657</v>
       </c>
-      <c r="U23" s="173"/>
-      <c r="V23" s="173"/>
-      <c r="W23" s="173"/>
-      <c r="X23" s="199"/>
-      <c r="Y23" s="199"/>
-      <c r="Z23" s="199"/>
-      <c r="AA23" s="199"/>
-      <c r="AB23" s="173" t="s">
+      <c r="U23" s="176"/>
+      <c r="V23" s="176"/>
+      <c r="W23" s="176"/>
+      <c r="X23" s="174"/>
+      <c r="Y23" s="174"/>
+      <c r="Z23" s="174"/>
+      <c r="AA23" s="174"/>
+      <c r="AB23" s="176" t="s">
         <v>665</v>
       </c>
-      <c r="AC23" s="173"/>
-      <c r="AD23" s="173"/>
-      <c r="AE23" s="217"/>
-      <c r="AF23" s="217"/>
-      <c r="AG23" s="217"/>
+      <c r="AC23" s="176"/>
+      <c r="AD23" s="176"/>
+      <c r="AE23" s="177"/>
+      <c r="AF23" s="177"/>
+      <c r="AG23" s="177"/>
       <c r="AH23" s="2"/>
       <c r="AI23" s="2"/>
       <c r="AK23" s="2"/>
@@ -8648,37 +8648,37 @@
       <c r="B24" s="138" t="s">
         <v>463</v>
       </c>
-      <c r="C24" s="175"/>
-      <c r="D24" s="175"/>
-      <c r="E24" s="175"/>
-      <c r="F24" s="175"/>
-      <c r="G24" s="175"/>
-      <c r="H24" s="175"/>
-      <c r="I24" s="175"/>
-      <c r="J24" s="175"/>
-      <c r="K24" s="175"/>
-      <c r="L24" s="175"/>
-      <c r="M24" s="175"/>
-      <c r="N24" s="175"/>
-      <c r="O24" s="175"/>
-      <c r="P24" s="175"/>
-      <c r="Q24" s="175"/>
-      <c r="R24" s="175"/>
-      <c r="S24" s="175"/>
-      <c r="T24" s="175"/>
-      <c r="U24" s="175"/>
-      <c r="V24" s="175"/>
-      <c r="W24" s="175"/>
-      <c r="X24" s="175"/>
-      <c r="Y24" s="175"/>
-      <c r="Z24" s="175"/>
-      <c r="AA24" s="175"/>
-      <c r="AB24" s="175"/>
-      <c r="AC24" s="175"/>
-      <c r="AD24" s="175"/>
-      <c r="AE24" s="175"/>
-      <c r="AF24" s="175"/>
-      <c r="AG24" s="175"/>
+      <c r="C24" s="195"/>
+      <c r="D24" s="195"/>
+      <c r="E24" s="195"/>
+      <c r="F24" s="195"/>
+      <c r="G24" s="195"/>
+      <c r="H24" s="195"/>
+      <c r="I24" s="195"/>
+      <c r="J24" s="195"/>
+      <c r="K24" s="195"/>
+      <c r="L24" s="195"/>
+      <c r="M24" s="195"/>
+      <c r="N24" s="195"/>
+      <c r="O24" s="195"/>
+      <c r="P24" s="195"/>
+      <c r="Q24" s="195"/>
+      <c r="R24" s="195"/>
+      <c r="S24" s="195"/>
+      <c r="T24" s="195"/>
+      <c r="U24" s="195"/>
+      <c r="V24" s="195"/>
+      <c r="W24" s="195"/>
+      <c r="X24" s="195"/>
+      <c r="Y24" s="195"/>
+      <c r="Z24" s="195"/>
+      <c r="AA24" s="195"/>
+      <c r="AB24" s="195"/>
+      <c r="AC24" s="195"/>
+      <c r="AD24" s="195"/>
+      <c r="AE24" s="195"/>
+      <c r="AF24" s="195"/>
+      <c r="AG24" s="195"/>
       <c r="AH24" s="2"/>
       <c r="AI24" s="2"/>
       <c r="AJ24" s="2"/>
@@ -8913,40 +8913,40 @@
     </row>
     <row r="25" spans="1:271" ht="23.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
-      <c r="B25" s="194" t="s">
+      <c r="B25" s="175" t="s">
         <v>691</v>
       </c>
-      <c r="C25" s="194"/>
-      <c r="D25" s="194"/>
-      <c r="E25" s="194"/>
-      <c r="F25" s="194"/>
-      <c r="G25" s="194"/>
-      <c r="H25" s="194"/>
-      <c r="I25" s="194"/>
-      <c r="J25" s="194"/>
-      <c r="K25" s="194"/>
-      <c r="L25" s="194"/>
-      <c r="M25" s="194"/>
-      <c r="N25" s="194"/>
-      <c r="O25" s="194"/>
-      <c r="P25" s="194"/>
-      <c r="Q25" s="194"/>
-      <c r="R25" s="194"/>
-      <c r="S25" s="194"/>
-      <c r="T25" s="194"/>
-      <c r="U25" s="194"/>
-      <c r="V25" s="194"/>
-      <c r="W25" s="194"/>
-      <c r="X25" s="194"/>
-      <c r="Y25" s="194"/>
-      <c r="Z25" s="194"/>
-      <c r="AA25" s="194"/>
-      <c r="AB25" s="194"/>
-      <c r="AC25" s="194"/>
-      <c r="AD25" s="194"/>
-      <c r="AE25" s="194"/>
-      <c r="AF25" s="194"/>
-      <c r="AG25" s="194"/>
+      <c r="C25" s="175"/>
+      <c r="D25" s="175"/>
+      <c r="E25" s="175"/>
+      <c r="F25" s="175"/>
+      <c r="G25" s="175"/>
+      <c r="H25" s="175"/>
+      <c r="I25" s="175"/>
+      <c r="J25" s="175"/>
+      <c r="K25" s="175"/>
+      <c r="L25" s="175"/>
+      <c r="M25" s="175"/>
+      <c r="N25" s="175"/>
+      <c r="O25" s="175"/>
+      <c r="P25" s="175"/>
+      <c r="Q25" s="175"/>
+      <c r="R25" s="175"/>
+      <c r="S25" s="175"/>
+      <c r="T25" s="175"/>
+      <c r="U25" s="175"/>
+      <c r="V25" s="175"/>
+      <c r="W25" s="175"/>
+      <c r="X25" s="175"/>
+      <c r="Y25" s="175"/>
+      <c r="Z25" s="175"/>
+      <c r="AA25" s="175"/>
+      <c r="AB25" s="175"/>
+      <c r="AC25" s="175"/>
+      <c r="AD25" s="175"/>
+      <c r="AE25" s="175"/>
+      <c r="AF25" s="175"/>
+      <c r="AG25" s="175"/>
       <c r="AH25" s="2"/>
       <c r="AI25" s="2"/>
       <c r="AJ25" s="2"/>
@@ -9184,37 +9184,37 @@
       <c r="B26" s="169" t="s">
         <v>662</v>
       </c>
-      <c r="C26" s="199"/>
-      <c r="D26" s="199"/>
-      <c r="E26" s="199"/>
-      <c r="F26" s="199"/>
-      <c r="G26" s="199"/>
-      <c r="H26" s="199"/>
-      <c r="I26" s="199"/>
-      <c r="J26" s="199"/>
-      <c r="K26" s="199"/>
-      <c r="L26" s="199"/>
-      <c r="M26" s="199"/>
-      <c r="N26" s="199"/>
-      <c r="O26" s="199"/>
-      <c r="P26" s="199"/>
-      <c r="Q26" s="199"/>
-      <c r="R26" s="199"/>
-      <c r="S26" s="199"/>
-      <c r="T26" s="199"/>
-      <c r="U26" s="199"/>
-      <c r="V26" s="199"/>
-      <c r="W26" s="199"/>
-      <c r="X26" s="199"/>
-      <c r="Y26" s="199"/>
-      <c r="Z26" s="199"/>
-      <c r="AA26" s="199"/>
-      <c r="AB26" s="199"/>
-      <c r="AC26" s="199"/>
-      <c r="AD26" s="199"/>
-      <c r="AE26" s="199"/>
-      <c r="AF26" s="199"/>
-      <c r="AG26" s="199"/>
+      <c r="C26" s="174"/>
+      <c r="D26" s="174"/>
+      <c r="E26" s="174"/>
+      <c r="F26" s="174"/>
+      <c r="G26" s="174"/>
+      <c r="H26" s="174"/>
+      <c r="I26" s="174"/>
+      <c r="J26" s="174"/>
+      <c r="K26" s="174"/>
+      <c r="L26" s="174"/>
+      <c r="M26" s="174"/>
+      <c r="N26" s="174"/>
+      <c r="O26" s="174"/>
+      <c r="P26" s="174"/>
+      <c r="Q26" s="174"/>
+      <c r="R26" s="174"/>
+      <c r="S26" s="174"/>
+      <c r="T26" s="174"/>
+      <c r="U26" s="174"/>
+      <c r="V26" s="174"/>
+      <c r="W26" s="174"/>
+      <c r="X26" s="174"/>
+      <c r="Y26" s="174"/>
+      <c r="Z26" s="174"/>
+      <c r="AA26" s="174"/>
+      <c r="AB26" s="174"/>
+      <c r="AC26" s="174"/>
+      <c r="AD26" s="174"/>
+      <c r="AE26" s="174"/>
+      <c r="AF26" s="174"/>
+      <c r="AG26" s="174"/>
       <c r="AH26" s="2"/>
       <c r="AI26" s="2"/>
       <c r="AJ26" s="2"/>
@@ -9452,47 +9452,47 @@
       <c r="B27" s="167" t="s">
         <v>709</v>
       </c>
-      <c r="C27" s="209" t="s">
+      <c r="C27" s="213" t="s">
         <v>710</v>
       </c>
-      <c r="D27" s="209"/>
-      <c r="E27" s="209"/>
-      <c r="F27" s="209"/>
-      <c r="G27" s="209"/>
-      <c r="H27" s="209"/>
-      <c r="I27" s="209"/>
-      <c r="J27" s="209"/>
-      <c r="K27" s="209"/>
-      <c r="L27" s="209"/>
-      <c r="M27" s="209"/>
-      <c r="N27" s="209"/>
-      <c r="O27" s="209"/>
-      <c r="P27" s="209"/>
-      <c r="Q27" s="207" t="s">
+      <c r="D27" s="213"/>
+      <c r="E27" s="213"/>
+      <c r="F27" s="213"/>
+      <c r="G27" s="213"/>
+      <c r="H27" s="213"/>
+      <c r="I27" s="213"/>
+      <c r="J27" s="213"/>
+      <c r="K27" s="213"/>
+      <c r="L27" s="213"/>
+      <c r="M27" s="213"/>
+      <c r="N27" s="213"/>
+      <c r="O27" s="213"/>
+      <c r="P27" s="213"/>
+      <c r="Q27" s="211" t="s">
         <v>711</v>
       </c>
-      <c r="R27" s="207"/>
-      <c r="S27" s="207"/>
-      <c r="T27" s="207"/>
-      <c r="U27" s="207"/>
-      <c r="V27" s="207" t="s">
+      <c r="R27" s="211"/>
+      <c r="S27" s="211"/>
+      <c r="T27" s="211"/>
+      <c r="U27" s="211"/>
+      <c r="V27" s="211" t="s">
         <v>663</v>
       </c>
-      <c r="W27" s="207"/>
-      <c r="X27" s="208" t="s">
+      <c r="W27" s="211"/>
+      <c r="X27" s="212" t="s">
         <v>664</v>
       </c>
-      <c r="Y27" s="208"/>
-      <c r="Z27" s="208"/>
-      <c r="AA27" s="208"/>
-      <c r="AB27" s="208"/>
-      <c r="AC27" s="208"/>
-      <c r="AD27" s="173" t="s">
+      <c r="Y27" s="212"/>
+      <c r="Z27" s="212"/>
+      <c r="AA27" s="212"/>
+      <c r="AB27" s="212"/>
+      <c r="AC27" s="212"/>
+      <c r="AD27" s="176" t="s">
         <v>693</v>
       </c>
-      <c r="AE27" s="173"/>
-      <c r="AF27" s="173"/>
-      <c r="AG27" s="173"/>
+      <c r="AE27" s="176"/>
+      <c r="AF27" s="176"/>
+      <c r="AG27" s="176"/>
       <c r="AH27" s="2"/>
       <c r="AI27" s="2"/>
       <c r="AJ27" s="2"/>
@@ -9727,40 +9727,40 @@
     </row>
     <row r="28" spans="1:271" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
-      <c r="B28" s="194" t="s">
+      <c r="B28" s="175" t="s">
         <v>692</v>
       </c>
-      <c r="C28" s="194"/>
-      <c r="D28" s="194"/>
-      <c r="E28" s="194"/>
-      <c r="F28" s="194"/>
-      <c r="G28" s="194"/>
-      <c r="H28" s="194"/>
-      <c r="I28" s="194"/>
-      <c r="J28" s="194"/>
-      <c r="K28" s="194"/>
-      <c r="L28" s="194"/>
-      <c r="M28" s="194"/>
-      <c r="N28" s="194"/>
-      <c r="O28" s="194"/>
-      <c r="P28" s="194"/>
-      <c r="Q28" s="194"/>
-      <c r="R28" s="194"/>
-      <c r="S28" s="194"/>
-      <c r="T28" s="194"/>
-      <c r="U28" s="194"/>
-      <c r="V28" s="194"/>
-      <c r="W28" s="194"/>
-      <c r="X28" s="194"/>
-      <c r="Y28" s="194"/>
-      <c r="Z28" s="194"/>
-      <c r="AA28" s="194"/>
-      <c r="AB28" s="194"/>
-      <c r="AC28" s="194"/>
-      <c r="AD28" s="194"/>
-      <c r="AE28" s="194"/>
-      <c r="AF28" s="194"/>
-      <c r="AG28" s="194"/>
+      <c r="C28" s="175"/>
+      <c r="D28" s="175"/>
+      <c r="E28" s="175"/>
+      <c r="F28" s="175"/>
+      <c r="G28" s="175"/>
+      <c r="H28" s="175"/>
+      <c r="I28" s="175"/>
+      <c r="J28" s="175"/>
+      <c r="K28" s="175"/>
+      <c r="L28" s="175"/>
+      <c r="M28" s="175"/>
+      <c r="N28" s="175"/>
+      <c r="O28" s="175"/>
+      <c r="P28" s="175"/>
+      <c r="Q28" s="175"/>
+      <c r="R28" s="175"/>
+      <c r="S28" s="175"/>
+      <c r="T28" s="175"/>
+      <c r="U28" s="175"/>
+      <c r="V28" s="175"/>
+      <c r="W28" s="175"/>
+      <c r="X28" s="175"/>
+      <c r="Y28" s="175"/>
+      <c r="Z28" s="175"/>
+      <c r="AA28" s="175"/>
+      <c r="AB28" s="175"/>
+      <c r="AC28" s="175"/>
+      <c r="AD28" s="175"/>
+      <c r="AE28" s="175"/>
+      <c r="AF28" s="175"/>
+      <c r="AG28" s="175"/>
       <c r="AH28" s="2"/>
       <c r="AI28" s="2"/>
       <c r="AJ28" s="2"/>
@@ -9998,51 +9998,51 @@
       <c r="B29" s="171" t="s">
         <v>712</v>
       </c>
-      <c r="C29" s="206" t="s">
+      <c r="C29" s="210" t="s">
         <v>474</v>
       </c>
-      <c r="D29" s="206"/>
-      <c r="E29" s="206"/>
-      <c r="F29" s="206"/>
-      <c r="G29" s="206"/>
-      <c r="H29" s="206"/>
-      <c r="I29" s="206" t="s">
+      <c r="D29" s="210"/>
+      <c r="E29" s="210"/>
+      <c r="F29" s="210"/>
+      <c r="G29" s="210"/>
+      <c r="H29" s="210"/>
+      <c r="I29" s="210" t="s">
         <v>713</v>
       </c>
-      <c r="J29" s="206"/>
-      <c r="K29" s="206"/>
-      <c r="L29" s="206"/>
-      <c r="M29" s="206" t="s">
+      <c r="J29" s="210"/>
+      <c r="K29" s="210"/>
+      <c r="L29" s="210"/>
+      <c r="M29" s="210" t="s">
         <v>714</v>
       </c>
-      <c r="N29" s="206"/>
-      <c r="O29" s="206"/>
-      <c r="P29" s="206" t="s">
+      <c r="N29" s="210"/>
+      <c r="O29" s="210"/>
+      <c r="P29" s="210" t="s">
         <v>715</v>
       </c>
-      <c r="Q29" s="206"/>
-      <c r="R29" s="206"/>
-      <c r="S29" s="206"/>
-      <c r="T29" s="206" t="s">
+      <c r="Q29" s="210"/>
+      <c r="R29" s="210"/>
+      <c r="S29" s="210"/>
+      <c r="T29" s="210" t="s">
         <v>697</v>
       </c>
-      <c r="U29" s="206"/>
-      <c r="V29" s="206"/>
-      <c r="W29" s="206"/>
-      <c r="X29" s="206" t="s">
+      <c r="U29" s="210"/>
+      <c r="V29" s="210"/>
+      <c r="W29" s="210"/>
+      <c r="X29" s="210" t="s">
         <v>716</v>
       </c>
-      <c r="Y29" s="206"/>
-      <c r="Z29" s="206"/>
-      <c r="AA29" s="206"/>
-      <c r="AB29" s="206"/>
-      <c r="AC29" s="206"/>
-      <c r="AD29" s="206" t="s">
+      <c r="Y29" s="210"/>
+      <c r="Z29" s="210"/>
+      <c r="AA29" s="210"/>
+      <c r="AB29" s="210"/>
+      <c r="AC29" s="210"/>
+      <c r="AD29" s="210" t="s">
         <v>717</v>
       </c>
-      <c r="AE29" s="206"/>
-      <c r="AF29" s="206"/>
-      <c r="AG29" s="206"/>
+      <c r="AE29" s="210"/>
+      <c r="AF29" s="210"/>
+      <c r="AG29" s="210"/>
       <c r="AH29" s="2"/>
       <c r="AI29" s="2"/>
       <c r="AJ29" s="2"/>
@@ -10277,40 +10277,40 @@
     </row>
     <row r="30" spans="1:271" ht="22.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1"/>
-      <c r="B30" s="194" t="s">
+      <c r="B30" s="175" t="s">
         <v>694</v>
       </c>
-      <c r="C30" s="194"/>
-      <c r="D30" s="194"/>
-      <c r="E30" s="194"/>
-      <c r="F30" s="194"/>
-      <c r="G30" s="194"/>
-      <c r="H30" s="194"/>
-      <c r="I30" s="194"/>
-      <c r="J30" s="194"/>
-      <c r="K30" s="194"/>
-      <c r="L30" s="194"/>
-      <c r="M30" s="194"/>
-      <c r="N30" s="194"/>
-      <c r="O30" s="194"/>
-      <c r="P30" s="194"/>
-      <c r="Q30" s="194"/>
-      <c r="R30" s="194"/>
-      <c r="S30" s="194"/>
-      <c r="T30" s="194"/>
-      <c r="U30" s="194"/>
-      <c r="V30" s="194"/>
-      <c r="W30" s="194"/>
-      <c r="X30" s="194"/>
-      <c r="Y30" s="194"/>
-      <c r="Z30" s="194"/>
-      <c r="AA30" s="194"/>
-      <c r="AB30" s="194"/>
-      <c r="AC30" s="194"/>
-      <c r="AD30" s="194"/>
-      <c r="AE30" s="194"/>
-      <c r="AF30" s="194"/>
-      <c r="AG30" s="194"/>
+      <c r="C30" s="175"/>
+      <c r="D30" s="175"/>
+      <c r="E30" s="175"/>
+      <c r="F30" s="175"/>
+      <c r="G30" s="175"/>
+      <c r="H30" s="175"/>
+      <c r="I30" s="175"/>
+      <c r="J30" s="175"/>
+      <c r="K30" s="175"/>
+      <c r="L30" s="175"/>
+      <c r="M30" s="175"/>
+      <c r="N30" s="175"/>
+      <c r="O30" s="175"/>
+      <c r="P30" s="175"/>
+      <c r="Q30" s="175"/>
+      <c r="R30" s="175"/>
+      <c r="S30" s="175"/>
+      <c r="T30" s="175"/>
+      <c r="U30" s="175"/>
+      <c r="V30" s="175"/>
+      <c r="W30" s="175"/>
+      <c r="X30" s="175"/>
+      <c r="Y30" s="175"/>
+      <c r="Z30" s="175"/>
+      <c r="AA30" s="175"/>
+      <c r="AB30" s="175"/>
+      <c r="AC30" s="175"/>
+      <c r="AD30" s="175"/>
+      <c r="AE30" s="175"/>
+      <c r="AF30" s="175"/>
+      <c r="AG30" s="175"/>
       <c r="AH30" s="2"/>
       <c r="AI30" s="2"/>
       <c r="AJ30" s="2"/>
@@ -10548,45 +10548,45 @@
       <c r="B31" s="168" t="s">
         <v>1</v>
       </c>
-      <c r="C31" s="196" t="s">
+      <c r="C31" s="178" t="s">
         <v>563</v>
       </c>
-      <c r="D31" s="196"/>
-      <c r="E31" s="196"/>
-      <c r="F31" s="174"/>
-      <c r="G31" s="174"/>
-      <c r="H31" s="174"/>
-      <c r="I31" s="180" t="s">
+      <c r="D31" s="178"/>
+      <c r="E31" s="178"/>
+      <c r="F31" s="214"/>
+      <c r="G31" s="214"/>
+      <c r="H31" s="214"/>
+      <c r="I31" s="179" t="s">
         <v>718</v>
       </c>
-      <c r="J31" s="180"/>
-      <c r="K31" s="180"/>
-      <c r="L31" s="180"/>
-      <c r="M31" s="181"/>
-      <c r="N31" s="181"/>
-      <c r="O31" s="181"/>
-      <c r="P31" s="181"/>
-      <c r="Q31" s="180" t="s">
+      <c r="J31" s="179"/>
+      <c r="K31" s="179"/>
+      <c r="L31" s="179"/>
+      <c r="M31" s="190"/>
+      <c r="N31" s="190"/>
+      <c r="O31" s="190"/>
+      <c r="P31" s="190"/>
+      <c r="Q31" s="179" t="s">
         <v>719</v>
       </c>
-      <c r="R31" s="180"/>
-      <c r="S31" s="180"/>
-      <c r="T31" s="180"/>
-      <c r="U31" s="180"/>
-      <c r="V31" s="181"/>
-      <c r="W31" s="181"/>
-      <c r="X31" s="181"/>
-      <c r="Y31" s="217"/>
-      <c r="Z31" s="217"/>
-      <c r="AA31" s="196" t="s">
+      <c r="R31" s="179"/>
+      <c r="S31" s="179"/>
+      <c r="T31" s="179"/>
+      <c r="U31" s="179"/>
+      <c r="V31" s="190"/>
+      <c r="W31" s="190"/>
+      <c r="X31" s="190"/>
+      <c r="Y31" s="177"/>
+      <c r="Z31" s="177"/>
+      <c r="AA31" s="178" t="s">
         <v>565</v>
       </c>
-      <c r="AB31" s="196"/>
-      <c r="AC31" s="196"/>
-      <c r="AD31" s="174"/>
-      <c r="AE31" s="174"/>
-      <c r="AF31" s="174"/>
-      <c r="AG31" s="174"/>
+      <c r="AB31" s="178"/>
+      <c r="AC31" s="178"/>
+      <c r="AD31" s="214"/>
+      <c r="AE31" s="214"/>
+      <c r="AF31" s="214"/>
+      <c r="AG31" s="214"/>
       <c r="AH31" s="2"/>
       <c r="AI31" s="2"/>
       <c r="AJ31" s="2"/>
@@ -10824,45 +10824,45 @@
       <c r="B32" s="168" t="s">
         <v>3</v>
       </c>
-      <c r="C32" s="180" t="s">
+      <c r="C32" s="179" t="s">
         <v>564</v>
       </c>
-      <c r="D32" s="180"/>
-      <c r="E32" s="180"/>
-      <c r="F32" s="174"/>
-      <c r="G32" s="174"/>
-      <c r="H32" s="174"/>
-      <c r="I32" s="197" t="s">
+      <c r="D32" s="179"/>
+      <c r="E32" s="179"/>
+      <c r="F32" s="214"/>
+      <c r="G32" s="214"/>
+      <c r="H32" s="214"/>
+      <c r="I32" s="236" t="s">
         <v>684</v>
       </c>
-      <c r="J32" s="197"/>
-      <c r="K32" s="197"/>
-      <c r="L32" s="197"/>
-      <c r="M32" s="181"/>
-      <c r="N32" s="181"/>
-      <c r="O32" s="181"/>
-      <c r="P32" s="181"/>
-      <c r="Q32" s="180" t="s">
+      <c r="J32" s="236"/>
+      <c r="K32" s="236"/>
+      <c r="L32" s="236"/>
+      <c r="M32" s="190"/>
+      <c r="N32" s="190"/>
+      <c r="O32" s="190"/>
+      <c r="P32" s="190"/>
+      <c r="Q32" s="179" t="s">
         <v>562</v>
       </c>
-      <c r="R32" s="180"/>
-      <c r="S32" s="180"/>
-      <c r="T32" s="180"/>
-      <c r="U32" s="180"/>
-      <c r="V32" s="181"/>
-      <c r="W32" s="181"/>
-      <c r="X32" s="181"/>
-      <c r="Y32" s="217"/>
-      <c r="Z32" s="217"/>
-      <c r="AA32" s="196" t="s">
+      <c r="R32" s="179"/>
+      <c r="S32" s="179"/>
+      <c r="T32" s="179"/>
+      <c r="U32" s="179"/>
+      <c r="V32" s="190"/>
+      <c r="W32" s="190"/>
+      <c r="X32" s="190"/>
+      <c r="Y32" s="177"/>
+      <c r="Z32" s="177"/>
+      <c r="AA32" s="178" t="s">
         <v>565</v>
       </c>
-      <c r="AB32" s="196"/>
-      <c r="AC32" s="196"/>
-      <c r="AD32" s="174"/>
-      <c r="AE32" s="174"/>
-      <c r="AF32" s="174"/>
-      <c r="AG32" s="174"/>
+      <c r="AB32" s="178"/>
+      <c r="AC32" s="178"/>
+      <c r="AD32" s="214"/>
+      <c r="AE32" s="214"/>
+      <c r="AF32" s="214"/>
+      <c r="AG32" s="214"/>
       <c r="AH32" s="2"/>
       <c r="AI32" s="2"/>
       <c r="AJ32" s="2"/>
@@ -11100,45 +11100,45 @@
       <c r="B33" s="168" t="s">
         <v>4</v>
       </c>
-      <c r="C33" s="180" t="s">
+      <c r="C33" s="179" t="s">
         <v>564</v>
       </c>
-      <c r="D33" s="180"/>
-      <c r="E33" s="180"/>
-      <c r="F33" s="174"/>
-      <c r="G33" s="174"/>
-      <c r="H33" s="174"/>
-      <c r="I33" s="180" t="s">
+      <c r="D33" s="179"/>
+      <c r="E33" s="179"/>
+      <c r="F33" s="214"/>
+      <c r="G33" s="214"/>
+      <c r="H33" s="214"/>
+      <c r="I33" s="179" t="s">
         <v>557</v>
       </c>
-      <c r="J33" s="180"/>
-      <c r="K33" s="180"/>
-      <c r="L33" s="180"/>
-      <c r="M33" s="181"/>
-      <c r="N33" s="181"/>
-      <c r="O33" s="181"/>
-      <c r="P33" s="181"/>
-      <c r="Q33" s="180" t="s">
+      <c r="J33" s="179"/>
+      <c r="K33" s="179"/>
+      <c r="L33" s="179"/>
+      <c r="M33" s="190"/>
+      <c r="N33" s="190"/>
+      <c r="O33" s="190"/>
+      <c r="P33" s="190"/>
+      <c r="Q33" s="179" t="s">
         <v>562</v>
       </c>
-      <c r="R33" s="180"/>
-      <c r="S33" s="180"/>
-      <c r="T33" s="180"/>
-      <c r="U33" s="180"/>
-      <c r="V33" s="181"/>
-      <c r="W33" s="181"/>
-      <c r="X33" s="181"/>
-      <c r="Y33" s="217"/>
-      <c r="Z33" s="217"/>
-      <c r="AA33" s="196" t="s">
+      <c r="R33" s="179"/>
+      <c r="S33" s="179"/>
+      <c r="T33" s="179"/>
+      <c r="U33" s="179"/>
+      <c r="V33" s="190"/>
+      <c r="W33" s="190"/>
+      <c r="X33" s="190"/>
+      <c r="Y33" s="177"/>
+      <c r="Z33" s="177"/>
+      <c r="AA33" s="178" t="s">
         <v>565</v>
       </c>
-      <c r="AB33" s="196"/>
-      <c r="AC33" s="196"/>
-      <c r="AD33" s="174"/>
-      <c r="AE33" s="174"/>
-      <c r="AF33" s="174"/>
-      <c r="AG33" s="174"/>
+      <c r="AB33" s="178"/>
+      <c r="AC33" s="178"/>
+      <c r="AD33" s="214"/>
+      <c r="AE33" s="214"/>
+      <c r="AF33" s="214"/>
+      <c r="AG33" s="214"/>
       <c r="AH33" s="2"/>
       <c r="AI33" s="2"/>
       <c r="AJ33" s="2"/>
@@ -11376,45 +11376,45 @@
       <c r="B34" s="140" t="s">
         <v>486</v>
       </c>
-      <c r="C34" s="180" t="s">
+      <c r="C34" s="179" t="s">
         <v>566</v>
       </c>
-      <c r="D34" s="180"/>
-      <c r="E34" s="180"/>
-      <c r="F34" s="174"/>
-      <c r="G34" s="174"/>
-      <c r="H34" s="174"/>
-      <c r="I34" s="180" t="s">
+      <c r="D34" s="179"/>
+      <c r="E34" s="179"/>
+      <c r="F34" s="214"/>
+      <c r="G34" s="214"/>
+      <c r="H34" s="214"/>
+      <c r="I34" s="179" t="s">
         <v>685</v>
       </c>
-      <c r="J34" s="180"/>
-      <c r="K34" s="180"/>
-      <c r="L34" s="180"/>
-      <c r="M34" s="181"/>
-      <c r="N34" s="181"/>
-      <c r="O34" s="181"/>
-      <c r="P34" s="181"/>
-      <c r="Q34" s="180" t="s">
+      <c r="J34" s="179"/>
+      <c r="K34" s="179"/>
+      <c r="L34" s="179"/>
+      <c r="M34" s="190"/>
+      <c r="N34" s="190"/>
+      <c r="O34" s="190"/>
+      <c r="P34" s="190"/>
+      <c r="Q34" s="179" t="s">
         <v>562</v>
       </c>
-      <c r="R34" s="180"/>
-      <c r="S34" s="180"/>
-      <c r="T34" s="180"/>
-      <c r="U34" s="180"/>
-      <c r="V34" s="181"/>
-      <c r="W34" s="181"/>
-      <c r="X34" s="181"/>
-      <c r="Y34" s="217"/>
-      <c r="Z34" s="217"/>
-      <c r="AA34" s="196" t="s">
+      <c r="R34" s="179"/>
+      <c r="S34" s="179"/>
+      <c r="T34" s="179"/>
+      <c r="U34" s="179"/>
+      <c r="V34" s="190"/>
+      <c r="W34" s="190"/>
+      <c r="X34" s="190"/>
+      <c r="Y34" s="177"/>
+      <c r="Z34" s="177"/>
+      <c r="AA34" s="178" t="s">
         <v>565</v>
       </c>
-      <c r="AB34" s="196"/>
-      <c r="AC34" s="196"/>
-      <c r="AD34" s="174"/>
-      <c r="AE34" s="174"/>
-      <c r="AF34" s="174"/>
-      <c r="AG34" s="174"/>
+      <c r="AB34" s="178"/>
+      <c r="AC34" s="178"/>
+      <c r="AD34" s="214"/>
+      <c r="AE34" s="214"/>
+      <c r="AF34" s="214"/>
+      <c r="AG34" s="214"/>
       <c r="AH34" s="2"/>
       <c r="AI34" s="2"/>
       <c r="AJ34" s="2"/>
@@ -11652,45 +11652,45 @@
       <c r="B35" s="168" t="s">
         <v>689</v>
       </c>
-      <c r="C35" s="175"/>
-      <c r="D35" s="175"/>
-      <c r="E35" s="175"/>
-      <c r="F35" s="175"/>
-      <c r="G35" s="175"/>
-      <c r="H35" s="175"/>
-      <c r="I35" s="180" t="s">
+      <c r="C35" s="195"/>
+      <c r="D35" s="195"/>
+      <c r="E35" s="195"/>
+      <c r="F35" s="195"/>
+      <c r="G35" s="195"/>
+      <c r="H35" s="195"/>
+      <c r="I35" s="179" t="s">
         <v>690</v>
       </c>
-      <c r="J35" s="180"/>
-      <c r="K35" s="180"/>
-      <c r="L35" s="180"/>
-      <c r="M35" s="199"/>
-      <c r="N35" s="199"/>
-      <c r="O35" s="199"/>
-      <c r="P35" s="199"/>
-      <c r="Q35" s="180" t="s">
+      <c r="J35" s="179"/>
+      <c r="K35" s="179"/>
+      <c r="L35" s="179"/>
+      <c r="M35" s="174"/>
+      <c r="N35" s="174"/>
+      <c r="O35" s="174"/>
+      <c r="P35" s="174"/>
+      <c r="Q35" s="179" t="s">
         <v>660</v>
       </c>
-      <c r="R35" s="180"/>
-      <c r="S35" s="180"/>
-      <c r="T35" s="180"/>
-      <c r="U35" s="180"/>
-      <c r="V35" s="173" t="s">
+      <c r="R35" s="179"/>
+      <c r="S35" s="179"/>
+      <c r="T35" s="179"/>
+      <c r="U35" s="179"/>
+      <c r="V35" s="176" t="s">
         <v>455</v>
       </c>
-      <c r="W35" s="173"/>
-      <c r="X35" s="175"/>
-      <c r="Y35" s="175"/>
-      <c r="Z35" s="175"/>
-      <c r="AA35" s="175"/>
-      <c r="AB35" s="173" t="s">
+      <c r="W35" s="176"/>
+      <c r="X35" s="195"/>
+      <c r="Y35" s="195"/>
+      <c r="Z35" s="195"/>
+      <c r="AA35" s="195"/>
+      <c r="AB35" s="176" t="s">
         <v>456</v>
       </c>
-      <c r="AC35" s="173"/>
-      <c r="AD35" s="175"/>
-      <c r="AE35" s="175"/>
-      <c r="AF35" s="175"/>
-      <c r="AG35" s="175"/>
+      <c r="AC35" s="176"/>
+      <c r="AD35" s="195"/>
+      <c r="AE35" s="195"/>
+      <c r="AF35" s="195"/>
+      <c r="AG35" s="195"/>
       <c r="AH35" s="2"/>
       <c r="AI35" s="2"/>
       <c r="AJ35" s="2"/>
@@ -11928,41 +11928,41 @@
       <c r="B36" s="168" t="s">
         <v>567</v>
       </c>
-      <c r="C36" s="180" t="s">
+      <c r="C36" s="179" t="s">
         <v>568</v>
       </c>
-      <c r="D36" s="180"/>
-      <c r="E36" s="180"/>
-      <c r="F36" s="180"/>
-      <c r="G36" s="180"/>
-      <c r="H36" s="180"/>
-      <c r="I36" s="181"/>
-      <c r="J36" s="181"/>
-      <c r="K36" s="181"/>
-      <c r="L36" s="181"/>
-      <c r="M36" s="181"/>
-      <c r="N36" s="181"/>
-      <c r="O36" s="181"/>
-      <c r="P36" s="181"/>
-      <c r="Q36" s="181"/>
-      <c r="R36" s="181"/>
-      <c r="S36" s="181"/>
-      <c r="T36" s="181"/>
-      <c r="U36" s="181"/>
-      <c r="V36" s="181"/>
-      <c r="W36" s="181"/>
-      <c r="X36" s="195" t="s">
+      <c r="D36" s="179"/>
+      <c r="E36" s="179"/>
+      <c r="F36" s="179"/>
+      <c r="G36" s="179"/>
+      <c r="H36" s="179"/>
+      <c r="I36" s="190"/>
+      <c r="J36" s="190"/>
+      <c r="K36" s="190"/>
+      <c r="L36" s="190"/>
+      <c r="M36" s="190"/>
+      <c r="N36" s="190"/>
+      <c r="O36" s="190"/>
+      <c r="P36" s="190"/>
+      <c r="Q36" s="190"/>
+      <c r="R36" s="190"/>
+      <c r="S36" s="190"/>
+      <c r="T36" s="190"/>
+      <c r="U36" s="190"/>
+      <c r="V36" s="190"/>
+      <c r="W36" s="190"/>
+      <c r="X36" s="235" t="s">
         <v>569</v>
       </c>
-      <c r="Y36" s="195"/>
-      <c r="Z36" s="195"/>
-      <c r="AA36" s="195"/>
-      <c r="AB36" s="195"/>
-      <c r="AC36" s="195"/>
-      <c r="AD36" s="174"/>
-      <c r="AE36" s="174"/>
-      <c r="AF36" s="174"/>
-      <c r="AG36" s="174"/>
+      <c r="Y36" s="235"/>
+      <c r="Z36" s="235"/>
+      <c r="AA36" s="235"/>
+      <c r="AB36" s="235"/>
+      <c r="AC36" s="235"/>
+      <c r="AD36" s="214"/>
+      <c r="AE36" s="214"/>
+      <c r="AF36" s="214"/>
+      <c r="AG36" s="214"/>
       <c r="AH36" s="2"/>
       <c r="AI36" s="2"/>
       <c r="AJ36" s="2"/>
@@ -12200,41 +12200,41 @@
       <c r="B37" s="150" t="s">
         <v>720</v>
       </c>
-      <c r="C37" s="203"/>
-      <c r="D37" s="203"/>
-      <c r="E37" s="203"/>
-      <c r="F37" s="203"/>
-      <c r="G37" s="203"/>
-      <c r="H37" s="203"/>
-      <c r="I37" s="203"/>
-      <c r="J37" s="203"/>
-      <c r="K37" s="204"/>
-      <c r="L37" s="204"/>
-      <c r="M37" s="205" t="s">
+      <c r="C37" s="217"/>
+      <c r="D37" s="217"/>
+      <c r="E37" s="217"/>
+      <c r="F37" s="217"/>
+      <c r="G37" s="217"/>
+      <c r="H37" s="217"/>
+      <c r="I37" s="217"/>
+      <c r="J37" s="217"/>
+      <c r="K37" s="218"/>
+      <c r="L37" s="218"/>
+      <c r="M37" s="219" t="s">
         <v>721</v>
       </c>
-      <c r="N37" s="205"/>
-      <c r="O37" s="205"/>
-      <c r="P37" s="205"/>
-      <c r="Q37" s="200"/>
-      <c r="R37" s="200"/>
-      <c r="S37" s="200"/>
-      <c r="T37" s="200"/>
-      <c r="U37" s="200"/>
-      <c r="V37" s="201"/>
-      <c r="W37" s="201"/>
-      <c r="X37" s="202" t="s">
+      <c r="N37" s="219"/>
+      <c r="O37" s="219"/>
+      <c r="P37" s="219"/>
+      <c r="Q37" s="215"/>
+      <c r="R37" s="215"/>
+      <c r="S37" s="215"/>
+      <c r="T37" s="215"/>
+      <c r="U37" s="215"/>
+      <c r="V37" s="216"/>
+      <c r="W37" s="216"/>
+      <c r="X37" s="187" t="s">
         <v>696</v>
       </c>
-      <c r="Y37" s="202"/>
-      <c r="Z37" s="202"/>
-      <c r="AA37" s="202"/>
-      <c r="AB37" s="202"/>
-      <c r="AC37" s="202"/>
-      <c r="AD37" s="232"/>
-      <c r="AE37" s="232"/>
-      <c r="AF37" s="232"/>
-      <c r="AG37" s="232"/>
+      <c r="Y37" s="187"/>
+      <c r="Z37" s="187"/>
+      <c r="AA37" s="187"/>
+      <c r="AB37" s="187"/>
+      <c r="AC37" s="187"/>
+      <c r="AD37" s="185"/>
+      <c r="AE37" s="185"/>
+      <c r="AF37" s="185"/>
+      <c r="AG37" s="185"/>
       <c r="AH37" s="2"/>
       <c r="AI37" s="2"/>
       <c r="AJ37" s="2"/>
@@ -12502,619 +12502,722 @@
       <c r="AG38" s="153"/>
     </row>
     <row r="39" spans="1:268" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="233" t="s">
+      <c r="B39" s="181" t="s">
         <v>574</v>
       </c>
-      <c r="C39" s="233"/>
-      <c r="D39" s="233"/>
-      <c r="E39" s="233"/>
-      <c r="F39" s="233"/>
-      <c r="G39" s="233"/>
-      <c r="H39" s="233"/>
-      <c r="I39" s="233"/>
-      <c r="J39" s="233"/>
-      <c r="K39" s="233"/>
-      <c r="L39" s="233"/>
-      <c r="M39" s="233"/>
-      <c r="N39" s="233"/>
-      <c r="O39" s="233"/>
-      <c r="P39" s="233"/>
-      <c r="Q39" s="233"/>
-      <c r="R39" s="233"/>
-      <c r="S39" s="233"/>
-      <c r="T39" s="233"/>
-      <c r="U39" s="233"/>
-      <c r="V39" s="233"/>
-      <c r="W39" s="233"/>
-      <c r="X39" s="233"/>
-      <c r="Y39" s="233"/>
-      <c r="Z39" s="233"/>
-      <c r="AA39" s="233"/>
-      <c r="AB39" s="233"/>
-      <c r="AC39" s="233"/>
-      <c r="AD39" s="233"/>
-      <c r="AE39" s="233"/>
-      <c r="AF39" s="233"/>
-      <c r="AG39" s="233"/>
+      <c r="C39" s="181"/>
+      <c r="D39" s="181"/>
+      <c r="E39" s="181"/>
+      <c r="F39" s="181"/>
+      <c r="G39" s="181"/>
+      <c r="H39" s="181"/>
+      <c r="I39" s="181"/>
+      <c r="J39" s="181"/>
+      <c r="K39" s="181"/>
+      <c r="L39" s="181"/>
+      <c r="M39" s="181"/>
+      <c r="N39" s="181"/>
+      <c r="O39" s="181"/>
+      <c r="P39" s="181"/>
+      <c r="Q39" s="181"/>
+      <c r="R39" s="181"/>
+      <c r="S39" s="181"/>
+      <c r="T39" s="181"/>
+      <c r="U39" s="181"/>
+      <c r="V39" s="181"/>
+      <c r="W39" s="181"/>
+      <c r="X39" s="181"/>
+      <c r="Y39" s="181"/>
+      <c r="Z39" s="181"/>
+      <c r="AA39" s="181"/>
+      <c r="AB39" s="181"/>
+      <c r="AC39" s="181"/>
+      <c r="AD39" s="181"/>
+      <c r="AE39" s="181"/>
+      <c r="AF39" s="181"/>
+      <c r="AG39" s="181"/>
     </row>
     <row r="40" spans="1:268" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="179" t="s">
+      <c r="B40" s="182" t="s">
         <v>575</v>
       </c>
-      <c r="C40" s="179"/>
-      <c r="D40" s="179"/>
-      <c r="E40" s="179"/>
-      <c r="F40" s="179"/>
-      <c r="G40" s="179"/>
-      <c r="H40" s="179"/>
-      <c r="I40" s="179"/>
-      <c r="J40" s="179"/>
-      <c r="K40" s="179"/>
-      <c r="L40" s="179"/>
-      <c r="M40" s="179"/>
-      <c r="N40" s="179"/>
-      <c r="O40" s="179"/>
-      <c r="P40" s="179"/>
-      <c r="Q40" s="179"/>
-      <c r="R40" s="179"/>
-      <c r="S40" s="179"/>
-      <c r="T40" s="179"/>
-      <c r="U40" s="179"/>
-      <c r="V40" s="179"/>
-      <c r="W40" s="179"/>
-      <c r="X40" s="179"/>
-      <c r="Y40" s="179"/>
-      <c r="Z40" s="179"/>
-      <c r="AA40" s="179"/>
-      <c r="AB40" s="179"/>
-      <c r="AC40" s="179"/>
-      <c r="AD40" s="179"/>
-      <c r="AE40" s="179"/>
-      <c r="AF40" s="179"/>
-      <c r="AG40" s="179"/>
+      <c r="C40" s="182"/>
+      <c r="D40" s="182"/>
+      <c r="E40" s="182"/>
+      <c r="F40" s="182"/>
+      <c r="G40" s="182"/>
+      <c r="H40" s="182"/>
+      <c r="I40" s="182"/>
+      <c r="J40" s="182"/>
+      <c r="K40" s="182"/>
+      <c r="L40" s="182"/>
+      <c r="M40" s="182"/>
+      <c r="N40" s="182"/>
+      <c r="O40" s="182"/>
+      <c r="P40" s="182"/>
+      <c r="Q40" s="182"/>
+      <c r="R40" s="182"/>
+      <c r="S40" s="182"/>
+      <c r="T40" s="182"/>
+      <c r="U40" s="182"/>
+      <c r="V40" s="182"/>
+      <c r="W40" s="182"/>
+      <c r="X40" s="182"/>
+      <c r="Y40" s="182"/>
+      <c r="Z40" s="182"/>
+      <c r="AA40" s="182"/>
+      <c r="AB40" s="182"/>
+      <c r="AC40" s="182"/>
+      <c r="AD40" s="182"/>
+      <c r="AE40" s="182"/>
+      <c r="AF40" s="182"/>
+      <c r="AG40" s="182"/>
     </row>
     <row r="41" spans="1:268" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B41" s="173" t="s">
+      <c r="B41" s="176" t="s">
         <v>570</v>
       </c>
-      <c r="C41" s="173"/>
-      <c r="D41" s="173"/>
-      <c r="E41" s="173"/>
-      <c r="F41" s="173"/>
-      <c r="G41" s="173"/>
-      <c r="H41" s="173"/>
-      <c r="I41" s="173"/>
-      <c r="J41" s="173"/>
-      <c r="K41" s="173"/>
-      <c r="L41" s="173"/>
-      <c r="M41" s="173"/>
-      <c r="N41" s="173"/>
-      <c r="O41" s="173"/>
-      <c r="P41" s="173"/>
-      <c r="Q41" s="173"/>
-      <c r="R41" s="172" t="s">
+      <c r="C41" s="176"/>
+      <c r="D41" s="176"/>
+      <c r="E41" s="176"/>
+      <c r="F41" s="176"/>
+      <c r="G41" s="176"/>
+      <c r="H41" s="176"/>
+      <c r="I41" s="176"/>
+      <c r="J41" s="176"/>
+      <c r="K41" s="176"/>
+      <c r="L41" s="176"/>
+      <c r="M41" s="176"/>
+      <c r="N41" s="176"/>
+      <c r="O41" s="176"/>
+      <c r="P41" s="176"/>
+      <c r="Q41" s="176"/>
+      <c r="R41" s="183" t="s">
         <v>571</v>
       </c>
-      <c r="S41" s="172"/>
-      <c r="T41" s="172"/>
-      <c r="U41" s="172"/>
-      <c r="V41" s="172"/>
-      <c r="W41" s="172"/>
-      <c r="X41" s="172"/>
-      <c r="Y41" s="172"/>
-      <c r="Z41" s="172"/>
-      <c r="AA41" s="172"/>
-      <c r="AB41" s="172"/>
-      <c r="AC41" s="172"/>
-      <c r="AD41" s="172"/>
-      <c r="AE41" s="172"/>
-      <c r="AF41" s="172"/>
-      <c r="AG41" s="172"/>
+      <c r="S41" s="183"/>
+      <c r="T41" s="183"/>
+      <c r="U41" s="183"/>
+      <c r="V41" s="183"/>
+      <c r="W41" s="183"/>
+      <c r="X41" s="183"/>
+      <c r="Y41" s="183"/>
+      <c r="Z41" s="183"/>
+      <c r="AA41" s="183"/>
+      <c r="AB41" s="183"/>
+      <c r="AC41" s="183"/>
+      <c r="AD41" s="183"/>
+      <c r="AE41" s="183"/>
+      <c r="AF41" s="183"/>
+      <c r="AG41" s="183"/>
     </row>
     <row r="42" spans="1:268" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="179" t="s">
+      <c r="B42" s="182" t="s">
         <v>579</v>
       </c>
-      <c r="C42" s="179"/>
-      <c r="D42" s="179"/>
-      <c r="E42" s="179"/>
-      <c r="F42" s="179"/>
-      <c r="G42" s="179"/>
-      <c r="H42" s="179"/>
-      <c r="I42" s="179"/>
-      <c r="J42" s="179"/>
-      <c r="K42" s="179"/>
-      <c r="L42" s="179"/>
-      <c r="M42" s="179"/>
-      <c r="N42" s="179"/>
-      <c r="O42" s="179"/>
-      <c r="P42" s="179"/>
-      <c r="Q42" s="179"/>
-      <c r="R42" s="179"/>
-      <c r="S42" s="179"/>
-      <c r="T42" s="179"/>
-      <c r="U42" s="179"/>
-      <c r="V42" s="179"/>
-      <c r="W42" s="179"/>
-      <c r="X42" s="179"/>
-      <c r="Y42" s="179"/>
-      <c r="Z42" s="179"/>
-      <c r="AA42" s="179"/>
-      <c r="AB42" s="179"/>
-      <c r="AC42" s="179"/>
-      <c r="AD42" s="179"/>
-      <c r="AE42" s="179"/>
-      <c r="AF42" s="179"/>
-      <c r="AG42" s="179"/>
+      <c r="C42" s="182"/>
+      <c r="D42" s="182"/>
+      <c r="E42" s="182"/>
+      <c r="F42" s="182"/>
+      <c r="G42" s="182"/>
+      <c r="H42" s="182"/>
+      <c r="I42" s="182"/>
+      <c r="J42" s="182"/>
+      <c r="K42" s="182"/>
+      <c r="L42" s="182"/>
+      <c r="M42" s="182"/>
+      <c r="N42" s="182"/>
+      <c r="O42" s="182"/>
+      <c r="P42" s="182"/>
+      <c r="Q42" s="182"/>
+      <c r="R42" s="182"/>
+      <c r="S42" s="182"/>
+      <c r="T42" s="182"/>
+      <c r="U42" s="182"/>
+      <c r="V42" s="182"/>
+      <c r="W42" s="182"/>
+      <c r="X42" s="182"/>
+      <c r="Y42" s="182"/>
+      <c r="Z42" s="182"/>
+      <c r="AA42" s="182"/>
+      <c r="AB42" s="182"/>
+      <c r="AC42" s="182"/>
+      <c r="AD42" s="182"/>
+      <c r="AE42" s="182"/>
+      <c r="AF42" s="182"/>
+      <c r="AG42" s="182"/>
     </row>
     <row r="43" spans="1:268" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="173" t="s">
+      <c r="B43" s="176" t="s">
         <v>572</v>
       </c>
-      <c r="C43" s="173"/>
-      <c r="D43" s="173"/>
-      <c r="E43" s="173"/>
-      <c r="F43" s="173"/>
-      <c r="G43" s="173"/>
-      <c r="H43" s="173"/>
-      <c r="I43" s="173"/>
-      <c r="J43" s="173"/>
-      <c r="K43" s="173"/>
-      <c r="L43" s="173"/>
-      <c r="M43" s="173"/>
-      <c r="N43" s="173"/>
-      <c r="O43" s="173"/>
-      <c r="P43" s="173"/>
-      <c r="Q43" s="173"/>
-      <c r="R43" s="172" t="s">
+      <c r="C43" s="176"/>
+      <c r="D43" s="176"/>
+      <c r="E43" s="176"/>
+      <c r="F43" s="176"/>
+      <c r="G43" s="176"/>
+      <c r="H43" s="176"/>
+      <c r="I43" s="176"/>
+      <c r="J43" s="176"/>
+      <c r="K43" s="176"/>
+      <c r="L43" s="176"/>
+      <c r="M43" s="176"/>
+      <c r="N43" s="176"/>
+      <c r="O43" s="176"/>
+      <c r="P43" s="176"/>
+      <c r="Q43" s="176"/>
+      <c r="R43" s="183" t="s">
         <v>571</v>
       </c>
-      <c r="S43" s="172"/>
-      <c r="T43" s="172"/>
-      <c r="U43" s="172"/>
-      <c r="V43" s="172"/>
-      <c r="W43" s="172"/>
-      <c r="X43" s="172"/>
-      <c r="Y43" s="172"/>
-      <c r="Z43" s="172"/>
-      <c r="AA43" s="172"/>
-      <c r="AB43" s="172"/>
-      <c r="AC43" s="172"/>
-      <c r="AD43" s="172"/>
-      <c r="AE43" s="172"/>
-      <c r="AF43" s="172"/>
-      <c r="AG43" s="172"/>
+      <c r="S43" s="183"/>
+      <c r="T43" s="183"/>
+      <c r="U43" s="183"/>
+      <c r="V43" s="183"/>
+      <c r="W43" s="183"/>
+      <c r="X43" s="183"/>
+      <c r="Y43" s="183"/>
+      <c r="Z43" s="183"/>
+      <c r="AA43" s="183"/>
+      <c r="AB43" s="183"/>
+      <c r="AC43" s="183"/>
+      <c r="AD43" s="183"/>
+      <c r="AE43" s="183"/>
+      <c r="AF43" s="183"/>
+      <c r="AG43" s="183"/>
     </row>
     <row r="44" spans="1:268" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B44" s="198" t="s">
+      <c r="B44" s="180" t="s">
         <v>585</v>
       </c>
-      <c r="C44" s="198"/>
-      <c r="D44" s="198"/>
-      <c r="E44" s="198"/>
-      <c r="F44" s="198"/>
-      <c r="G44" s="198"/>
-      <c r="H44" s="198"/>
-      <c r="I44" s="198"/>
-      <c r="J44" s="198"/>
-      <c r="K44" s="198"/>
-      <c r="L44" s="198"/>
-      <c r="M44" s="198"/>
-      <c r="N44" s="198"/>
-      <c r="O44" s="198"/>
-      <c r="P44" s="198"/>
-      <c r="Q44" s="198"/>
-      <c r="R44" s="198"/>
-      <c r="S44" s="198"/>
-      <c r="T44" s="198"/>
-      <c r="U44" s="198"/>
-      <c r="V44" s="198"/>
-      <c r="W44" s="198"/>
-      <c r="X44" s="198"/>
-      <c r="Y44" s="198"/>
-      <c r="Z44" s="198"/>
-      <c r="AA44" s="198"/>
-      <c r="AB44" s="198"/>
-      <c r="AC44" s="198"/>
-      <c r="AD44" s="198"/>
-      <c r="AE44" s="198"/>
-      <c r="AF44" s="198"/>
-      <c r="AG44" s="198"/>
+      <c r="C44" s="180"/>
+      <c r="D44" s="180"/>
+      <c r="E44" s="180"/>
+      <c r="F44" s="180"/>
+      <c r="G44" s="180"/>
+      <c r="H44" s="180"/>
+      <c r="I44" s="180"/>
+      <c r="J44" s="180"/>
+      <c r="K44" s="180"/>
+      <c r="L44" s="180"/>
+      <c r="M44" s="180"/>
+      <c r="N44" s="180"/>
+      <c r="O44" s="180"/>
+      <c r="P44" s="180"/>
+      <c r="Q44" s="180"/>
+      <c r="R44" s="180"/>
+      <c r="S44" s="180"/>
+      <c r="T44" s="180"/>
+      <c r="U44" s="180"/>
+      <c r="V44" s="180"/>
+      <c r="W44" s="180"/>
+      <c r="X44" s="180"/>
+      <c r="Y44" s="180"/>
+      <c r="Z44" s="180"/>
+      <c r="AA44" s="180"/>
+      <c r="AB44" s="180"/>
+      <c r="AC44" s="180"/>
+      <c r="AD44" s="180"/>
+      <c r="AE44" s="180"/>
+      <c r="AF44" s="180"/>
+      <c r="AG44" s="180"/>
     </row>
     <row r="45" spans="1:268" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B45" s="179" t="s">
+      <c r="B45" s="182" t="s">
         <v>584</v>
       </c>
-      <c r="C45" s="179"/>
-      <c r="D45" s="179"/>
-      <c r="E45" s="179"/>
-      <c r="F45" s="179"/>
-      <c r="G45" s="179"/>
-      <c r="H45" s="179"/>
-      <c r="I45" s="179"/>
-      <c r="J45" s="179"/>
-      <c r="K45" s="179"/>
-      <c r="L45" s="179"/>
-      <c r="M45" s="179"/>
-      <c r="N45" s="179"/>
-      <c r="O45" s="179"/>
-      <c r="P45" s="179"/>
-      <c r="Q45" s="179"/>
-      <c r="R45" s="179"/>
-      <c r="S45" s="179"/>
-      <c r="T45" s="179"/>
-      <c r="U45" s="179"/>
-      <c r="V45" s="179"/>
-      <c r="W45" s="179"/>
-      <c r="X45" s="179"/>
-      <c r="Y45" s="179"/>
-      <c r="Z45" s="179"/>
-      <c r="AA45" s="179"/>
-      <c r="AB45" s="179"/>
-      <c r="AC45" s="179"/>
-      <c r="AD45" s="179"/>
-      <c r="AE45" s="179"/>
-      <c r="AF45" s="179"/>
-      <c r="AG45" s="179"/>
+      <c r="C45" s="182"/>
+      <c r="D45" s="182"/>
+      <c r="E45" s="182"/>
+      <c r="F45" s="182"/>
+      <c r="G45" s="182"/>
+      <c r="H45" s="182"/>
+      <c r="I45" s="182"/>
+      <c r="J45" s="182"/>
+      <c r="K45" s="182"/>
+      <c r="L45" s="182"/>
+      <c r="M45" s="182"/>
+      <c r="N45" s="182"/>
+      <c r="O45" s="182"/>
+      <c r="P45" s="182"/>
+      <c r="Q45" s="182"/>
+      <c r="R45" s="182"/>
+      <c r="S45" s="182"/>
+      <c r="T45" s="182"/>
+      <c r="U45" s="182"/>
+      <c r="V45" s="182"/>
+      <c r="W45" s="182"/>
+      <c r="X45" s="182"/>
+      <c r="Y45" s="182"/>
+      <c r="Z45" s="182"/>
+      <c r="AA45" s="182"/>
+      <c r="AB45" s="182"/>
+      <c r="AC45" s="182"/>
+      <c r="AD45" s="182"/>
+      <c r="AE45" s="182"/>
+      <c r="AF45" s="182"/>
+      <c r="AG45" s="182"/>
     </row>
     <row r="46" spans="1:268" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B46" s="173" t="s">
+      <c r="B46" s="176" t="s">
         <v>580</v>
       </c>
-      <c r="C46" s="173"/>
-      <c r="D46" s="173"/>
-      <c r="E46" s="173"/>
-      <c r="F46" s="173"/>
-      <c r="G46" s="173"/>
-      <c r="H46" s="173"/>
-      <c r="I46" s="173"/>
-      <c r="J46" s="173"/>
-      <c r="K46" s="173"/>
-      <c r="L46" s="173"/>
-      <c r="M46" s="173"/>
-      <c r="N46" s="173"/>
-      <c r="O46" s="173"/>
-      <c r="P46" s="173"/>
-      <c r="Q46" s="173"/>
-      <c r="R46" s="173" t="s">
+      <c r="C46" s="176"/>
+      <c r="D46" s="176"/>
+      <c r="E46" s="176"/>
+      <c r="F46" s="176"/>
+      <c r="G46" s="176"/>
+      <c r="H46" s="176"/>
+      <c r="I46" s="176"/>
+      <c r="J46" s="176"/>
+      <c r="K46" s="176"/>
+      <c r="L46" s="176"/>
+      <c r="M46" s="176"/>
+      <c r="N46" s="176"/>
+      <c r="O46" s="176"/>
+      <c r="P46" s="176"/>
+      <c r="Q46" s="176"/>
+      <c r="R46" s="176" t="s">
         <v>581</v>
       </c>
-      <c r="S46" s="173"/>
-      <c r="T46" s="173"/>
-      <c r="U46" s="173"/>
-      <c r="V46" s="176" t="s">
+      <c r="S46" s="176"/>
+      <c r="T46" s="176"/>
+      <c r="U46" s="176"/>
+      <c r="V46" s="232" t="s">
         <v>708</v>
       </c>
-      <c r="W46" s="177"/>
-      <c r="X46" s="177"/>
-      <c r="Y46" s="178"/>
-      <c r="Z46" s="176" t="s">
+      <c r="W46" s="233"/>
+      <c r="X46" s="233"/>
+      <c r="Y46" s="234"/>
+      <c r="Z46" s="232" t="s">
         <v>702</v>
       </c>
-      <c r="AA46" s="177"/>
-      <c r="AB46" s="177"/>
-      <c r="AC46" s="178"/>
-      <c r="AD46" s="172" t="s">
+      <c r="AA46" s="233"/>
+      <c r="AB46" s="233"/>
+      <c r="AC46" s="234"/>
+      <c r="AD46" s="183" t="s">
         <v>5</v>
       </c>
-      <c r="AE46" s="172"/>
-      <c r="AF46" s="172"/>
-      <c r="AG46" s="172"/>
+      <c r="AE46" s="183"/>
+      <c r="AF46" s="183"/>
+      <c r="AG46" s="183"/>
     </row>
     <row r="47" spans="1:268" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B47" s="179" t="s">
+      <c r="B47" s="182" t="s">
         <v>586</v>
       </c>
-      <c r="C47" s="179"/>
-      <c r="D47" s="179"/>
-      <c r="E47" s="179"/>
-      <c r="F47" s="179"/>
-      <c r="G47" s="179"/>
-      <c r="H47" s="179"/>
-      <c r="I47" s="179"/>
-      <c r="J47" s="179"/>
-      <c r="K47" s="179"/>
-      <c r="L47" s="179"/>
-      <c r="M47" s="179"/>
-      <c r="N47" s="179"/>
-      <c r="O47" s="179"/>
-      <c r="P47" s="179"/>
-      <c r="Q47" s="179"/>
-      <c r="R47" s="179"/>
-      <c r="S47" s="179"/>
-      <c r="T47" s="179"/>
-      <c r="U47" s="179"/>
-      <c r="V47" s="179"/>
-      <c r="W47" s="179"/>
-      <c r="X47" s="179"/>
-      <c r="Y47" s="179"/>
-      <c r="Z47" s="179"/>
-      <c r="AA47" s="179"/>
-      <c r="AB47" s="179"/>
-      <c r="AC47" s="179"/>
-      <c r="AD47" s="179"/>
-      <c r="AE47" s="179"/>
-      <c r="AF47" s="179"/>
-      <c r="AG47" s="179"/>
+      <c r="C47" s="182"/>
+      <c r="D47" s="182"/>
+      <c r="E47" s="182"/>
+      <c r="F47" s="182"/>
+      <c r="G47" s="182"/>
+      <c r="H47" s="182"/>
+      <c r="I47" s="182"/>
+      <c r="J47" s="182"/>
+      <c r="K47" s="182"/>
+      <c r="L47" s="182"/>
+      <c r="M47" s="182"/>
+      <c r="N47" s="182"/>
+      <c r="O47" s="182"/>
+      <c r="P47" s="182"/>
+      <c r="Q47" s="182"/>
+      <c r="R47" s="182"/>
+      <c r="S47" s="182"/>
+      <c r="T47" s="182"/>
+      <c r="U47" s="182"/>
+      <c r="V47" s="182"/>
+      <c r="W47" s="182"/>
+      <c r="X47" s="182"/>
+      <c r="Y47" s="182"/>
+      <c r="Z47" s="182"/>
+      <c r="AA47" s="182"/>
+      <c r="AB47" s="182"/>
+      <c r="AC47" s="182"/>
+      <c r="AD47" s="182"/>
+      <c r="AE47" s="182"/>
+      <c r="AF47" s="182"/>
+      <c r="AG47" s="182"/>
     </row>
     <row r="48" spans="1:268" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B48" s="173" t="s">
+      <c r="B48" s="176" t="s">
         <v>582</v>
       </c>
-      <c r="C48" s="173"/>
-      <c r="D48" s="173"/>
-      <c r="E48" s="173"/>
-      <c r="F48" s="173"/>
-      <c r="G48" s="173"/>
-      <c r="H48" s="173"/>
-      <c r="I48" s="173"/>
-      <c r="J48" s="173"/>
-      <c r="K48" s="173"/>
-      <c r="L48" s="173"/>
-      <c r="M48" s="173"/>
-      <c r="N48" s="173"/>
-      <c r="O48" s="173"/>
-      <c r="P48" s="173"/>
-      <c r="Q48" s="173"/>
-      <c r="R48" s="173" t="s">
+      <c r="C48" s="176"/>
+      <c r="D48" s="176"/>
+      <c r="E48" s="176"/>
+      <c r="F48" s="176"/>
+      <c r="G48" s="176"/>
+      <c r="H48" s="176"/>
+      <c r="I48" s="176"/>
+      <c r="J48" s="176"/>
+      <c r="K48" s="176"/>
+      <c r="L48" s="176"/>
+      <c r="M48" s="176"/>
+      <c r="N48" s="176"/>
+      <c r="O48" s="176"/>
+      <c r="P48" s="176"/>
+      <c r="Q48" s="176"/>
+      <c r="R48" s="176" t="s">
         <v>583</v>
       </c>
-      <c r="S48" s="173"/>
-      <c r="T48" s="173"/>
-      <c r="U48" s="173"/>
-      <c r="V48" s="176" t="s">
+      <c r="S48" s="176"/>
+      <c r="T48" s="176"/>
+      <c r="U48" s="176"/>
+      <c r="V48" s="232" t="s">
         <v>708</v>
       </c>
-      <c r="W48" s="177"/>
-      <c r="X48" s="177"/>
-      <c r="Y48" s="178"/>
-      <c r="Z48" s="176" t="s">
+      <c r="W48" s="233"/>
+      <c r="X48" s="233"/>
+      <c r="Y48" s="234"/>
+      <c r="Z48" s="232" t="s">
         <v>702</v>
       </c>
-      <c r="AA48" s="177"/>
-      <c r="AB48" s="177"/>
-      <c r="AC48" s="178"/>
-      <c r="AD48" s="172" t="s">
+      <c r="AA48" s="233"/>
+      <c r="AB48" s="233"/>
+      <c r="AC48" s="234"/>
+      <c r="AD48" s="183" t="s">
         <v>5</v>
       </c>
-      <c r="AE48" s="172"/>
-      <c r="AF48" s="172"/>
-      <c r="AG48" s="172"/>
+      <c r="AE48" s="183"/>
+      <c r="AF48" s="183"/>
+      <c r="AG48" s="183"/>
     </row>
     <row r="49" spans="2:33" x14ac:dyDescent="0.2">
-      <c r="B49" s="191" t="s">
+      <c r="B49" s="229" t="s">
         <v>704</v>
       </c>
-      <c r="C49" s="192"/>
-      <c r="D49" s="192"/>
-      <c r="E49" s="192"/>
-      <c r="F49" s="192"/>
-      <c r="G49" s="192"/>
-      <c r="H49" s="192"/>
-      <c r="I49" s="192"/>
-      <c r="J49" s="192"/>
-      <c r="K49" s="192"/>
-      <c r="L49" s="192"/>
-      <c r="M49" s="192"/>
-      <c r="N49" s="192"/>
-      <c r="O49" s="192"/>
-      <c r="P49" s="192"/>
-      <c r="Q49" s="192"/>
-      <c r="R49" s="192"/>
-      <c r="S49" s="192"/>
-      <c r="T49" s="192"/>
-      <c r="U49" s="192"/>
-      <c r="V49" s="192"/>
-      <c r="W49" s="192"/>
-      <c r="X49" s="192"/>
-      <c r="Y49" s="192"/>
-      <c r="Z49" s="192"/>
-      <c r="AA49" s="192"/>
-      <c r="AB49" s="192"/>
-      <c r="AC49" s="192"/>
-      <c r="AD49" s="192"/>
-      <c r="AE49" s="192"/>
-      <c r="AF49" s="192"/>
-      <c r="AG49" s="193"/>
+      <c r="C49" s="230"/>
+      <c r="D49" s="230"/>
+      <c r="E49" s="230"/>
+      <c r="F49" s="230"/>
+      <c r="G49" s="230"/>
+      <c r="H49" s="230"/>
+      <c r="I49" s="230"/>
+      <c r="J49" s="230"/>
+      <c r="K49" s="230"/>
+      <c r="L49" s="230"/>
+      <c r="M49" s="230"/>
+      <c r="N49" s="230"/>
+      <c r="O49" s="230"/>
+      <c r="P49" s="230"/>
+      <c r="Q49" s="230"/>
+      <c r="R49" s="230"/>
+      <c r="S49" s="230"/>
+      <c r="T49" s="230"/>
+      <c r="U49" s="230"/>
+      <c r="V49" s="230"/>
+      <c r="W49" s="230"/>
+      <c r="X49" s="230"/>
+      <c r="Y49" s="230"/>
+      <c r="Z49" s="230"/>
+      <c r="AA49" s="230"/>
+      <c r="AB49" s="230"/>
+      <c r="AC49" s="230"/>
+      <c r="AD49" s="230"/>
+      <c r="AE49" s="230"/>
+      <c r="AF49" s="230"/>
+      <c r="AG49" s="231"/>
     </row>
     <row r="50" spans="2:33" x14ac:dyDescent="0.2">
-      <c r="B50" s="182" t="s">
+      <c r="B50" s="220" t="s">
         <v>603</v>
       </c>
-      <c r="C50" s="183"/>
-      <c r="D50" s="183"/>
-      <c r="E50" s="183"/>
-      <c r="F50" s="183"/>
-      <c r="G50" s="183"/>
-      <c r="H50" s="183"/>
-      <c r="I50" s="183"/>
-      <c r="J50" s="183"/>
-      <c r="K50" s="183"/>
-      <c r="L50" s="183"/>
-      <c r="M50" s="183"/>
-      <c r="N50" s="183"/>
-      <c r="O50" s="183"/>
-      <c r="P50" s="183"/>
-      <c r="Q50" s="183"/>
-      <c r="R50" s="183"/>
-      <c r="S50" s="183"/>
-      <c r="T50" s="183"/>
-      <c r="U50" s="183"/>
-      <c r="V50" s="183"/>
-      <c r="W50" s="183"/>
-      <c r="X50" s="183"/>
-      <c r="Y50" s="183"/>
-      <c r="Z50" s="183"/>
-      <c r="AA50" s="183"/>
-      <c r="AB50" s="183"/>
-      <c r="AC50" s="183"/>
-      <c r="AD50" s="183"/>
-      <c r="AE50" s="183"/>
-      <c r="AF50" s="183"/>
-      <c r="AG50" s="184"/>
+      <c r="C50" s="221"/>
+      <c r="D50" s="221"/>
+      <c r="E50" s="221"/>
+      <c r="F50" s="221"/>
+      <c r="G50" s="221"/>
+      <c r="H50" s="221"/>
+      <c r="I50" s="221"/>
+      <c r="J50" s="221"/>
+      <c r="K50" s="221"/>
+      <c r="L50" s="221"/>
+      <c r="M50" s="221"/>
+      <c r="N50" s="221"/>
+      <c r="O50" s="221"/>
+      <c r="P50" s="221"/>
+      <c r="Q50" s="221"/>
+      <c r="R50" s="221"/>
+      <c r="S50" s="221"/>
+      <c r="T50" s="221"/>
+      <c r="U50" s="221"/>
+      <c r="V50" s="221"/>
+      <c r="W50" s="221"/>
+      <c r="X50" s="221"/>
+      <c r="Y50" s="221"/>
+      <c r="Z50" s="221"/>
+      <c r="AA50" s="221"/>
+      <c r="AB50" s="221"/>
+      <c r="AC50" s="221"/>
+      <c r="AD50" s="221"/>
+      <c r="AE50" s="221"/>
+      <c r="AF50" s="221"/>
+      <c r="AG50" s="222"/>
     </row>
     <row r="51" spans="2:33" x14ac:dyDescent="0.2">
-      <c r="B51" s="185"/>
-      <c r="C51" s="186"/>
-      <c r="D51" s="186"/>
-      <c r="E51" s="186"/>
-      <c r="F51" s="186"/>
-      <c r="G51" s="186"/>
-      <c r="H51" s="186"/>
-      <c r="I51" s="186"/>
-      <c r="J51" s="186"/>
-      <c r="K51" s="186"/>
-      <c r="L51" s="186"/>
-      <c r="M51" s="186"/>
-      <c r="N51" s="186"/>
-      <c r="O51" s="186"/>
-      <c r="P51" s="186"/>
-      <c r="Q51" s="186"/>
-      <c r="R51" s="186"/>
-      <c r="S51" s="186"/>
-      <c r="T51" s="186"/>
-      <c r="U51" s="186"/>
-      <c r="V51" s="186"/>
-      <c r="W51" s="186"/>
-      <c r="X51" s="186"/>
-      <c r="Y51" s="186"/>
-      <c r="Z51" s="186"/>
-      <c r="AA51" s="186"/>
-      <c r="AB51" s="186"/>
-      <c r="AC51" s="186"/>
-      <c r="AD51" s="186"/>
-      <c r="AE51" s="186"/>
-      <c r="AF51" s="186"/>
-      <c r="AG51" s="187"/>
+      <c r="B51" s="223"/>
+      <c r="C51" s="224"/>
+      <c r="D51" s="224"/>
+      <c r="E51" s="224"/>
+      <c r="F51" s="224"/>
+      <c r="G51" s="224"/>
+      <c r="H51" s="224"/>
+      <c r="I51" s="224"/>
+      <c r="J51" s="224"/>
+      <c r="K51" s="224"/>
+      <c r="L51" s="224"/>
+      <c r="M51" s="224"/>
+      <c r="N51" s="224"/>
+      <c r="O51" s="224"/>
+      <c r="P51" s="224"/>
+      <c r="Q51" s="224"/>
+      <c r="R51" s="224"/>
+      <c r="S51" s="224"/>
+      <c r="T51" s="224"/>
+      <c r="U51" s="224"/>
+      <c r="V51" s="224"/>
+      <c r="W51" s="224"/>
+      <c r="X51" s="224"/>
+      <c r="Y51" s="224"/>
+      <c r="Z51" s="224"/>
+      <c r="AA51" s="224"/>
+      <c r="AB51" s="224"/>
+      <c r="AC51" s="224"/>
+      <c r="AD51" s="224"/>
+      <c r="AE51" s="224"/>
+      <c r="AF51" s="224"/>
+      <c r="AG51" s="225"/>
     </row>
     <row r="52" spans="2:33" x14ac:dyDescent="0.2">
-      <c r="B52" s="188"/>
-      <c r="C52" s="189"/>
-      <c r="D52" s="189"/>
-      <c r="E52" s="189"/>
-      <c r="F52" s="189"/>
-      <c r="G52" s="189"/>
-      <c r="H52" s="189"/>
-      <c r="I52" s="189"/>
-      <c r="J52" s="189"/>
-      <c r="K52" s="189"/>
-      <c r="L52" s="189"/>
-      <c r="M52" s="189"/>
-      <c r="N52" s="189"/>
-      <c r="O52" s="189"/>
-      <c r="P52" s="189"/>
-      <c r="Q52" s="189"/>
-      <c r="R52" s="189"/>
-      <c r="S52" s="189"/>
-      <c r="T52" s="189"/>
-      <c r="U52" s="189"/>
-      <c r="V52" s="189"/>
-      <c r="W52" s="189"/>
-      <c r="X52" s="189"/>
-      <c r="Y52" s="189"/>
-      <c r="Z52" s="189"/>
-      <c r="AA52" s="189"/>
-      <c r="AB52" s="189"/>
-      <c r="AC52" s="189"/>
-      <c r="AD52" s="189"/>
-      <c r="AE52" s="189"/>
-      <c r="AF52" s="189"/>
-      <c r="AG52" s="190"/>
+      <c r="B52" s="226"/>
+      <c r="C52" s="227"/>
+      <c r="D52" s="227"/>
+      <c r="E52" s="227"/>
+      <c r="F52" s="227"/>
+      <c r="G52" s="227"/>
+      <c r="H52" s="227"/>
+      <c r="I52" s="227"/>
+      <c r="J52" s="227"/>
+      <c r="K52" s="227"/>
+      <c r="L52" s="227"/>
+      <c r="M52" s="227"/>
+      <c r="N52" s="227"/>
+      <c r="O52" s="227"/>
+      <c r="P52" s="227"/>
+      <c r="Q52" s="227"/>
+      <c r="R52" s="227"/>
+      <c r="S52" s="227"/>
+      <c r="T52" s="227"/>
+      <c r="U52" s="227"/>
+      <c r="V52" s="227"/>
+      <c r="W52" s="227"/>
+      <c r="X52" s="227"/>
+      <c r="Y52" s="227"/>
+      <c r="Z52" s="227"/>
+      <c r="AA52" s="227"/>
+      <c r="AB52" s="227"/>
+      <c r="AC52" s="227"/>
+      <c r="AD52" s="227"/>
+      <c r="AE52" s="227"/>
+      <c r="AF52" s="227"/>
+      <c r="AG52" s="228"/>
     </row>
     <row r="53" spans="2:33" x14ac:dyDescent="0.2">
-      <c r="B53" s="198" t="s">
+      <c r="B53" s="180" t="s">
         <v>703</v>
       </c>
-      <c r="C53" s="198"/>
-      <c r="D53" s="198"/>
-      <c r="E53" s="198"/>
-      <c r="F53" s="198"/>
-      <c r="G53" s="198"/>
-      <c r="H53" s="198"/>
-      <c r="I53" s="198"/>
-      <c r="J53" s="198"/>
-      <c r="K53" s="198"/>
-      <c r="L53" s="198"/>
-      <c r="M53" s="198"/>
-      <c r="N53" s="198"/>
-      <c r="O53" s="198"/>
-      <c r="P53" s="198"/>
-      <c r="Q53" s="198"/>
-      <c r="R53" s="198"/>
-      <c r="S53" s="198"/>
-      <c r="T53" s="198"/>
-      <c r="U53" s="198"/>
-      <c r="V53" s="198"/>
-      <c r="W53" s="198"/>
-      <c r="X53" s="198"/>
-      <c r="Y53" s="198"/>
-      <c r="Z53" s="198"/>
-      <c r="AA53" s="198"/>
-      <c r="AB53" s="198"/>
-      <c r="AC53" s="198"/>
-      <c r="AD53" s="198"/>
-      <c r="AE53" s="198"/>
-      <c r="AF53" s="198"/>
-      <c r="AG53" s="198"/>
+      <c r="C53" s="180"/>
+      <c r="D53" s="180"/>
+      <c r="E53" s="180"/>
+      <c r="F53" s="180"/>
+      <c r="G53" s="180"/>
+      <c r="H53" s="180"/>
+      <c r="I53" s="180"/>
+      <c r="J53" s="180"/>
+      <c r="K53" s="180"/>
+      <c r="L53" s="180"/>
+      <c r="M53" s="180"/>
+      <c r="N53" s="180"/>
+      <c r="O53" s="180"/>
+      <c r="P53" s="180"/>
+      <c r="Q53" s="180"/>
+      <c r="R53" s="180"/>
+      <c r="S53" s="180"/>
+      <c r="T53" s="180"/>
+      <c r="U53" s="180"/>
+      <c r="V53" s="180"/>
+      <c r="W53" s="180"/>
+      <c r="X53" s="180"/>
+      <c r="Y53" s="180"/>
+      <c r="Z53" s="180"/>
+      <c r="AA53" s="180"/>
+      <c r="AB53" s="180"/>
+      <c r="AC53" s="180"/>
+      <c r="AD53" s="180"/>
+      <c r="AE53" s="180"/>
+      <c r="AF53" s="180"/>
+      <c r="AG53" s="180"/>
     </row>
     <row r="54" spans="2:33" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B54" s="180" t="s">
+      <c r="B54" s="179" t="s">
         <v>602</v>
       </c>
-      <c r="C54" s="180"/>
-      <c r="D54" s="180"/>
-      <c r="E54" s="180"/>
-      <c r="F54" s="180"/>
-      <c r="G54" s="180"/>
-      <c r="H54" s="180"/>
-      <c r="I54" s="180"/>
-      <c r="J54" s="180"/>
-      <c r="K54" s="180"/>
-      <c r="L54" s="180"/>
-      <c r="M54" s="180"/>
-      <c r="N54" s="180"/>
-      <c r="O54" s="180"/>
-      <c r="P54" s="217"/>
-      <c r="Q54" s="217"/>
-      <c r="R54" s="217"/>
-      <c r="S54" s="217"/>
-      <c r="T54" s="217"/>
-      <c r="U54" s="217"/>
-      <c r="V54" s="217"/>
-      <c r="W54" s="217"/>
-      <c r="X54" s="217"/>
-      <c r="Y54" s="217"/>
-      <c r="Z54" s="217"/>
-      <c r="AA54" s="217"/>
-      <c r="AB54" s="217"/>
-      <c r="AC54" s="217"/>
-      <c r="AD54" s="217"/>
-      <c r="AE54" s="217"/>
-      <c r="AF54" s="217"/>
-      <c r="AG54" s="217"/>
+      <c r="C54" s="179"/>
+      <c r="D54" s="179"/>
+      <c r="E54" s="179"/>
+      <c r="F54" s="179"/>
+      <c r="G54" s="179"/>
+      <c r="H54" s="179"/>
+      <c r="I54" s="179"/>
+      <c r="J54" s="179"/>
+      <c r="K54" s="179"/>
+      <c r="L54" s="179"/>
+      <c r="M54" s="179"/>
+      <c r="N54" s="179"/>
+      <c r="O54" s="179"/>
+      <c r="P54" s="177"/>
+      <c r="Q54" s="177"/>
+      <c r="R54" s="177"/>
+      <c r="S54" s="177"/>
+      <c r="T54" s="177"/>
+      <c r="U54" s="177"/>
+      <c r="V54" s="177"/>
+      <c r="W54" s="177"/>
+      <c r="X54" s="177"/>
+      <c r="Y54" s="177"/>
+      <c r="Z54" s="177"/>
+      <c r="AA54" s="177"/>
+      <c r="AB54" s="177"/>
+      <c r="AC54" s="177"/>
+      <c r="AD54" s="177"/>
+      <c r="AE54" s="177"/>
+      <c r="AF54" s="177"/>
+      <c r="AG54" s="177"/>
     </row>
   </sheetData>
   <mergeCells count="167">
-    <mergeCell ref="B10:AG10"/>
-    <mergeCell ref="U12:X12"/>
-    <mergeCell ref="C12:M12"/>
-    <mergeCell ref="B19:AG19"/>
-    <mergeCell ref="B28:AG28"/>
-    <mergeCell ref="T21:W21"/>
-    <mergeCell ref="X21:AA21"/>
-    <mergeCell ref="U15:X15"/>
-    <mergeCell ref="AB21:AG21"/>
-    <mergeCell ref="X23:AA23"/>
-    <mergeCell ref="X20:AG20"/>
-    <mergeCell ref="C21:K21"/>
-    <mergeCell ref="O12:T12"/>
-    <mergeCell ref="Y12:AG12"/>
-    <mergeCell ref="Y13:AG13"/>
-    <mergeCell ref="C23:K23"/>
-    <mergeCell ref="L22:P22"/>
-    <mergeCell ref="Q22:S22"/>
-    <mergeCell ref="T22:W22"/>
-    <mergeCell ref="C26:AG26"/>
+    <mergeCell ref="AD46:AG46"/>
+    <mergeCell ref="R43:AG43"/>
+    <mergeCell ref="B43:Q43"/>
+    <mergeCell ref="F34:H34"/>
+    <mergeCell ref="AD35:AG35"/>
+    <mergeCell ref="V48:Y48"/>
+    <mergeCell ref="Z48:AC48"/>
+    <mergeCell ref="B48:Q48"/>
+    <mergeCell ref="B47:AG47"/>
+    <mergeCell ref="R48:U48"/>
+    <mergeCell ref="AD48:AG48"/>
+    <mergeCell ref="R46:U46"/>
+    <mergeCell ref="C36:H36"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="B50:AG52"/>
+    <mergeCell ref="B49:AG49"/>
+    <mergeCell ref="V46:Y46"/>
+    <mergeCell ref="Z46:AC46"/>
+    <mergeCell ref="B46:Q46"/>
+    <mergeCell ref="B30:AG30"/>
+    <mergeCell ref="O31:P31"/>
+    <mergeCell ref="O32:P32"/>
+    <mergeCell ref="X36:AC36"/>
+    <mergeCell ref="I36:W36"/>
+    <mergeCell ref="AD36:AG36"/>
+    <mergeCell ref="O34:P34"/>
+    <mergeCell ref="C35:H35"/>
+    <mergeCell ref="I35:L35"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="F31:H31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="F33:H33"/>
+    <mergeCell ref="I31:L31"/>
+    <mergeCell ref="I32:L32"/>
+    <mergeCell ref="I33:L33"/>
+    <mergeCell ref="B44:AG44"/>
+    <mergeCell ref="B45:AG45"/>
+    <mergeCell ref="AD33:AG33"/>
+    <mergeCell ref="V32:X32"/>
+    <mergeCell ref="AD32:AG32"/>
+    <mergeCell ref="AD34:AG34"/>
+    <mergeCell ref="B42:AG42"/>
+    <mergeCell ref="Q23:S23"/>
+    <mergeCell ref="T23:W23"/>
+    <mergeCell ref="C24:AG24"/>
+    <mergeCell ref="B25:AG25"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="M35:P35"/>
+    <mergeCell ref="Q35:U35"/>
+    <mergeCell ref="V35:W35"/>
+    <mergeCell ref="AD31:AG31"/>
+    <mergeCell ref="Q37:U37"/>
+    <mergeCell ref="V37:W37"/>
+    <mergeCell ref="X37:AC37"/>
+    <mergeCell ref="C37:J37"/>
+    <mergeCell ref="K37:L37"/>
+    <mergeCell ref="M37:P37"/>
+    <mergeCell ref="X35:AA35"/>
+    <mergeCell ref="AB35:AC35"/>
+    <mergeCell ref="V33:X33"/>
+    <mergeCell ref="AA31:AC31"/>
+    <mergeCell ref="I29:L29"/>
+    <mergeCell ref="T29:W29"/>
+    <mergeCell ref="X29:AC29"/>
+    <mergeCell ref="AD29:AG29"/>
+    <mergeCell ref="C29:H29"/>
+    <mergeCell ref="P29:S29"/>
+    <mergeCell ref="M29:O29"/>
+    <mergeCell ref="Q27:U27"/>
+    <mergeCell ref="AD27:AG27"/>
+    <mergeCell ref="X27:AC27"/>
+    <mergeCell ref="V27:W27"/>
+    <mergeCell ref="C27:P27"/>
+    <mergeCell ref="M3:O3"/>
+    <mergeCell ref="P3:S3"/>
+    <mergeCell ref="O4:S4"/>
+    <mergeCell ref="B11:AG11"/>
+    <mergeCell ref="Y7:AB7"/>
+    <mergeCell ref="AC7:AG7"/>
+    <mergeCell ref="AE22:AG22"/>
+    <mergeCell ref="C22:K22"/>
+    <mergeCell ref="B6:AG6"/>
+    <mergeCell ref="T4:X4"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="E4:L4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="V3:AB3"/>
+    <mergeCell ref="Y4:AB4"/>
+    <mergeCell ref="C2:AB2"/>
+    <mergeCell ref="F3:L3"/>
+    <mergeCell ref="AC2:AG4"/>
+    <mergeCell ref="T7:X7"/>
+    <mergeCell ref="N7:Q7"/>
+    <mergeCell ref="K7:M7"/>
+    <mergeCell ref="AB22:AD22"/>
+    <mergeCell ref="X22:AA22"/>
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="C8:Q8"/>
+    <mergeCell ref="R8:X8"/>
+    <mergeCell ref="Y8:AG8"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="Y31:Z31"/>
+    <mergeCell ref="Y32:Z32"/>
+    <mergeCell ref="Q34:U34"/>
+    <mergeCell ref="V34:X34"/>
+    <mergeCell ref="Y33:Z33"/>
+    <mergeCell ref="I34:L34"/>
+    <mergeCell ref="Q32:U32"/>
+    <mergeCell ref="V31:X31"/>
+    <mergeCell ref="Q31:U31"/>
+    <mergeCell ref="Q33:U33"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="M33:N33"/>
+    <mergeCell ref="Y34:Z34"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="C13:Q13"/>
+    <mergeCell ref="R13:X13"/>
+    <mergeCell ref="L23:P23"/>
+    <mergeCell ref="AB23:AD23"/>
     <mergeCell ref="AA32:AC32"/>
     <mergeCell ref="AA33:AC33"/>
     <mergeCell ref="AA34:AC34"/>
@@ -13139,129 +13242,26 @@
     <mergeCell ref="R16:X16"/>
     <mergeCell ref="Y16:AG16"/>
     <mergeCell ref="AE23:AG23"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="C8:Q8"/>
-    <mergeCell ref="R8:X8"/>
-    <mergeCell ref="Y8:AG8"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="Y31:Z31"/>
-    <mergeCell ref="Y32:Z32"/>
-    <mergeCell ref="Q34:U34"/>
-    <mergeCell ref="V34:X34"/>
-    <mergeCell ref="Y33:Z33"/>
-    <mergeCell ref="I34:L34"/>
-    <mergeCell ref="Q32:U32"/>
-    <mergeCell ref="V31:X31"/>
-    <mergeCell ref="Q31:U31"/>
-    <mergeCell ref="Q33:U33"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="Y34:Z34"/>
-    <mergeCell ref="O33:P33"/>
-    <mergeCell ref="C13:Q13"/>
-    <mergeCell ref="R13:X13"/>
-    <mergeCell ref="L23:P23"/>
-    <mergeCell ref="AB23:AD23"/>
-    <mergeCell ref="M3:O3"/>
-    <mergeCell ref="P3:S3"/>
-    <mergeCell ref="O4:S4"/>
-    <mergeCell ref="B11:AG11"/>
-    <mergeCell ref="Y7:AB7"/>
-    <mergeCell ref="AC7:AG7"/>
-    <mergeCell ref="AE22:AG22"/>
-    <mergeCell ref="C22:K22"/>
-    <mergeCell ref="B6:AG6"/>
-    <mergeCell ref="T4:X4"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="E4:L4"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="V3:AB3"/>
-    <mergeCell ref="Y4:AB4"/>
-    <mergeCell ref="C2:AB2"/>
-    <mergeCell ref="F3:L3"/>
-    <mergeCell ref="AC2:AG4"/>
-    <mergeCell ref="T7:X7"/>
-    <mergeCell ref="N7:Q7"/>
-    <mergeCell ref="K7:M7"/>
-    <mergeCell ref="AB22:AD22"/>
-    <mergeCell ref="X22:AA22"/>
-    <mergeCell ref="I29:L29"/>
-    <mergeCell ref="T29:W29"/>
-    <mergeCell ref="X29:AC29"/>
-    <mergeCell ref="AD29:AG29"/>
-    <mergeCell ref="C29:H29"/>
-    <mergeCell ref="P29:S29"/>
-    <mergeCell ref="M29:O29"/>
-    <mergeCell ref="Q27:U27"/>
-    <mergeCell ref="AD27:AG27"/>
-    <mergeCell ref="X27:AC27"/>
-    <mergeCell ref="V27:W27"/>
-    <mergeCell ref="C27:P27"/>
-    <mergeCell ref="AD33:AG33"/>
-    <mergeCell ref="V32:X32"/>
-    <mergeCell ref="AD32:AG32"/>
-    <mergeCell ref="AD34:AG34"/>
-    <mergeCell ref="B42:AG42"/>
-    <mergeCell ref="Q23:S23"/>
-    <mergeCell ref="T23:W23"/>
-    <mergeCell ref="C24:AG24"/>
-    <mergeCell ref="B25:AG25"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="M35:P35"/>
-    <mergeCell ref="Q35:U35"/>
-    <mergeCell ref="V35:W35"/>
-    <mergeCell ref="AD31:AG31"/>
-    <mergeCell ref="Q37:U37"/>
-    <mergeCell ref="V37:W37"/>
-    <mergeCell ref="X37:AC37"/>
-    <mergeCell ref="C37:J37"/>
-    <mergeCell ref="K37:L37"/>
-    <mergeCell ref="M37:P37"/>
-    <mergeCell ref="X35:AA35"/>
-    <mergeCell ref="AB35:AC35"/>
-    <mergeCell ref="V33:X33"/>
-    <mergeCell ref="AA31:AC31"/>
-    <mergeCell ref="B50:AG52"/>
-    <mergeCell ref="B49:AG49"/>
-    <mergeCell ref="V46:Y46"/>
-    <mergeCell ref="Z46:AC46"/>
-    <mergeCell ref="B46:Q46"/>
-    <mergeCell ref="B30:AG30"/>
-    <mergeCell ref="O31:P31"/>
-    <mergeCell ref="O32:P32"/>
-    <mergeCell ref="X36:AC36"/>
-    <mergeCell ref="I36:W36"/>
-    <mergeCell ref="AD36:AG36"/>
-    <mergeCell ref="O34:P34"/>
-    <mergeCell ref="C35:H35"/>
-    <mergeCell ref="I35:L35"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="F31:H31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="F33:H33"/>
-    <mergeCell ref="I31:L31"/>
-    <mergeCell ref="I32:L32"/>
-    <mergeCell ref="I33:L33"/>
-    <mergeCell ref="B44:AG44"/>
-    <mergeCell ref="B45:AG45"/>
-    <mergeCell ref="AD46:AG46"/>
-    <mergeCell ref="R43:AG43"/>
-    <mergeCell ref="B43:Q43"/>
-    <mergeCell ref="F34:H34"/>
-    <mergeCell ref="AD35:AG35"/>
-    <mergeCell ref="V48:Y48"/>
-    <mergeCell ref="Z48:AC48"/>
-    <mergeCell ref="B48:Q48"/>
-    <mergeCell ref="B47:AG47"/>
-    <mergeCell ref="R48:U48"/>
-    <mergeCell ref="AD48:AG48"/>
-    <mergeCell ref="R46:U46"/>
-    <mergeCell ref="C36:H36"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="B10:AG10"/>
+    <mergeCell ref="U12:X12"/>
+    <mergeCell ref="C12:M12"/>
+    <mergeCell ref="B19:AG19"/>
+    <mergeCell ref="B28:AG28"/>
+    <mergeCell ref="T21:W21"/>
+    <mergeCell ref="X21:AA21"/>
+    <mergeCell ref="U15:X15"/>
+    <mergeCell ref="AB21:AG21"/>
+    <mergeCell ref="X23:AA23"/>
+    <mergeCell ref="X20:AG20"/>
+    <mergeCell ref="C21:K21"/>
+    <mergeCell ref="O12:T12"/>
+    <mergeCell ref="Y12:AG12"/>
+    <mergeCell ref="Y13:AG13"/>
+    <mergeCell ref="C23:K23"/>
+    <mergeCell ref="L22:P22"/>
+    <mergeCell ref="Q22:S22"/>
+    <mergeCell ref="T22:W22"/>
+    <mergeCell ref="C26:AG26"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -21392,6 +21392,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101001A44C1F890FCF34BA30D378D3367D63B" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="22c88173e6d2a076a971b39a2faa4e23">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="c039d5ce-a415-4a5e-b4fe-9520c78c43c3" xmlns:ns4="fcb16455-6622-4065-81a7-84fea1f9c666" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd62c2bcfd6751c569a4b8d22a7ba344" ns3:_="" ns4:_="">
     <xsd:import namespace="c039d5ce-a415-4a5e-b4fe-9520c78c43c3"/>
@@ -21614,22 +21629,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C2D343A-F610-42B3-83A0-EEB5E4786A2A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="c039d5ce-a415-4a5e-b4fe-9520c78c43c3"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="fcb16455-6622-4065-81a7-84fea1f9c666"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1BA01D47-E7F6-48AD-8D5C-202680BAB15C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F489C8EF-CFF0-4606-955D-42F7AEA2B205}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21646,29 +21671,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1BA01D47-E7F6-48AD-8D5C-202680BAB15C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C2D343A-F610-42B3-83A0-EEB5E4786A2A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="c039d5ce-a415-4a5e-b4fe-9520c78c43c3"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="fcb16455-6622-4065-81a7-84fea1f9c666"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Cambios: Nuevo campo ResponsableMarcobre2 - Acción de investigación de incidentes ambientales
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/Incidentes/Investigacion/JU-MAP-STD-001.F02_Investigación final de incidente ambiental_V00.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/Incidentes/Investigacion/JU-MAP-STD-001.F02_Investigación final de incidente ambiental_V00.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="21929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24527"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\PruebaMerge3y4\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\Incidentes\Investigacion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Rediseño\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\Incidentes\Investigacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB6EA616-C00A-4CE0-A304-CEFF8B0C8526}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AF6BBA8-8E33-43D5-9E10-76DE33FFC68A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IFIA" sheetId="3" r:id="rId1"/>
@@ -20,12 +20,15 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">IFIA!$B$2:$AG$52</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcOnSave="0" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -4890,199 +4893,199 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -5652,40 +5655,40 @@
     <row r="1" spans="1:271" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="1:271" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
-      <c r="B2" s="202"/>
-      <c r="C2" s="205" t="s">
+      <c r="B2" s="224"/>
+      <c r="C2" s="227" t="s">
         <v>604</v>
       </c>
-      <c r="D2" s="206"/>
-      <c r="E2" s="206"/>
-      <c r="F2" s="206"/>
-      <c r="G2" s="206"/>
-      <c r="H2" s="206"/>
-      <c r="I2" s="206"/>
-      <c r="J2" s="206"/>
-      <c r="K2" s="206"/>
-      <c r="L2" s="206"/>
-      <c r="M2" s="206"/>
-      <c r="N2" s="206"/>
-      <c r="O2" s="206"/>
-      <c r="P2" s="206"/>
-      <c r="Q2" s="206"/>
-      <c r="R2" s="206"/>
-      <c r="S2" s="206"/>
-      <c r="T2" s="206"/>
-      <c r="U2" s="206"/>
-      <c r="V2" s="206"/>
-      <c r="W2" s="206"/>
-      <c r="X2" s="206"/>
-      <c r="Y2" s="206"/>
-      <c r="Z2" s="206"/>
-      <c r="AA2" s="206"/>
-      <c r="AB2" s="206"/>
-      <c r="AC2" s="209"/>
-      <c r="AD2" s="209"/>
-      <c r="AE2" s="209"/>
-      <c r="AF2" s="209"/>
-      <c r="AG2" s="209"/>
+      <c r="D2" s="228"/>
+      <c r="E2" s="228"/>
+      <c r="F2" s="228"/>
+      <c r="G2" s="228"/>
+      <c r="H2" s="228"/>
+      <c r="I2" s="228"/>
+      <c r="J2" s="228"/>
+      <c r="K2" s="228"/>
+      <c r="L2" s="228"/>
+      <c r="M2" s="228"/>
+      <c r="N2" s="228"/>
+      <c r="O2" s="228"/>
+      <c r="P2" s="228"/>
+      <c r="Q2" s="228"/>
+      <c r="R2" s="228"/>
+      <c r="S2" s="228"/>
+      <c r="T2" s="228"/>
+      <c r="U2" s="228"/>
+      <c r="V2" s="228"/>
+      <c r="W2" s="228"/>
+      <c r="X2" s="228"/>
+      <c r="Y2" s="228"/>
+      <c r="Z2" s="228"/>
+      <c r="AA2" s="228"/>
+      <c r="AB2" s="228"/>
+      <c r="AC2" s="231"/>
+      <c r="AD2" s="231"/>
+      <c r="AE2" s="231"/>
+      <c r="AF2" s="231"/>
+      <c r="AG2" s="231"/>
       <c r="AH2" s="2"/>
       <c r="AI2" s="2"/>
       <c r="AJ2" s="2"/>
@@ -5923,50 +5926,50 @@
     </row>
     <row r="3" spans="1:271" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
-      <c r="B3" s="202"/>
-      <c r="C3" s="199" t="s">
+      <c r="B3" s="224"/>
+      <c r="C3" s="221" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="200"/>
-      <c r="E3" s="200"/>
-      <c r="F3" s="207" t="s">
+      <c r="D3" s="222"/>
+      <c r="E3" s="222"/>
+      <c r="F3" s="229" t="s">
         <v>607</v>
       </c>
-      <c r="G3" s="207"/>
-      <c r="H3" s="207"/>
-      <c r="I3" s="207"/>
-      <c r="J3" s="207"/>
-      <c r="K3" s="207"/>
-      <c r="L3" s="208"/>
-      <c r="M3" s="188" t="s">
+      <c r="G3" s="229"/>
+      <c r="H3" s="229"/>
+      <c r="I3" s="229"/>
+      <c r="J3" s="229"/>
+      <c r="K3" s="229"/>
+      <c r="L3" s="230"/>
+      <c r="M3" s="210" t="s">
         <v>10</v>
       </c>
-      <c r="N3" s="189"/>
-      <c r="O3" s="189"/>
-      <c r="P3" s="191">
+      <c r="N3" s="211"/>
+      <c r="O3" s="211"/>
+      <c r="P3" s="212">
         <v>43831</v>
       </c>
-      <c r="Q3" s="192"/>
-      <c r="R3" s="192"/>
-      <c r="S3" s="193"/>
+      <c r="Q3" s="213"/>
+      <c r="R3" s="213"/>
+      <c r="S3" s="214"/>
       <c r="T3" s="3" t="s">
         <v>9</v>
       </c>
       <c r="U3" s="37"/>
-      <c r="V3" s="189">
+      <c r="V3" s="211">
         <v>0</v>
       </c>
-      <c r="W3" s="189"/>
-      <c r="X3" s="189"/>
-      <c r="Y3" s="189"/>
-      <c r="Z3" s="189"/>
-      <c r="AA3" s="189"/>
-      <c r="AB3" s="189"/>
-      <c r="AC3" s="209"/>
-      <c r="AD3" s="209"/>
-      <c r="AE3" s="209"/>
-      <c r="AF3" s="209"/>
-      <c r="AG3" s="209"/>
+      <c r="W3" s="211"/>
+      <c r="X3" s="211"/>
+      <c r="Y3" s="211"/>
+      <c r="Z3" s="211"/>
+      <c r="AA3" s="211"/>
+      <c r="AB3" s="211"/>
+      <c r="AC3" s="231"/>
+      <c r="AD3" s="231"/>
+      <c r="AE3" s="231"/>
+      <c r="AF3" s="231"/>
+      <c r="AG3" s="231"/>
       <c r="AI3" s="2"/>
       <c r="AK3" s="2"/>
       <c r="AL3" s="2"/>
@@ -6202,50 +6205,50 @@
     </row>
     <row r="4" spans="1:271" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
-      <c r="B4" s="202"/>
-      <c r="C4" s="199" t="s">
+      <c r="B4" s="224"/>
+      <c r="C4" s="221" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="200"/>
-      <c r="E4" s="200" t="s">
+      <c r="D4" s="222"/>
+      <c r="E4" s="222" t="s">
         <v>376</v>
       </c>
-      <c r="F4" s="200"/>
-      <c r="G4" s="200"/>
-      <c r="H4" s="200"/>
-      <c r="I4" s="200"/>
-      <c r="J4" s="200"/>
-      <c r="K4" s="200"/>
-      <c r="L4" s="201"/>
-      <c r="M4" s="188" t="s">
+      <c r="F4" s="222"/>
+      <c r="G4" s="222"/>
+      <c r="H4" s="222"/>
+      <c r="I4" s="222"/>
+      <c r="J4" s="222"/>
+      <c r="K4" s="222"/>
+      <c r="L4" s="223"/>
+      <c r="M4" s="210" t="s">
         <v>0</v>
       </c>
-      <c r="N4" s="189"/>
-      <c r="O4" s="189">
+      <c r="N4" s="211"/>
+      <c r="O4" s="211">
         <v>1</v>
       </c>
-      <c r="P4" s="189"/>
-      <c r="Q4" s="189"/>
-      <c r="R4" s="189"/>
-      <c r="S4" s="194"/>
-      <c r="T4" s="197" t="s">
+      <c r="P4" s="211"/>
+      <c r="Q4" s="211"/>
+      <c r="R4" s="211"/>
+      <c r="S4" s="215"/>
+      <c r="T4" s="219" t="s">
         <v>11</v>
       </c>
-      <c r="U4" s="198"/>
-      <c r="V4" s="198"/>
-      <c r="W4" s="198"/>
-      <c r="X4" s="198"/>
-      <c r="Y4" s="203">
+      <c r="U4" s="220"/>
+      <c r="V4" s="220"/>
+      <c r="W4" s="220"/>
+      <c r="X4" s="220"/>
+      <c r="Y4" s="225">
         <v>43818</v>
       </c>
-      <c r="Z4" s="204"/>
-      <c r="AA4" s="204"/>
-      <c r="AB4" s="204"/>
-      <c r="AC4" s="209"/>
-      <c r="AD4" s="209"/>
-      <c r="AE4" s="209"/>
-      <c r="AF4" s="209"/>
-      <c r="AG4" s="209"/>
+      <c r="Z4" s="226"/>
+      <c r="AA4" s="226"/>
+      <c r="AB4" s="226"/>
+      <c r="AC4" s="231"/>
+      <c r="AD4" s="231"/>
+      <c r="AE4" s="231"/>
+      <c r="AF4" s="231"/>
+      <c r="AG4" s="231"/>
       <c r="AI4" s="2"/>
       <c r="AK4" s="2"/>
       <c r="AL4" s="2"/>
@@ -6747,40 +6750,40 @@
       <c r="JK5" s="2"/>
     </row>
     <row r="6" spans="1:271" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="196" t="s">
+      <c r="B6" s="218" t="s">
         <v>470</v>
       </c>
-      <c r="C6" s="196"/>
-      <c r="D6" s="196"/>
-      <c r="E6" s="196"/>
-      <c r="F6" s="196"/>
-      <c r="G6" s="196"/>
-      <c r="H6" s="196"/>
-      <c r="I6" s="196"/>
-      <c r="J6" s="196"/>
-      <c r="K6" s="196"/>
-      <c r="L6" s="196"/>
-      <c r="M6" s="196"/>
-      <c r="N6" s="196"/>
-      <c r="O6" s="196"/>
-      <c r="P6" s="196"/>
-      <c r="Q6" s="196"/>
-      <c r="R6" s="196"/>
-      <c r="S6" s="196"/>
-      <c r="T6" s="196"/>
-      <c r="U6" s="196"/>
-      <c r="V6" s="196"/>
-      <c r="W6" s="196"/>
-      <c r="X6" s="196"/>
-      <c r="Y6" s="196"/>
-      <c r="Z6" s="196"/>
-      <c r="AA6" s="196"/>
-      <c r="AB6" s="196"/>
-      <c r="AC6" s="196"/>
-      <c r="AD6" s="196"/>
-      <c r="AE6" s="196"/>
-      <c r="AF6" s="196"/>
-      <c r="AG6" s="196"/>
+      <c r="C6" s="218"/>
+      <c r="D6" s="218"/>
+      <c r="E6" s="218"/>
+      <c r="F6" s="218"/>
+      <c r="G6" s="218"/>
+      <c r="H6" s="218"/>
+      <c r="I6" s="218"/>
+      <c r="J6" s="218"/>
+      <c r="K6" s="218"/>
+      <c r="L6" s="218"/>
+      <c r="M6" s="218"/>
+      <c r="N6" s="218"/>
+      <c r="O6" s="218"/>
+      <c r="P6" s="218"/>
+      <c r="Q6" s="218"/>
+      <c r="R6" s="218"/>
+      <c r="S6" s="218"/>
+      <c r="T6" s="218"/>
+      <c r="U6" s="218"/>
+      <c r="V6" s="218"/>
+      <c r="W6" s="218"/>
+      <c r="X6" s="218"/>
+      <c r="Y6" s="218"/>
+      <c r="Z6" s="218"/>
+      <c r="AA6" s="218"/>
+      <c r="AB6" s="218"/>
+      <c r="AC6" s="218"/>
+      <c r="AD6" s="218"/>
+      <c r="AE6" s="218"/>
+      <c r="AF6" s="218"/>
+      <c r="AG6" s="218"/>
       <c r="AH6" s="2"/>
       <c r="AI6" s="2"/>
       <c r="AK6" s="2"/>
@@ -6789,51 +6792,51 @@
       <c r="B7" s="139" t="s">
         <v>440</v>
       </c>
-      <c r="C7" s="174" t="s">
+      <c r="C7" s="199" t="s">
         <v>609</v>
       </c>
-      <c r="D7" s="174"/>
-      <c r="E7" s="174"/>
-      <c r="F7" s="174"/>
-      <c r="G7" s="174"/>
-      <c r="H7" s="174"/>
-      <c r="I7" s="174"/>
-      <c r="J7" s="174"/>
-      <c r="K7" s="183" t="s">
+      <c r="D7" s="199"/>
+      <c r="E7" s="199"/>
+      <c r="F7" s="199"/>
+      <c r="G7" s="199"/>
+      <c r="H7" s="199"/>
+      <c r="I7" s="199"/>
+      <c r="J7" s="199"/>
+      <c r="K7" s="172" t="s">
         <v>443</v>
       </c>
-      <c r="L7" s="183"/>
-      <c r="M7" s="183"/>
-      <c r="N7" s="177" t="s">
+      <c r="L7" s="172"/>
+      <c r="M7" s="172"/>
+      <c r="N7" s="217" t="s">
         <v>384</v>
       </c>
-      <c r="O7" s="177"/>
-      <c r="P7" s="177"/>
-      <c r="Q7" s="177"/>
+      <c r="O7" s="217"/>
+      <c r="P7" s="217"/>
+      <c r="Q7" s="217"/>
       <c r="R7" s="139" t="s">
         <v>441</v>
       </c>
       <c r="S7" s="139"/>
-      <c r="T7" s="174">
+      <c r="T7" s="199">
         <v>20508972734</v>
       </c>
-      <c r="U7" s="174"/>
-      <c r="V7" s="174"/>
-      <c r="W7" s="174"/>
-      <c r="X7" s="174"/>
-      <c r="Y7" s="173" t="s">
+      <c r="U7" s="199"/>
+      <c r="V7" s="199"/>
+      <c r="W7" s="199"/>
+      <c r="X7" s="199"/>
+      <c r="Y7" s="216" t="s">
         <v>444</v>
       </c>
-      <c r="Z7" s="173"/>
-      <c r="AA7" s="173"/>
-      <c r="AB7" s="173"/>
-      <c r="AC7" s="174" t="s">
+      <c r="Z7" s="216"/>
+      <c r="AA7" s="216"/>
+      <c r="AB7" s="216"/>
+      <c r="AC7" s="199" t="s">
         <v>608</v>
       </c>
-      <c r="AD7" s="174"/>
-      <c r="AE7" s="174"/>
-      <c r="AF7" s="174"/>
-      <c r="AG7" s="174"/>
+      <c r="AD7" s="199"/>
+      <c r="AE7" s="199"/>
+      <c r="AF7" s="199"/>
+      <c r="AG7" s="199"/>
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
       <c r="AK7" s="2"/>
@@ -6842,41 +6845,41 @@
       <c r="B8" s="150" t="s">
         <v>442</v>
       </c>
-      <c r="C8" s="185" t="s">
+      <c r="C8" s="232" t="s">
         <v>610</v>
       </c>
-      <c r="D8" s="185"/>
-      <c r="E8" s="185"/>
-      <c r="F8" s="185"/>
-      <c r="G8" s="185"/>
-      <c r="H8" s="185"/>
-      <c r="I8" s="185"/>
-      <c r="J8" s="185"/>
-      <c r="K8" s="185"/>
-      <c r="L8" s="185"/>
-      <c r="M8" s="185"/>
-      <c r="N8" s="185"/>
-      <c r="O8" s="185"/>
-      <c r="P8" s="185"/>
-      <c r="Q8" s="185"/>
-      <c r="R8" s="187" t="s">
+      <c r="D8" s="232"/>
+      <c r="E8" s="232"/>
+      <c r="F8" s="232"/>
+      <c r="G8" s="232"/>
+      <c r="H8" s="232"/>
+      <c r="I8" s="232"/>
+      <c r="J8" s="232"/>
+      <c r="K8" s="232"/>
+      <c r="L8" s="232"/>
+      <c r="M8" s="232"/>
+      <c r="N8" s="232"/>
+      <c r="O8" s="232"/>
+      <c r="P8" s="232"/>
+      <c r="Q8" s="232"/>
+      <c r="R8" s="202" t="s">
         <v>611</v>
       </c>
-      <c r="S8" s="187"/>
-      <c r="T8" s="187"/>
-      <c r="U8" s="187"/>
-      <c r="V8" s="187"/>
-      <c r="W8" s="187"/>
-      <c r="X8" s="187"/>
-      <c r="Y8" s="185"/>
-      <c r="Z8" s="185"/>
-      <c r="AA8" s="185"/>
-      <c r="AB8" s="185"/>
-      <c r="AC8" s="185"/>
-      <c r="AD8" s="185"/>
-      <c r="AE8" s="185"/>
-      <c r="AF8" s="185"/>
-      <c r="AG8" s="185"/>
+      <c r="S8" s="202"/>
+      <c r="T8" s="202"/>
+      <c r="U8" s="202"/>
+      <c r="V8" s="202"/>
+      <c r="W8" s="202"/>
+      <c r="X8" s="202"/>
+      <c r="Y8" s="232"/>
+      <c r="Z8" s="232"/>
+      <c r="AA8" s="232"/>
+      <c r="AB8" s="232"/>
+      <c r="AC8" s="232"/>
+      <c r="AD8" s="232"/>
+      <c r="AE8" s="232"/>
+      <c r="AF8" s="232"/>
+      <c r="AG8" s="232"/>
       <c r="AH8" s="2"/>
       <c r="AI8" s="2"/>
       <c r="AK8" s="2"/>
@@ -7150,79 +7153,79 @@
       <c r="JK9" s="2"/>
     </row>
     <row r="10" spans="1:271" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="172" t="s">
+      <c r="B10" s="236" t="s">
         <v>471</v>
       </c>
-      <c r="C10" s="172"/>
-      <c r="D10" s="172"/>
-      <c r="E10" s="172"/>
-      <c r="F10" s="172"/>
-      <c r="G10" s="172"/>
-      <c r="H10" s="172"/>
-      <c r="I10" s="172"/>
-      <c r="J10" s="172"/>
-      <c r="K10" s="172"/>
-      <c r="L10" s="172"/>
-      <c r="M10" s="172"/>
-      <c r="N10" s="172"/>
-      <c r="O10" s="172"/>
-      <c r="P10" s="172"/>
-      <c r="Q10" s="172"/>
-      <c r="R10" s="172"/>
-      <c r="S10" s="172"/>
-      <c r="T10" s="172"/>
-      <c r="U10" s="172"/>
-      <c r="V10" s="172"/>
-      <c r="W10" s="172"/>
-      <c r="X10" s="172"/>
-      <c r="Y10" s="172"/>
-      <c r="Z10" s="172"/>
-      <c r="AA10" s="172"/>
-      <c r="AB10" s="172"/>
-      <c r="AC10" s="172"/>
-      <c r="AD10" s="172"/>
-      <c r="AE10" s="172"/>
-      <c r="AF10" s="172"/>
-      <c r="AG10" s="172"/>
+      <c r="C10" s="236"/>
+      <c r="D10" s="236"/>
+      <c r="E10" s="236"/>
+      <c r="F10" s="236"/>
+      <c r="G10" s="236"/>
+      <c r="H10" s="236"/>
+      <c r="I10" s="236"/>
+      <c r="J10" s="236"/>
+      <c r="K10" s="236"/>
+      <c r="L10" s="236"/>
+      <c r="M10" s="236"/>
+      <c r="N10" s="236"/>
+      <c r="O10" s="236"/>
+      <c r="P10" s="236"/>
+      <c r="Q10" s="236"/>
+      <c r="R10" s="236"/>
+      <c r="S10" s="236"/>
+      <c r="T10" s="236"/>
+      <c r="U10" s="236"/>
+      <c r="V10" s="236"/>
+      <c r="W10" s="236"/>
+      <c r="X10" s="236"/>
+      <c r="Y10" s="236"/>
+      <c r="Z10" s="236"/>
+      <c r="AA10" s="236"/>
+      <c r="AB10" s="236"/>
+      <c r="AC10" s="236"/>
+      <c r="AD10" s="236"/>
+      <c r="AE10" s="236"/>
+      <c r="AF10" s="236"/>
+      <c r="AG10" s="236"/>
       <c r="AH10" s="2"/>
       <c r="AI10" s="2"/>
       <c r="AK10" s="2"/>
     </row>
     <row r="11" spans="1:271" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="175" t="s">
+      <c r="B11" s="194" t="s">
         <v>612</v>
       </c>
-      <c r="C11" s="175"/>
-      <c r="D11" s="175"/>
-      <c r="E11" s="175"/>
-      <c r="F11" s="175"/>
-      <c r="G11" s="175"/>
-      <c r="H11" s="175"/>
-      <c r="I11" s="175"/>
-      <c r="J11" s="175"/>
-      <c r="K11" s="175"/>
-      <c r="L11" s="175"/>
-      <c r="M11" s="175"/>
-      <c r="N11" s="175"/>
-      <c r="O11" s="175"/>
-      <c r="P11" s="175"/>
-      <c r="Q11" s="175"/>
-      <c r="R11" s="175"/>
-      <c r="S11" s="175"/>
-      <c r="T11" s="175"/>
-      <c r="U11" s="175"/>
-      <c r="V11" s="175"/>
-      <c r="W11" s="175"/>
-      <c r="X11" s="175"/>
-      <c r="Y11" s="175"/>
-      <c r="Z11" s="175"/>
-      <c r="AA11" s="175"/>
-      <c r="AB11" s="175"/>
-      <c r="AC11" s="175"/>
-      <c r="AD11" s="175"/>
-      <c r="AE11" s="175"/>
-      <c r="AF11" s="175"/>
-      <c r="AG11" s="175"/>
+      <c r="C11" s="194"/>
+      <c r="D11" s="194"/>
+      <c r="E11" s="194"/>
+      <c r="F11" s="194"/>
+      <c r="G11" s="194"/>
+      <c r="H11" s="194"/>
+      <c r="I11" s="194"/>
+      <c r="J11" s="194"/>
+      <c r="K11" s="194"/>
+      <c r="L11" s="194"/>
+      <c r="M11" s="194"/>
+      <c r="N11" s="194"/>
+      <c r="O11" s="194"/>
+      <c r="P11" s="194"/>
+      <c r="Q11" s="194"/>
+      <c r="R11" s="194"/>
+      <c r="S11" s="194"/>
+      <c r="T11" s="194"/>
+      <c r="U11" s="194"/>
+      <c r="V11" s="194"/>
+      <c r="W11" s="194"/>
+      <c r="X11" s="194"/>
+      <c r="Y11" s="194"/>
+      <c r="Z11" s="194"/>
+      <c r="AA11" s="194"/>
+      <c r="AB11" s="194"/>
+      <c r="AC11" s="194"/>
+      <c r="AD11" s="194"/>
+      <c r="AE11" s="194"/>
+      <c r="AF11" s="194"/>
+      <c r="AG11" s="194"/>
       <c r="AH11" s="2"/>
       <c r="AI11" s="2"/>
       <c r="AK11" s="2"/>
@@ -7231,118 +7234,118 @@
       <c r="B12" s="139" t="s">
         <v>440</v>
       </c>
-      <c r="C12" s="174"/>
-      <c r="D12" s="174"/>
-      <c r="E12" s="174"/>
-      <c r="F12" s="174"/>
-      <c r="G12" s="174"/>
-      <c r="H12" s="174"/>
-      <c r="I12" s="174"/>
-      <c r="J12" s="174"/>
-      <c r="K12" s="174"/>
-      <c r="L12" s="174"/>
-      <c r="M12" s="174"/>
+      <c r="C12" s="199"/>
+      <c r="D12" s="199"/>
+      <c r="E12" s="199"/>
+      <c r="F12" s="199"/>
+      <c r="G12" s="199"/>
+      <c r="H12" s="199"/>
+      <c r="I12" s="199"/>
+      <c r="J12" s="199"/>
+      <c r="K12" s="199"/>
+      <c r="L12" s="199"/>
+      <c r="M12" s="199"/>
       <c r="N12" s="170" t="s">
         <v>441</v>
       </c>
-      <c r="O12" s="174"/>
-      <c r="P12" s="174"/>
-      <c r="Q12" s="174"/>
-      <c r="R12" s="174"/>
-      <c r="S12" s="174"/>
-      <c r="T12" s="174"/>
-      <c r="U12" s="173" t="s">
+      <c r="O12" s="199"/>
+      <c r="P12" s="199"/>
+      <c r="Q12" s="199"/>
+      <c r="R12" s="199"/>
+      <c r="S12" s="199"/>
+      <c r="T12" s="199"/>
+      <c r="U12" s="216" t="s">
         <v>444</v>
       </c>
-      <c r="V12" s="173"/>
-      <c r="W12" s="173"/>
-      <c r="X12" s="173"/>
-      <c r="Y12" s="174"/>
-      <c r="Z12" s="174"/>
-      <c r="AA12" s="174"/>
-      <c r="AB12" s="174"/>
-      <c r="AC12" s="174"/>
-      <c r="AD12" s="174"/>
-      <c r="AE12" s="174"/>
-      <c r="AF12" s="174"/>
-      <c r="AG12" s="174"/>
+      <c r="V12" s="216"/>
+      <c r="W12" s="216"/>
+      <c r="X12" s="216"/>
+      <c r="Y12" s="199"/>
+      <c r="Z12" s="199"/>
+      <c r="AA12" s="199"/>
+      <c r="AB12" s="199"/>
+      <c r="AC12" s="199"/>
+      <c r="AD12" s="199"/>
+      <c r="AE12" s="199"/>
+      <c r="AF12" s="199"/>
+      <c r="AG12" s="199"/>
     </row>
     <row r="13" spans="1:271" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="138" t="s">
         <v>442</v>
       </c>
-      <c r="C13" s="177"/>
-      <c r="D13" s="177"/>
-      <c r="E13" s="177"/>
-      <c r="F13" s="177"/>
-      <c r="G13" s="177"/>
-      <c r="H13" s="177"/>
-      <c r="I13" s="177"/>
-      <c r="J13" s="177"/>
-      <c r="K13" s="177"/>
-      <c r="L13" s="177"/>
-      <c r="M13" s="177"/>
-      <c r="N13" s="177"/>
-      <c r="O13" s="177"/>
-      <c r="P13" s="177"/>
-      <c r="Q13" s="177"/>
-      <c r="R13" s="176" t="s">
+      <c r="C13" s="217"/>
+      <c r="D13" s="217"/>
+      <c r="E13" s="217"/>
+      <c r="F13" s="217"/>
+      <c r="G13" s="217"/>
+      <c r="H13" s="217"/>
+      <c r="I13" s="217"/>
+      <c r="J13" s="217"/>
+      <c r="K13" s="217"/>
+      <c r="L13" s="217"/>
+      <c r="M13" s="217"/>
+      <c r="N13" s="217"/>
+      <c r="O13" s="217"/>
+      <c r="P13" s="217"/>
+      <c r="Q13" s="217"/>
+      <c r="R13" s="173" t="s">
         <v>611</v>
       </c>
-      <c r="S13" s="176"/>
-      <c r="T13" s="176"/>
-      <c r="U13" s="176"/>
-      <c r="V13" s="176"/>
-      <c r="W13" s="176"/>
-      <c r="X13" s="176"/>
-      <c r="Y13" s="177"/>
-      <c r="Z13" s="177"/>
-      <c r="AA13" s="177"/>
-      <c r="AB13" s="177"/>
-      <c r="AC13" s="177"/>
-      <c r="AD13" s="177"/>
-      <c r="AE13" s="177"/>
-      <c r="AF13" s="177"/>
-      <c r="AG13" s="177"/>
+      <c r="S13" s="173"/>
+      <c r="T13" s="173"/>
+      <c r="U13" s="173"/>
+      <c r="V13" s="173"/>
+      <c r="W13" s="173"/>
+      <c r="X13" s="173"/>
+      <c r="Y13" s="217"/>
+      <c r="Z13" s="217"/>
+      <c r="AA13" s="217"/>
+      <c r="AB13" s="217"/>
+      <c r="AC13" s="217"/>
+      <c r="AD13" s="217"/>
+      <c r="AE13" s="217"/>
+      <c r="AF13" s="217"/>
+      <c r="AG13" s="217"/>
       <c r="AH13" s="2"/>
       <c r="AI13" s="2"/>
       <c r="AK13" s="2"/>
     </row>
     <row r="14" spans="1:271" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="175" t="s">
+      <c r="B14" s="194" t="s">
         <v>472</v>
       </c>
-      <c r="C14" s="175"/>
-      <c r="D14" s="175"/>
-      <c r="E14" s="175"/>
-      <c r="F14" s="175"/>
-      <c r="G14" s="175"/>
-      <c r="H14" s="175"/>
-      <c r="I14" s="175"/>
-      <c r="J14" s="175"/>
-      <c r="K14" s="175"/>
-      <c r="L14" s="175"/>
-      <c r="M14" s="175"/>
-      <c r="N14" s="175"/>
-      <c r="O14" s="175"/>
-      <c r="P14" s="175"/>
-      <c r="Q14" s="175"/>
-      <c r="R14" s="175"/>
-      <c r="S14" s="175"/>
-      <c r="T14" s="175"/>
-      <c r="U14" s="175"/>
-      <c r="V14" s="175"/>
-      <c r="W14" s="175"/>
-      <c r="X14" s="175"/>
-      <c r="Y14" s="175"/>
-      <c r="Z14" s="175"/>
-      <c r="AA14" s="175"/>
-      <c r="AB14" s="175"/>
-      <c r="AC14" s="175"/>
-      <c r="AD14" s="175"/>
-      <c r="AE14" s="175"/>
-      <c r="AF14" s="175"/>
-      <c r="AG14" s="175"/>
+      <c r="C14" s="194"/>
+      <c r="D14" s="194"/>
+      <c r="E14" s="194"/>
+      <c r="F14" s="194"/>
+      <c r="G14" s="194"/>
+      <c r="H14" s="194"/>
+      <c r="I14" s="194"/>
+      <c r="J14" s="194"/>
+      <c r="K14" s="194"/>
+      <c r="L14" s="194"/>
+      <c r="M14" s="194"/>
+      <c r="N14" s="194"/>
+      <c r="O14" s="194"/>
+      <c r="P14" s="194"/>
+      <c r="Q14" s="194"/>
+      <c r="R14" s="194"/>
+      <c r="S14" s="194"/>
+      <c r="T14" s="194"/>
+      <c r="U14" s="194"/>
+      <c r="V14" s="194"/>
+      <c r="W14" s="194"/>
+      <c r="X14" s="194"/>
+      <c r="Y14" s="194"/>
+      <c r="Z14" s="194"/>
+      <c r="AA14" s="194"/>
+      <c r="AB14" s="194"/>
+      <c r="AC14" s="194"/>
+      <c r="AD14" s="194"/>
+      <c r="AE14" s="194"/>
+      <c r="AF14" s="194"/>
+      <c r="AG14" s="194"/>
       <c r="AH14" s="2"/>
       <c r="AI14" s="2"/>
       <c r="AK14" s="2"/>
@@ -7351,79 +7354,79 @@
       <c r="B15" s="139" t="s">
         <v>440</v>
       </c>
-      <c r="C15" s="174"/>
-      <c r="D15" s="174"/>
-      <c r="E15" s="174"/>
-      <c r="F15" s="174"/>
-      <c r="G15" s="174"/>
-      <c r="H15" s="174"/>
-      <c r="I15" s="174"/>
-      <c r="J15" s="174"/>
-      <c r="K15" s="174"/>
-      <c r="L15" s="174"/>
-      <c r="M15" s="174"/>
+      <c r="C15" s="199"/>
+      <c r="D15" s="199"/>
+      <c r="E15" s="199"/>
+      <c r="F15" s="199"/>
+      <c r="G15" s="199"/>
+      <c r="H15" s="199"/>
+      <c r="I15" s="199"/>
+      <c r="J15" s="199"/>
+      <c r="K15" s="199"/>
+      <c r="L15" s="199"/>
+      <c r="M15" s="199"/>
       <c r="N15" s="170" t="s">
         <v>441</v>
       </c>
-      <c r="O15" s="174"/>
-      <c r="P15" s="174"/>
-      <c r="Q15" s="174"/>
-      <c r="R15" s="174"/>
-      <c r="S15" s="174"/>
-      <c r="T15" s="174"/>
-      <c r="U15" s="173" t="s">
+      <c r="O15" s="199"/>
+      <c r="P15" s="199"/>
+      <c r="Q15" s="199"/>
+      <c r="R15" s="199"/>
+      <c r="S15" s="199"/>
+      <c r="T15" s="199"/>
+      <c r="U15" s="216" t="s">
         <v>444</v>
       </c>
-      <c r="V15" s="173"/>
-      <c r="W15" s="173"/>
-      <c r="X15" s="173"/>
-      <c r="Y15" s="174"/>
-      <c r="Z15" s="174"/>
-      <c r="AA15" s="174"/>
-      <c r="AB15" s="174"/>
-      <c r="AC15" s="174"/>
-      <c r="AD15" s="174"/>
-      <c r="AE15" s="174"/>
-      <c r="AF15" s="174"/>
-      <c r="AG15" s="174"/>
+      <c r="V15" s="216"/>
+      <c r="W15" s="216"/>
+      <c r="X15" s="216"/>
+      <c r="Y15" s="199"/>
+      <c r="Z15" s="199"/>
+      <c r="AA15" s="199"/>
+      <c r="AB15" s="199"/>
+      <c r="AC15" s="199"/>
+      <c r="AD15" s="199"/>
+      <c r="AE15" s="199"/>
+      <c r="AF15" s="199"/>
+      <c r="AG15" s="199"/>
     </row>
     <row r="16" spans="1:271" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="150" t="s">
         <v>442</v>
       </c>
-      <c r="C16" s="185"/>
-      <c r="D16" s="185"/>
-      <c r="E16" s="185"/>
-      <c r="F16" s="185"/>
-      <c r="G16" s="185"/>
-      <c r="H16" s="185"/>
-      <c r="I16" s="185"/>
-      <c r="J16" s="185"/>
-      <c r="K16" s="185"/>
-      <c r="L16" s="185"/>
-      <c r="M16" s="185"/>
-      <c r="N16" s="185"/>
-      <c r="O16" s="185"/>
-      <c r="P16" s="185"/>
-      <c r="Q16" s="185"/>
-      <c r="R16" s="187" t="s">
+      <c r="C16" s="232"/>
+      <c r="D16" s="232"/>
+      <c r="E16" s="232"/>
+      <c r="F16" s="232"/>
+      <c r="G16" s="232"/>
+      <c r="H16" s="232"/>
+      <c r="I16" s="232"/>
+      <c r="J16" s="232"/>
+      <c r="K16" s="232"/>
+      <c r="L16" s="232"/>
+      <c r="M16" s="232"/>
+      <c r="N16" s="232"/>
+      <c r="O16" s="232"/>
+      <c r="P16" s="232"/>
+      <c r="Q16" s="232"/>
+      <c r="R16" s="202" t="s">
         <v>611</v>
       </c>
-      <c r="S16" s="187"/>
-      <c r="T16" s="187"/>
-      <c r="U16" s="187"/>
-      <c r="V16" s="187"/>
-      <c r="W16" s="187"/>
-      <c r="X16" s="187"/>
-      <c r="Y16" s="185"/>
-      <c r="Z16" s="185"/>
-      <c r="AA16" s="185"/>
-      <c r="AB16" s="185"/>
-      <c r="AC16" s="185"/>
-      <c r="AD16" s="185"/>
-      <c r="AE16" s="185"/>
-      <c r="AF16" s="185"/>
-      <c r="AG16" s="185"/>
+      <c r="S16" s="202"/>
+      <c r="T16" s="202"/>
+      <c r="U16" s="202"/>
+      <c r="V16" s="202"/>
+      <c r="W16" s="202"/>
+      <c r="X16" s="202"/>
+      <c r="Y16" s="232"/>
+      <c r="Z16" s="232"/>
+      <c r="AA16" s="232"/>
+      <c r="AB16" s="232"/>
+      <c r="AC16" s="232"/>
+      <c r="AD16" s="232"/>
+      <c r="AE16" s="232"/>
+      <c r="AF16" s="232"/>
+      <c r="AG16" s="232"/>
       <c r="AH16" s="2"/>
       <c r="AI16" s="2"/>
       <c r="AK16" s="2"/>
@@ -7466,79 +7469,79 @@
       <c r="AK17" s="2"/>
     </row>
     <row r="18" spans="1:271" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="184" t="s">
+      <c r="B18" s="234" t="s">
         <v>473</v>
       </c>
-      <c r="C18" s="184"/>
-      <c r="D18" s="184"/>
-      <c r="E18" s="184"/>
-      <c r="F18" s="184"/>
-      <c r="G18" s="184"/>
-      <c r="H18" s="184"/>
-      <c r="I18" s="184"/>
-      <c r="J18" s="184"/>
-      <c r="K18" s="184"/>
-      <c r="L18" s="184"/>
-      <c r="M18" s="184"/>
-      <c r="N18" s="184"/>
-      <c r="O18" s="184"/>
-      <c r="P18" s="184"/>
-      <c r="Q18" s="184"/>
-      <c r="R18" s="184"/>
-      <c r="S18" s="184"/>
-      <c r="T18" s="184"/>
-      <c r="U18" s="184"/>
-      <c r="V18" s="184"/>
-      <c r="W18" s="184"/>
-      <c r="X18" s="184"/>
-      <c r="Y18" s="184"/>
-      <c r="Z18" s="184"/>
-      <c r="AA18" s="184"/>
-      <c r="AB18" s="184"/>
-      <c r="AC18" s="184"/>
-      <c r="AD18" s="184"/>
-      <c r="AE18" s="184"/>
-      <c r="AF18" s="184"/>
-      <c r="AG18" s="184"/>
+      <c r="C18" s="234"/>
+      <c r="D18" s="234"/>
+      <c r="E18" s="234"/>
+      <c r="F18" s="234"/>
+      <c r="G18" s="234"/>
+      <c r="H18" s="234"/>
+      <c r="I18" s="234"/>
+      <c r="J18" s="234"/>
+      <c r="K18" s="234"/>
+      <c r="L18" s="234"/>
+      <c r="M18" s="234"/>
+      <c r="N18" s="234"/>
+      <c r="O18" s="234"/>
+      <c r="P18" s="234"/>
+      <c r="Q18" s="234"/>
+      <c r="R18" s="234"/>
+      <c r="S18" s="234"/>
+      <c r="T18" s="234"/>
+      <c r="U18" s="234"/>
+      <c r="V18" s="234"/>
+      <c r="W18" s="234"/>
+      <c r="X18" s="234"/>
+      <c r="Y18" s="234"/>
+      <c r="Z18" s="234"/>
+      <c r="AA18" s="234"/>
+      <c r="AB18" s="234"/>
+      <c r="AC18" s="234"/>
+      <c r="AD18" s="234"/>
+      <c r="AE18" s="234"/>
+      <c r="AF18" s="234"/>
+      <c r="AG18" s="234"/>
       <c r="AH18" s="2"/>
       <c r="AI18" s="2"/>
       <c r="AK18" s="2"/>
     </row>
     <row r="19" spans="1:271" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="175" t="s">
+      <c r="B19" s="194" t="s">
         <v>561</v>
       </c>
-      <c r="C19" s="175"/>
-      <c r="D19" s="175"/>
-      <c r="E19" s="175"/>
-      <c r="F19" s="175"/>
-      <c r="G19" s="175"/>
-      <c r="H19" s="175"/>
-      <c r="I19" s="175"/>
-      <c r="J19" s="175"/>
-      <c r="K19" s="175"/>
-      <c r="L19" s="175"/>
-      <c r="M19" s="175"/>
-      <c r="N19" s="175"/>
-      <c r="O19" s="175"/>
-      <c r="P19" s="175"/>
-      <c r="Q19" s="175"/>
-      <c r="R19" s="175"/>
-      <c r="S19" s="175"/>
-      <c r="T19" s="175"/>
-      <c r="U19" s="175"/>
-      <c r="V19" s="175"/>
-      <c r="W19" s="175"/>
-      <c r="X19" s="175"/>
-      <c r="Y19" s="175"/>
-      <c r="Z19" s="175"/>
-      <c r="AA19" s="175"/>
-      <c r="AB19" s="175"/>
-      <c r="AC19" s="175"/>
-      <c r="AD19" s="175"/>
-      <c r="AE19" s="175"/>
-      <c r="AF19" s="175"/>
-      <c r="AG19" s="175"/>
+      <c r="C19" s="194"/>
+      <c r="D19" s="194"/>
+      <c r="E19" s="194"/>
+      <c r="F19" s="194"/>
+      <c r="G19" s="194"/>
+      <c r="H19" s="194"/>
+      <c r="I19" s="194"/>
+      <c r="J19" s="194"/>
+      <c r="K19" s="194"/>
+      <c r="L19" s="194"/>
+      <c r="M19" s="194"/>
+      <c r="N19" s="194"/>
+      <c r="O19" s="194"/>
+      <c r="P19" s="194"/>
+      <c r="Q19" s="194"/>
+      <c r="R19" s="194"/>
+      <c r="S19" s="194"/>
+      <c r="T19" s="194"/>
+      <c r="U19" s="194"/>
+      <c r="V19" s="194"/>
+      <c r="W19" s="194"/>
+      <c r="X19" s="194"/>
+      <c r="Y19" s="194"/>
+      <c r="Z19" s="194"/>
+      <c r="AA19" s="194"/>
+      <c r="AB19" s="194"/>
+      <c r="AC19" s="194"/>
+      <c r="AD19" s="194"/>
+      <c r="AE19" s="194"/>
+      <c r="AF19" s="194"/>
+      <c r="AG19" s="194"/>
       <c r="AH19" s="2"/>
       <c r="AI19" s="2"/>
       <c r="AK19" s="2"/>
@@ -7548,39 +7551,39 @@
       <c r="B20" s="137" t="s">
         <v>447</v>
       </c>
-      <c r="C20" s="177"/>
-      <c r="D20" s="177"/>
-      <c r="E20" s="177"/>
-      <c r="F20" s="177"/>
-      <c r="G20" s="177"/>
-      <c r="H20" s="177"/>
-      <c r="I20" s="177"/>
-      <c r="J20" s="177"/>
-      <c r="K20" s="177"/>
-      <c r="L20" s="177"/>
-      <c r="M20" s="177"/>
-      <c r="N20" s="177"/>
-      <c r="O20" s="177"/>
-      <c r="P20" s="177"/>
-      <c r="Q20" s="183" t="s">
+      <c r="C20" s="217"/>
+      <c r="D20" s="217"/>
+      <c r="E20" s="217"/>
+      <c r="F20" s="217"/>
+      <c r="G20" s="217"/>
+      <c r="H20" s="217"/>
+      <c r="I20" s="217"/>
+      <c r="J20" s="217"/>
+      <c r="K20" s="217"/>
+      <c r="L20" s="217"/>
+      <c r="M20" s="217"/>
+      <c r="N20" s="217"/>
+      <c r="O20" s="217"/>
+      <c r="P20" s="217"/>
+      <c r="Q20" s="172" t="s">
         <v>448</v>
       </c>
-      <c r="R20" s="183"/>
-      <c r="S20" s="183"/>
-      <c r="T20" s="183"/>
-      <c r="U20" s="183"/>
-      <c r="V20" s="183"/>
-      <c r="W20" s="183"/>
-      <c r="X20" s="177"/>
-      <c r="Y20" s="177"/>
-      <c r="Z20" s="177"/>
-      <c r="AA20" s="177"/>
-      <c r="AB20" s="177"/>
-      <c r="AC20" s="177"/>
-      <c r="AD20" s="177"/>
-      <c r="AE20" s="177"/>
-      <c r="AF20" s="177"/>
-      <c r="AG20" s="177"/>
+      <c r="R20" s="172"/>
+      <c r="S20" s="172"/>
+      <c r="T20" s="172"/>
+      <c r="U20" s="172"/>
+      <c r="V20" s="172"/>
+      <c r="W20" s="172"/>
+      <c r="X20" s="217"/>
+      <c r="Y20" s="217"/>
+      <c r="Z20" s="217"/>
+      <c r="AA20" s="217"/>
+      <c r="AB20" s="217"/>
+      <c r="AC20" s="217"/>
+      <c r="AD20" s="217"/>
+      <c r="AE20" s="217"/>
+      <c r="AF20" s="217"/>
+      <c r="AG20" s="217"/>
       <c r="AH20" s="2"/>
       <c r="AI20" s="2"/>
       <c r="AK20" s="2"/>
@@ -7820,43 +7823,43 @@
       <c r="B21" s="138" t="s">
         <v>450</v>
       </c>
-      <c r="C21" s="177"/>
-      <c r="D21" s="177"/>
-      <c r="E21" s="177"/>
-      <c r="F21" s="177"/>
-      <c r="G21" s="177"/>
-      <c r="H21" s="177"/>
-      <c r="I21" s="177"/>
-      <c r="J21" s="177"/>
-      <c r="K21" s="177"/>
-      <c r="L21" s="186" t="s">
+      <c r="C21" s="217"/>
+      <c r="D21" s="217"/>
+      <c r="E21" s="217"/>
+      <c r="F21" s="217"/>
+      <c r="G21" s="217"/>
+      <c r="H21" s="217"/>
+      <c r="I21" s="217"/>
+      <c r="J21" s="217"/>
+      <c r="K21" s="217"/>
+      <c r="L21" s="235" t="s">
         <v>660</v>
       </c>
-      <c r="M21" s="186"/>
-      <c r="N21" s="186"/>
-      <c r="O21" s="186"/>
-      <c r="P21" s="186"/>
-      <c r="Q21" s="176" t="s">
+      <c r="M21" s="235"/>
+      <c r="N21" s="235"/>
+      <c r="O21" s="235"/>
+      <c r="P21" s="235"/>
+      <c r="Q21" s="173" t="s">
         <v>455</v>
       </c>
-      <c r="R21" s="176"/>
-      <c r="S21" s="176"/>
-      <c r="T21" s="174"/>
-      <c r="U21" s="174"/>
-      <c r="V21" s="174"/>
-      <c r="W21" s="174"/>
-      <c r="X21" s="176" t="s">
+      <c r="R21" s="173"/>
+      <c r="S21" s="173"/>
+      <c r="T21" s="199"/>
+      <c r="U21" s="199"/>
+      <c r="V21" s="199"/>
+      <c r="W21" s="199"/>
+      <c r="X21" s="173" t="s">
         <v>456</v>
       </c>
-      <c r="Y21" s="176"/>
-      <c r="Z21" s="176"/>
-      <c r="AA21" s="176"/>
-      <c r="AB21" s="177"/>
-      <c r="AC21" s="177"/>
-      <c r="AD21" s="177"/>
-      <c r="AE21" s="177"/>
-      <c r="AF21" s="177"/>
-      <c r="AG21" s="177"/>
+      <c r="Y21" s="173"/>
+      <c r="Z21" s="173"/>
+      <c r="AA21" s="173"/>
+      <c r="AB21" s="217"/>
+      <c r="AC21" s="217"/>
+      <c r="AD21" s="217"/>
+      <c r="AE21" s="217"/>
+      <c r="AF21" s="217"/>
+      <c r="AG21" s="217"/>
       <c r="AH21" s="2"/>
       <c r="AI21" s="2"/>
       <c r="AK21" s="2"/>
@@ -8096,43 +8099,43 @@
       <c r="B22" s="139" t="s">
         <v>661</v>
       </c>
-      <c r="C22" s="177"/>
-      <c r="D22" s="177"/>
-      <c r="E22" s="177"/>
-      <c r="F22" s="177"/>
-      <c r="G22" s="177"/>
-      <c r="H22" s="177"/>
-      <c r="I22" s="177"/>
-      <c r="J22" s="177"/>
-      <c r="K22" s="177"/>
-      <c r="L22" s="176" t="s">
+      <c r="C22" s="217"/>
+      <c r="D22" s="217"/>
+      <c r="E22" s="217"/>
+      <c r="F22" s="217"/>
+      <c r="G22" s="217"/>
+      <c r="H22" s="217"/>
+      <c r="I22" s="217"/>
+      <c r="J22" s="217"/>
+      <c r="K22" s="217"/>
+      <c r="L22" s="173" t="s">
         <v>445</v>
       </c>
-      <c r="M22" s="176"/>
-      <c r="N22" s="176"/>
-      <c r="O22" s="176"/>
-      <c r="P22" s="176"/>
-      <c r="Q22" s="177"/>
-      <c r="R22" s="177"/>
-      <c r="S22" s="177"/>
-      <c r="T22" s="176" t="s">
+      <c r="M22" s="173"/>
+      <c r="N22" s="173"/>
+      <c r="O22" s="173"/>
+      <c r="P22" s="173"/>
+      <c r="Q22" s="217"/>
+      <c r="R22" s="217"/>
+      <c r="S22" s="217"/>
+      <c r="T22" s="173" t="s">
         <v>446</v>
       </c>
-      <c r="U22" s="176"/>
-      <c r="V22" s="176"/>
-      <c r="W22" s="176"/>
-      <c r="X22" s="177"/>
-      <c r="Y22" s="177"/>
-      <c r="Z22" s="177"/>
-      <c r="AA22" s="177"/>
-      <c r="AB22" s="176" t="s">
+      <c r="U22" s="173"/>
+      <c r="V22" s="173"/>
+      <c r="W22" s="173"/>
+      <c r="X22" s="217"/>
+      <c r="Y22" s="217"/>
+      <c r="Z22" s="217"/>
+      <c r="AA22" s="217"/>
+      <c r="AB22" s="173" t="s">
         <v>449</v>
       </c>
-      <c r="AC22" s="176"/>
-      <c r="AD22" s="176"/>
-      <c r="AE22" s="195"/>
-      <c r="AF22" s="195"/>
-      <c r="AG22" s="195"/>
+      <c r="AC22" s="173"/>
+      <c r="AD22" s="173"/>
+      <c r="AE22" s="175"/>
+      <c r="AF22" s="175"/>
+      <c r="AG22" s="175"/>
       <c r="AH22" s="2"/>
       <c r="AI22" s="2"/>
       <c r="AK22" s="2"/>
@@ -8372,43 +8375,43 @@
       <c r="B23" s="138" t="s">
         <v>658</v>
       </c>
-      <c r="C23" s="177"/>
-      <c r="D23" s="177"/>
-      <c r="E23" s="177"/>
-      <c r="F23" s="177"/>
-      <c r="G23" s="177"/>
-      <c r="H23" s="177"/>
-      <c r="I23" s="177"/>
-      <c r="J23" s="177"/>
-      <c r="K23" s="177"/>
-      <c r="L23" s="176" t="s">
+      <c r="C23" s="217"/>
+      <c r="D23" s="217"/>
+      <c r="E23" s="217"/>
+      <c r="F23" s="217"/>
+      <c r="G23" s="217"/>
+      <c r="H23" s="217"/>
+      <c r="I23" s="217"/>
+      <c r="J23" s="217"/>
+      <c r="K23" s="217"/>
+      <c r="L23" s="173" t="s">
         <v>659</v>
       </c>
-      <c r="M23" s="176"/>
-      <c r="N23" s="176"/>
-      <c r="O23" s="176"/>
-      <c r="P23" s="176"/>
-      <c r="Q23" s="195"/>
-      <c r="R23" s="195"/>
-      <c r="S23" s="195"/>
-      <c r="T23" s="176" t="s">
+      <c r="M23" s="173"/>
+      <c r="N23" s="173"/>
+      <c r="O23" s="173"/>
+      <c r="P23" s="173"/>
+      <c r="Q23" s="175"/>
+      <c r="R23" s="175"/>
+      <c r="S23" s="175"/>
+      <c r="T23" s="173" t="s">
         <v>657</v>
       </c>
-      <c r="U23" s="176"/>
-      <c r="V23" s="176"/>
-      <c r="W23" s="176"/>
-      <c r="X23" s="174"/>
-      <c r="Y23" s="174"/>
-      <c r="Z23" s="174"/>
-      <c r="AA23" s="174"/>
-      <c r="AB23" s="176" t="s">
+      <c r="U23" s="173"/>
+      <c r="V23" s="173"/>
+      <c r="W23" s="173"/>
+      <c r="X23" s="199"/>
+      <c r="Y23" s="199"/>
+      <c r="Z23" s="199"/>
+      <c r="AA23" s="199"/>
+      <c r="AB23" s="173" t="s">
         <v>665</v>
       </c>
-      <c r="AC23" s="176"/>
-      <c r="AD23" s="176"/>
-      <c r="AE23" s="177"/>
-      <c r="AF23" s="177"/>
-      <c r="AG23" s="177"/>
+      <c r="AC23" s="173"/>
+      <c r="AD23" s="173"/>
+      <c r="AE23" s="217"/>
+      <c r="AF23" s="217"/>
+      <c r="AG23" s="217"/>
       <c r="AH23" s="2"/>
       <c r="AI23" s="2"/>
       <c r="AK23" s="2"/>
@@ -8648,37 +8651,37 @@
       <c r="B24" s="138" t="s">
         <v>463</v>
       </c>
-      <c r="C24" s="195"/>
-      <c r="D24" s="195"/>
-      <c r="E24" s="195"/>
-      <c r="F24" s="195"/>
-      <c r="G24" s="195"/>
-      <c r="H24" s="195"/>
-      <c r="I24" s="195"/>
-      <c r="J24" s="195"/>
-      <c r="K24" s="195"/>
-      <c r="L24" s="195"/>
-      <c r="M24" s="195"/>
-      <c r="N24" s="195"/>
-      <c r="O24" s="195"/>
-      <c r="P24" s="195"/>
-      <c r="Q24" s="195"/>
-      <c r="R24" s="195"/>
-      <c r="S24" s="195"/>
-      <c r="T24" s="195"/>
-      <c r="U24" s="195"/>
-      <c r="V24" s="195"/>
-      <c r="W24" s="195"/>
-      <c r="X24" s="195"/>
-      <c r="Y24" s="195"/>
-      <c r="Z24" s="195"/>
-      <c r="AA24" s="195"/>
-      <c r="AB24" s="195"/>
-      <c r="AC24" s="195"/>
-      <c r="AD24" s="195"/>
-      <c r="AE24" s="195"/>
-      <c r="AF24" s="195"/>
-      <c r="AG24" s="195"/>
+      <c r="C24" s="175"/>
+      <c r="D24" s="175"/>
+      <c r="E24" s="175"/>
+      <c r="F24" s="175"/>
+      <c r="G24" s="175"/>
+      <c r="H24" s="175"/>
+      <c r="I24" s="175"/>
+      <c r="J24" s="175"/>
+      <c r="K24" s="175"/>
+      <c r="L24" s="175"/>
+      <c r="M24" s="175"/>
+      <c r="N24" s="175"/>
+      <c r="O24" s="175"/>
+      <c r="P24" s="175"/>
+      <c r="Q24" s="175"/>
+      <c r="R24" s="175"/>
+      <c r="S24" s="175"/>
+      <c r="T24" s="175"/>
+      <c r="U24" s="175"/>
+      <c r="V24" s="175"/>
+      <c r="W24" s="175"/>
+      <c r="X24" s="175"/>
+      <c r="Y24" s="175"/>
+      <c r="Z24" s="175"/>
+      <c r="AA24" s="175"/>
+      <c r="AB24" s="175"/>
+      <c r="AC24" s="175"/>
+      <c r="AD24" s="175"/>
+      <c r="AE24" s="175"/>
+      <c r="AF24" s="175"/>
+      <c r="AG24" s="175"/>
       <c r="AH24" s="2"/>
       <c r="AI24" s="2"/>
       <c r="AJ24" s="2"/>
@@ -8913,40 +8916,40 @@
     </row>
     <row r="25" spans="1:271" ht="23.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
-      <c r="B25" s="175" t="s">
+      <c r="B25" s="194" t="s">
         <v>691</v>
       </c>
-      <c r="C25" s="175"/>
-      <c r="D25" s="175"/>
-      <c r="E25" s="175"/>
-      <c r="F25" s="175"/>
-      <c r="G25" s="175"/>
-      <c r="H25" s="175"/>
-      <c r="I25" s="175"/>
-      <c r="J25" s="175"/>
-      <c r="K25" s="175"/>
-      <c r="L25" s="175"/>
-      <c r="M25" s="175"/>
-      <c r="N25" s="175"/>
-      <c r="O25" s="175"/>
-      <c r="P25" s="175"/>
-      <c r="Q25" s="175"/>
-      <c r="R25" s="175"/>
-      <c r="S25" s="175"/>
-      <c r="T25" s="175"/>
-      <c r="U25" s="175"/>
-      <c r="V25" s="175"/>
-      <c r="W25" s="175"/>
-      <c r="X25" s="175"/>
-      <c r="Y25" s="175"/>
-      <c r="Z25" s="175"/>
-      <c r="AA25" s="175"/>
-      <c r="AB25" s="175"/>
-      <c r="AC25" s="175"/>
-      <c r="AD25" s="175"/>
-      <c r="AE25" s="175"/>
-      <c r="AF25" s="175"/>
-      <c r="AG25" s="175"/>
+      <c r="C25" s="194"/>
+      <c r="D25" s="194"/>
+      <c r="E25" s="194"/>
+      <c r="F25" s="194"/>
+      <c r="G25" s="194"/>
+      <c r="H25" s="194"/>
+      <c r="I25" s="194"/>
+      <c r="J25" s="194"/>
+      <c r="K25" s="194"/>
+      <c r="L25" s="194"/>
+      <c r="M25" s="194"/>
+      <c r="N25" s="194"/>
+      <c r="O25" s="194"/>
+      <c r="P25" s="194"/>
+      <c r="Q25" s="194"/>
+      <c r="R25" s="194"/>
+      <c r="S25" s="194"/>
+      <c r="T25" s="194"/>
+      <c r="U25" s="194"/>
+      <c r="V25" s="194"/>
+      <c r="W25" s="194"/>
+      <c r="X25" s="194"/>
+      <c r="Y25" s="194"/>
+      <c r="Z25" s="194"/>
+      <c r="AA25" s="194"/>
+      <c r="AB25" s="194"/>
+      <c r="AC25" s="194"/>
+      <c r="AD25" s="194"/>
+      <c r="AE25" s="194"/>
+      <c r="AF25" s="194"/>
+      <c r="AG25" s="194"/>
       <c r="AH25" s="2"/>
       <c r="AI25" s="2"/>
       <c r="AJ25" s="2"/>
@@ -9184,37 +9187,37 @@
       <c r="B26" s="169" t="s">
         <v>662</v>
       </c>
-      <c r="C26" s="174"/>
-      <c r="D26" s="174"/>
-      <c r="E26" s="174"/>
-      <c r="F26" s="174"/>
-      <c r="G26" s="174"/>
-      <c r="H26" s="174"/>
-      <c r="I26" s="174"/>
-      <c r="J26" s="174"/>
-      <c r="K26" s="174"/>
-      <c r="L26" s="174"/>
-      <c r="M26" s="174"/>
-      <c r="N26" s="174"/>
-      <c r="O26" s="174"/>
-      <c r="P26" s="174"/>
-      <c r="Q26" s="174"/>
-      <c r="R26" s="174"/>
-      <c r="S26" s="174"/>
-      <c r="T26" s="174"/>
-      <c r="U26" s="174"/>
-      <c r="V26" s="174"/>
-      <c r="W26" s="174"/>
-      <c r="X26" s="174"/>
-      <c r="Y26" s="174"/>
-      <c r="Z26" s="174"/>
-      <c r="AA26" s="174"/>
-      <c r="AB26" s="174"/>
-      <c r="AC26" s="174"/>
-      <c r="AD26" s="174"/>
-      <c r="AE26" s="174"/>
-      <c r="AF26" s="174"/>
-      <c r="AG26" s="174"/>
+      <c r="C26" s="199"/>
+      <c r="D26" s="199"/>
+      <c r="E26" s="199"/>
+      <c r="F26" s="199"/>
+      <c r="G26" s="199"/>
+      <c r="H26" s="199"/>
+      <c r="I26" s="199"/>
+      <c r="J26" s="199"/>
+      <c r="K26" s="199"/>
+      <c r="L26" s="199"/>
+      <c r="M26" s="199"/>
+      <c r="N26" s="199"/>
+      <c r="O26" s="199"/>
+      <c r="P26" s="199"/>
+      <c r="Q26" s="199"/>
+      <c r="R26" s="199"/>
+      <c r="S26" s="199"/>
+      <c r="T26" s="199"/>
+      <c r="U26" s="199"/>
+      <c r="V26" s="199"/>
+      <c r="W26" s="199"/>
+      <c r="X26" s="199"/>
+      <c r="Y26" s="199"/>
+      <c r="Z26" s="199"/>
+      <c r="AA26" s="199"/>
+      <c r="AB26" s="199"/>
+      <c r="AC26" s="199"/>
+      <c r="AD26" s="199"/>
+      <c r="AE26" s="199"/>
+      <c r="AF26" s="199"/>
+      <c r="AG26" s="199"/>
       <c r="AH26" s="2"/>
       <c r="AI26" s="2"/>
       <c r="AJ26" s="2"/>
@@ -9452,47 +9455,47 @@
       <c r="B27" s="167" t="s">
         <v>709</v>
       </c>
-      <c r="C27" s="213" t="s">
+      <c r="C27" s="209" t="s">
         <v>710</v>
       </c>
-      <c r="D27" s="213"/>
-      <c r="E27" s="213"/>
-      <c r="F27" s="213"/>
-      <c r="G27" s="213"/>
-      <c r="H27" s="213"/>
-      <c r="I27" s="213"/>
-      <c r="J27" s="213"/>
-      <c r="K27" s="213"/>
-      <c r="L27" s="213"/>
-      <c r="M27" s="213"/>
-      <c r="N27" s="213"/>
-      <c r="O27" s="213"/>
-      <c r="P27" s="213"/>
-      <c r="Q27" s="211" t="s">
+      <c r="D27" s="209"/>
+      <c r="E27" s="209"/>
+      <c r="F27" s="209"/>
+      <c r="G27" s="209"/>
+      <c r="H27" s="209"/>
+      <c r="I27" s="209"/>
+      <c r="J27" s="209"/>
+      <c r="K27" s="209"/>
+      <c r="L27" s="209"/>
+      <c r="M27" s="209"/>
+      <c r="N27" s="209"/>
+      <c r="O27" s="209"/>
+      <c r="P27" s="209"/>
+      <c r="Q27" s="207" t="s">
         <v>711</v>
       </c>
-      <c r="R27" s="211"/>
-      <c r="S27" s="211"/>
-      <c r="T27" s="211"/>
-      <c r="U27" s="211"/>
-      <c r="V27" s="211" t="s">
+      <c r="R27" s="207"/>
+      <c r="S27" s="207"/>
+      <c r="T27" s="207"/>
+      <c r="U27" s="207"/>
+      <c r="V27" s="207" t="s">
         <v>663</v>
       </c>
-      <c r="W27" s="211"/>
-      <c r="X27" s="212" t="s">
+      <c r="W27" s="207"/>
+      <c r="X27" s="208" t="s">
         <v>664</v>
       </c>
-      <c r="Y27" s="212"/>
-      <c r="Z27" s="212"/>
-      <c r="AA27" s="212"/>
-      <c r="AB27" s="212"/>
-      <c r="AC27" s="212"/>
-      <c r="AD27" s="176" t="s">
+      <c r="Y27" s="208"/>
+      <c r="Z27" s="208"/>
+      <c r="AA27" s="208"/>
+      <c r="AB27" s="208"/>
+      <c r="AC27" s="208"/>
+      <c r="AD27" s="173" t="s">
         <v>693</v>
       </c>
-      <c r="AE27" s="176"/>
-      <c r="AF27" s="176"/>
-      <c r="AG27" s="176"/>
+      <c r="AE27" s="173"/>
+      <c r="AF27" s="173"/>
+      <c r="AG27" s="173"/>
       <c r="AH27" s="2"/>
       <c r="AI27" s="2"/>
       <c r="AJ27" s="2"/>
@@ -9727,40 +9730,40 @@
     </row>
     <row r="28" spans="1:271" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
-      <c r="B28" s="175" t="s">
+      <c r="B28" s="194" t="s">
         <v>692</v>
       </c>
-      <c r="C28" s="175"/>
-      <c r="D28" s="175"/>
-      <c r="E28" s="175"/>
-      <c r="F28" s="175"/>
-      <c r="G28" s="175"/>
-      <c r="H28" s="175"/>
-      <c r="I28" s="175"/>
-      <c r="J28" s="175"/>
-      <c r="K28" s="175"/>
-      <c r="L28" s="175"/>
-      <c r="M28" s="175"/>
-      <c r="N28" s="175"/>
-      <c r="O28" s="175"/>
-      <c r="P28" s="175"/>
-      <c r="Q28" s="175"/>
-      <c r="R28" s="175"/>
-      <c r="S28" s="175"/>
-      <c r="T28" s="175"/>
-      <c r="U28" s="175"/>
-      <c r="V28" s="175"/>
-      <c r="W28" s="175"/>
-      <c r="X28" s="175"/>
-      <c r="Y28" s="175"/>
-      <c r="Z28" s="175"/>
-      <c r="AA28" s="175"/>
-      <c r="AB28" s="175"/>
-      <c r="AC28" s="175"/>
-      <c r="AD28" s="175"/>
-      <c r="AE28" s="175"/>
-      <c r="AF28" s="175"/>
-      <c r="AG28" s="175"/>
+      <c r="C28" s="194"/>
+      <c r="D28" s="194"/>
+      <c r="E28" s="194"/>
+      <c r="F28" s="194"/>
+      <c r="G28" s="194"/>
+      <c r="H28" s="194"/>
+      <c r="I28" s="194"/>
+      <c r="J28" s="194"/>
+      <c r="K28" s="194"/>
+      <c r="L28" s="194"/>
+      <c r="M28" s="194"/>
+      <c r="N28" s="194"/>
+      <c r="O28" s="194"/>
+      <c r="P28" s="194"/>
+      <c r="Q28" s="194"/>
+      <c r="R28" s="194"/>
+      <c r="S28" s="194"/>
+      <c r="T28" s="194"/>
+      <c r="U28" s="194"/>
+      <c r="V28" s="194"/>
+      <c r="W28" s="194"/>
+      <c r="X28" s="194"/>
+      <c r="Y28" s="194"/>
+      <c r="Z28" s="194"/>
+      <c r="AA28" s="194"/>
+      <c r="AB28" s="194"/>
+      <c r="AC28" s="194"/>
+      <c r="AD28" s="194"/>
+      <c r="AE28" s="194"/>
+      <c r="AF28" s="194"/>
+      <c r="AG28" s="194"/>
       <c r="AH28" s="2"/>
       <c r="AI28" s="2"/>
       <c r="AJ28" s="2"/>
@@ -9998,51 +10001,51 @@
       <c r="B29" s="171" t="s">
         <v>712</v>
       </c>
-      <c r="C29" s="210" t="s">
+      <c r="C29" s="206" t="s">
         <v>474</v>
       </c>
-      <c r="D29" s="210"/>
-      <c r="E29" s="210"/>
-      <c r="F29" s="210"/>
-      <c r="G29" s="210"/>
-      <c r="H29" s="210"/>
-      <c r="I29" s="210" t="s">
+      <c r="D29" s="206"/>
+      <c r="E29" s="206"/>
+      <c r="F29" s="206"/>
+      <c r="G29" s="206"/>
+      <c r="H29" s="206"/>
+      <c r="I29" s="206" t="s">
         <v>713</v>
       </c>
-      <c r="J29" s="210"/>
-      <c r="K29" s="210"/>
-      <c r="L29" s="210"/>
-      <c r="M29" s="210" t="s">
+      <c r="J29" s="206"/>
+      <c r="K29" s="206"/>
+      <c r="L29" s="206"/>
+      <c r="M29" s="206" t="s">
         <v>714</v>
       </c>
-      <c r="N29" s="210"/>
-      <c r="O29" s="210"/>
-      <c r="P29" s="210" t="s">
+      <c r="N29" s="206"/>
+      <c r="O29" s="206"/>
+      <c r="P29" s="206" t="s">
         <v>715</v>
       </c>
-      <c r="Q29" s="210"/>
-      <c r="R29" s="210"/>
-      <c r="S29" s="210"/>
-      <c r="T29" s="210" t="s">
+      <c r="Q29" s="206"/>
+      <c r="R29" s="206"/>
+      <c r="S29" s="206"/>
+      <c r="T29" s="206" t="s">
         <v>697</v>
       </c>
-      <c r="U29" s="210"/>
-      <c r="V29" s="210"/>
-      <c r="W29" s="210"/>
-      <c r="X29" s="210" t="s">
+      <c r="U29" s="206"/>
+      <c r="V29" s="206"/>
+      <c r="W29" s="206"/>
+      <c r="X29" s="206" t="s">
         <v>716</v>
       </c>
-      <c r="Y29" s="210"/>
-      <c r="Z29" s="210"/>
-      <c r="AA29" s="210"/>
-      <c r="AB29" s="210"/>
-      <c r="AC29" s="210"/>
-      <c r="AD29" s="210" t="s">
+      <c r="Y29" s="206"/>
+      <c r="Z29" s="206"/>
+      <c r="AA29" s="206"/>
+      <c r="AB29" s="206"/>
+      <c r="AC29" s="206"/>
+      <c r="AD29" s="206" t="s">
         <v>717</v>
       </c>
-      <c r="AE29" s="210"/>
-      <c r="AF29" s="210"/>
-      <c r="AG29" s="210"/>
+      <c r="AE29" s="206"/>
+      <c r="AF29" s="206"/>
+      <c r="AG29" s="206"/>
       <c r="AH29" s="2"/>
       <c r="AI29" s="2"/>
       <c r="AJ29" s="2"/>
@@ -10277,40 +10280,40 @@
     </row>
     <row r="30" spans="1:271" ht="22.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1"/>
-      <c r="B30" s="175" t="s">
+      <c r="B30" s="194" t="s">
         <v>694</v>
       </c>
-      <c r="C30" s="175"/>
-      <c r="D30" s="175"/>
-      <c r="E30" s="175"/>
-      <c r="F30" s="175"/>
-      <c r="G30" s="175"/>
-      <c r="H30" s="175"/>
-      <c r="I30" s="175"/>
-      <c r="J30" s="175"/>
-      <c r="K30" s="175"/>
-      <c r="L30" s="175"/>
-      <c r="M30" s="175"/>
-      <c r="N30" s="175"/>
-      <c r="O30" s="175"/>
-      <c r="P30" s="175"/>
-      <c r="Q30" s="175"/>
-      <c r="R30" s="175"/>
-      <c r="S30" s="175"/>
-      <c r="T30" s="175"/>
-      <c r="U30" s="175"/>
-      <c r="V30" s="175"/>
-      <c r="W30" s="175"/>
-      <c r="X30" s="175"/>
-      <c r="Y30" s="175"/>
-      <c r="Z30" s="175"/>
-      <c r="AA30" s="175"/>
-      <c r="AB30" s="175"/>
-      <c r="AC30" s="175"/>
-      <c r="AD30" s="175"/>
-      <c r="AE30" s="175"/>
-      <c r="AF30" s="175"/>
-      <c r="AG30" s="175"/>
+      <c r="C30" s="194"/>
+      <c r="D30" s="194"/>
+      <c r="E30" s="194"/>
+      <c r="F30" s="194"/>
+      <c r="G30" s="194"/>
+      <c r="H30" s="194"/>
+      <c r="I30" s="194"/>
+      <c r="J30" s="194"/>
+      <c r="K30" s="194"/>
+      <c r="L30" s="194"/>
+      <c r="M30" s="194"/>
+      <c r="N30" s="194"/>
+      <c r="O30" s="194"/>
+      <c r="P30" s="194"/>
+      <c r="Q30" s="194"/>
+      <c r="R30" s="194"/>
+      <c r="S30" s="194"/>
+      <c r="T30" s="194"/>
+      <c r="U30" s="194"/>
+      <c r="V30" s="194"/>
+      <c r="W30" s="194"/>
+      <c r="X30" s="194"/>
+      <c r="Y30" s="194"/>
+      <c r="Z30" s="194"/>
+      <c r="AA30" s="194"/>
+      <c r="AB30" s="194"/>
+      <c r="AC30" s="194"/>
+      <c r="AD30" s="194"/>
+      <c r="AE30" s="194"/>
+      <c r="AF30" s="194"/>
+      <c r="AG30" s="194"/>
       <c r="AH30" s="2"/>
       <c r="AI30" s="2"/>
       <c r="AJ30" s="2"/>
@@ -10548,45 +10551,45 @@
       <c r="B31" s="168" t="s">
         <v>1</v>
       </c>
-      <c r="C31" s="178" t="s">
+      <c r="C31" s="196" t="s">
         <v>563</v>
       </c>
-      <c r="D31" s="178"/>
-      <c r="E31" s="178"/>
-      <c r="F31" s="214"/>
-      <c r="G31" s="214"/>
-      <c r="H31" s="214"/>
-      <c r="I31" s="179" t="s">
+      <c r="D31" s="196"/>
+      <c r="E31" s="196"/>
+      <c r="F31" s="174"/>
+      <c r="G31" s="174"/>
+      <c r="H31" s="174"/>
+      <c r="I31" s="180" t="s">
         <v>718</v>
       </c>
-      <c r="J31" s="179"/>
-      <c r="K31" s="179"/>
-      <c r="L31" s="179"/>
-      <c r="M31" s="190"/>
-      <c r="N31" s="190"/>
-      <c r="O31" s="190"/>
-      <c r="P31" s="190"/>
-      <c r="Q31" s="179" t="s">
+      <c r="J31" s="180"/>
+      <c r="K31" s="180"/>
+      <c r="L31" s="180"/>
+      <c r="M31" s="181"/>
+      <c r="N31" s="181"/>
+      <c r="O31" s="181"/>
+      <c r="P31" s="181"/>
+      <c r="Q31" s="180" t="s">
         <v>719</v>
       </c>
-      <c r="R31" s="179"/>
-      <c r="S31" s="179"/>
-      <c r="T31" s="179"/>
-      <c r="U31" s="179"/>
-      <c r="V31" s="190"/>
-      <c r="W31" s="190"/>
-      <c r="X31" s="190"/>
-      <c r="Y31" s="177"/>
-      <c r="Z31" s="177"/>
-      <c r="AA31" s="178" t="s">
+      <c r="R31" s="180"/>
+      <c r="S31" s="180"/>
+      <c r="T31" s="180"/>
+      <c r="U31" s="180"/>
+      <c r="V31" s="181"/>
+      <c r="W31" s="181"/>
+      <c r="X31" s="181"/>
+      <c r="Y31" s="217"/>
+      <c r="Z31" s="217"/>
+      <c r="AA31" s="196" t="s">
         <v>565</v>
       </c>
-      <c r="AB31" s="178"/>
-      <c r="AC31" s="178"/>
-      <c r="AD31" s="214"/>
-      <c r="AE31" s="214"/>
-      <c r="AF31" s="214"/>
-      <c r="AG31" s="214"/>
+      <c r="AB31" s="196"/>
+      <c r="AC31" s="196"/>
+      <c r="AD31" s="174"/>
+      <c r="AE31" s="174"/>
+      <c r="AF31" s="174"/>
+      <c r="AG31" s="174"/>
       <c r="AH31" s="2"/>
       <c r="AI31" s="2"/>
       <c r="AJ31" s="2"/>
@@ -10824,45 +10827,45 @@
       <c r="B32" s="168" t="s">
         <v>3</v>
       </c>
-      <c r="C32" s="179" t="s">
+      <c r="C32" s="180" t="s">
         <v>564</v>
       </c>
-      <c r="D32" s="179"/>
-      <c r="E32" s="179"/>
-      <c r="F32" s="214"/>
-      <c r="G32" s="214"/>
-      <c r="H32" s="214"/>
-      <c r="I32" s="236" t="s">
+      <c r="D32" s="180"/>
+      <c r="E32" s="180"/>
+      <c r="F32" s="174"/>
+      <c r="G32" s="174"/>
+      <c r="H32" s="174"/>
+      <c r="I32" s="197" t="s">
         <v>684</v>
       </c>
-      <c r="J32" s="236"/>
-      <c r="K32" s="236"/>
-      <c r="L32" s="236"/>
-      <c r="M32" s="190"/>
-      <c r="N32" s="190"/>
-      <c r="O32" s="190"/>
-      <c r="P32" s="190"/>
-      <c r="Q32" s="179" t="s">
+      <c r="J32" s="197"/>
+      <c r="K32" s="197"/>
+      <c r="L32" s="197"/>
+      <c r="M32" s="181"/>
+      <c r="N32" s="181"/>
+      <c r="O32" s="181"/>
+      <c r="P32" s="181"/>
+      <c r="Q32" s="180" t="s">
         <v>562</v>
       </c>
-      <c r="R32" s="179"/>
-      <c r="S32" s="179"/>
-      <c r="T32" s="179"/>
-      <c r="U32" s="179"/>
-      <c r="V32" s="190"/>
-      <c r="W32" s="190"/>
-      <c r="X32" s="190"/>
-      <c r="Y32" s="177"/>
-      <c r="Z32" s="177"/>
-      <c r="AA32" s="178" t="s">
+      <c r="R32" s="180"/>
+      <c r="S32" s="180"/>
+      <c r="T32" s="180"/>
+      <c r="U32" s="180"/>
+      <c r="V32" s="181"/>
+      <c r="W32" s="181"/>
+      <c r="X32" s="181"/>
+      <c r="Y32" s="217"/>
+      <c r="Z32" s="217"/>
+      <c r="AA32" s="196" t="s">
         <v>565</v>
       </c>
-      <c r="AB32" s="178"/>
-      <c r="AC32" s="178"/>
-      <c r="AD32" s="214"/>
-      <c r="AE32" s="214"/>
-      <c r="AF32" s="214"/>
-      <c r="AG32" s="214"/>
+      <c r="AB32" s="196"/>
+      <c r="AC32" s="196"/>
+      <c r="AD32" s="174"/>
+      <c r="AE32" s="174"/>
+      <c r="AF32" s="174"/>
+      <c r="AG32" s="174"/>
       <c r="AH32" s="2"/>
       <c r="AI32" s="2"/>
       <c r="AJ32" s="2"/>
@@ -11100,45 +11103,45 @@
       <c r="B33" s="168" t="s">
         <v>4</v>
       </c>
-      <c r="C33" s="179" t="s">
+      <c r="C33" s="180" t="s">
         <v>564</v>
       </c>
-      <c r="D33" s="179"/>
-      <c r="E33" s="179"/>
-      <c r="F33" s="214"/>
-      <c r="G33" s="214"/>
-      <c r="H33" s="214"/>
-      <c r="I33" s="179" t="s">
+      <c r="D33" s="180"/>
+      <c r="E33" s="180"/>
+      <c r="F33" s="174"/>
+      <c r="G33" s="174"/>
+      <c r="H33" s="174"/>
+      <c r="I33" s="180" t="s">
         <v>557</v>
       </c>
-      <c r="J33" s="179"/>
-      <c r="K33" s="179"/>
-      <c r="L33" s="179"/>
-      <c r="M33" s="190"/>
-      <c r="N33" s="190"/>
-      <c r="O33" s="190"/>
-      <c r="P33" s="190"/>
-      <c r="Q33" s="179" t="s">
+      <c r="J33" s="180"/>
+      <c r="K33" s="180"/>
+      <c r="L33" s="180"/>
+      <c r="M33" s="181"/>
+      <c r="N33" s="181"/>
+      <c r="O33" s="181"/>
+      <c r="P33" s="181"/>
+      <c r="Q33" s="180" t="s">
         <v>562</v>
       </c>
-      <c r="R33" s="179"/>
-      <c r="S33" s="179"/>
-      <c r="T33" s="179"/>
-      <c r="U33" s="179"/>
-      <c r="V33" s="190"/>
-      <c r="W33" s="190"/>
-      <c r="X33" s="190"/>
-      <c r="Y33" s="177"/>
-      <c r="Z33" s="177"/>
-      <c r="AA33" s="178" t="s">
+      <c r="R33" s="180"/>
+      <c r="S33" s="180"/>
+      <c r="T33" s="180"/>
+      <c r="U33" s="180"/>
+      <c r="V33" s="181"/>
+      <c r="W33" s="181"/>
+      <c r="X33" s="181"/>
+      <c r="Y33" s="217"/>
+      <c r="Z33" s="217"/>
+      <c r="AA33" s="196" t="s">
         <v>565</v>
       </c>
-      <c r="AB33" s="178"/>
-      <c r="AC33" s="178"/>
-      <c r="AD33" s="214"/>
-      <c r="AE33" s="214"/>
-      <c r="AF33" s="214"/>
-      <c r="AG33" s="214"/>
+      <c r="AB33" s="196"/>
+      <c r="AC33" s="196"/>
+      <c r="AD33" s="174"/>
+      <c r="AE33" s="174"/>
+      <c r="AF33" s="174"/>
+      <c r="AG33" s="174"/>
       <c r="AH33" s="2"/>
       <c r="AI33" s="2"/>
       <c r="AJ33" s="2"/>
@@ -11376,45 +11379,45 @@
       <c r="B34" s="140" t="s">
         <v>486</v>
       </c>
-      <c r="C34" s="179" t="s">
+      <c r="C34" s="180" t="s">
         <v>566</v>
       </c>
-      <c r="D34" s="179"/>
-      <c r="E34" s="179"/>
-      <c r="F34" s="214"/>
-      <c r="G34" s="214"/>
-      <c r="H34" s="214"/>
-      <c r="I34" s="179" t="s">
+      <c r="D34" s="180"/>
+      <c r="E34" s="180"/>
+      <c r="F34" s="174"/>
+      <c r="G34" s="174"/>
+      <c r="H34" s="174"/>
+      <c r="I34" s="180" t="s">
         <v>685</v>
       </c>
-      <c r="J34" s="179"/>
-      <c r="K34" s="179"/>
-      <c r="L34" s="179"/>
-      <c r="M34" s="190"/>
-      <c r="N34" s="190"/>
-      <c r="O34" s="190"/>
-      <c r="P34" s="190"/>
-      <c r="Q34" s="179" t="s">
+      <c r="J34" s="180"/>
+      <c r="K34" s="180"/>
+      <c r="L34" s="180"/>
+      <c r="M34" s="181"/>
+      <c r="N34" s="181"/>
+      <c r="O34" s="181"/>
+      <c r="P34" s="181"/>
+      <c r="Q34" s="180" t="s">
         <v>562</v>
       </c>
-      <c r="R34" s="179"/>
-      <c r="S34" s="179"/>
-      <c r="T34" s="179"/>
-      <c r="U34" s="179"/>
-      <c r="V34" s="190"/>
-      <c r="W34" s="190"/>
-      <c r="X34" s="190"/>
-      <c r="Y34" s="177"/>
-      <c r="Z34" s="177"/>
-      <c r="AA34" s="178" t="s">
+      <c r="R34" s="180"/>
+      <c r="S34" s="180"/>
+      <c r="T34" s="180"/>
+      <c r="U34" s="180"/>
+      <c r="V34" s="181"/>
+      <c r="W34" s="181"/>
+      <c r="X34" s="181"/>
+      <c r="Y34" s="217"/>
+      <c r="Z34" s="217"/>
+      <c r="AA34" s="196" t="s">
         <v>565</v>
       </c>
-      <c r="AB34" s="178"/>
-      <c r="AC34" s="178"/>
-      <c r="AD34" s="214"/>
-      <c r="AE34" s="214"/>
-      <c r="AF34" s="214"/>
-      <c r="AG34" s="214"/>
+      <c r="AB34" s="196"/>
+      <c r="AC34" s="196"/>
+      <c r="AD34" s="174"/>
+      <c r="AE34" s="174"/>
+      <c r="AF34" s="174"/>
+      <c r="AG34" s="174"/>
       <c r="AH34" s="2"/>
       <c r="AI34" s="2"/>
       <c r="AJ34" s="2"/>
@@ -11652,45 +11655,45 @@
       <c r="B35" s="168" t="s">
         <v>689</v>
       </c>
-      <c r="C35" s="195"/>
-      <c r="D35" s="195"/>
-      <c r="E35" s="195"/>
-      <c r="F35" s="195"/>
-      <c r="G35" s="195"/>
-      <c r="H35" s="195"/>
-      <c r="I35" s="179" t="s">
+      <c r="C35" s="175"/>
+      <c r="D35" s="175"/>
+      <c r="E35" s="175"/>
+      <c r="F35" s="175"/>
+      <c r="G35" s="175"/>
+      <c r="H35" s="175"/>
+      <c r="I35" s="180" t="s">
         <v>690</v>
       </c>
-      <c r="J35" s="179"/>
-      <c r="K35" s="179"/>
-      <c r="L35" s="179"/>
-      <c r="M35" s="174"/>
-      <c r="N35" s="174"/>
-      <c r="O35" s="174"/>
-      <c r="P35" s="174"/>
-      <c r="Q35" s="179" t="s">
+      <c r="J35" s="180"/>
+      <c r="K35" s="180"/>
+      <c r="L35" s="180"/>
+      <c r="M35" s="199"/>
+      <c r="N35" s="199"/>
+      <c r="O35" s="199"/>
+      <c r="P35" s="199"/>
+      <c r="Q35" s="180" t="s">
         <v>660</v>
       </c>
-      <c r="R35" s="179"/>
-      <c r="S35" s="179"/>
-      <c r="T35" s="179"/>
-      <c r="U35" s="179"/>
-      <c r="V35" s="176" t="s">
+      <c r="R35" s="180"/>
+      <c r="S35" s="180"/>
+      <c r="T35" s="180"/>
+      <c r="U35" s="180"/>
+      <c r="V35" s="173" t="s">
         <v>455</v>
       </c>
-      <c r="W35" s="176"/>
-      <c r="X35" s="195"/>
-      <c r="Y35" s="195"/>
-      <c r="Z35" s="195"/>
-      <c r="AA35" s="195"/>
-      <c r="AB35" s="176" t="s">
+      <c r="W35" s="173"/>
+      <c r="X35" s="175"/>
+      <c r="Y35" s="175"/>
+      <c r="Z35" s="175"/>
+      <c r="AA35" s="175"/>
+      <c r="AB35" s="173" t="s">
         <v>456</v>
       </c>
-      <c r="AC35" s="176"/>
-      <c r="AD35" s="195"/>
-      <c r="AE35" s="195"/>
-      <c r="AF35" s="195"/>
-      <c r="AG35" s="195"/>
+      <c r="AC35" s="173"/>
+      <c r="AD35" s="175"/>
+      <c r="AE35" s="175"/>
+      <c r="AF35" s="175"/>
+      <c r="AG35" s="175"/>
       <c r="AH35" s="2"/>
       <c r="AI35" s="2"/>
       <c r="AJ35" s="2"/>
@@ -11928,41 +11931,41 @@
       <c r="B36" s="168" t="s">
         <v>567</v>
       </c>
-      <c r="C36" s="179" t="s">
+      <c r="C36" s="180" t="s">
         <v>568</v>
       </c>
-      <c r="D36" s="179"/>
-      <c r="E36" s="179"/>
-      <c r="F36" s="179"/>
-      <c r="G36" s="179"/>
-      <c r="H36" s="179"/>
-      <c r="I36" s="190"/>
-      <c r="J36" s="190"/>
-      <c r="K36" s="190"/>
-      <c r="L36" s="190"/>
-      <c r="M36" s="190"/>
-      <c r="N36" s="190"/>
-      <c r="O36" s="190"/>
-      <c r="P36" s="190"/>
-      <c r="Q36" s="190"/>
-      <c r="R36" s="190"/>
-      <c r="S36" s="190"/>
-      <c r="T36" s="190"/>
-      <c r="U36" s="190"/>
-      <c r="V36" s="190"/>
-      <c r="W36" s="190"/>
-      <c r="X36" s="235" t="s">
+      <c r="D36" s="180"/>
+      <c r="E36" s="180"/>
+      <c r="F36" s="180"/>
+      <c r="G36" s="180"/>
+      <c r="H36" s="180"/>
+      <c r="I36" s="181"/>
+      <c r="J36" s="181"/>
+      <c r="K36" s="181"/>
+      <c r="L36" s="181"/>
+      <c r="M36" s="181"/>
+      <c r="N36" s="181"/>
+      <c r="O36" s="181"/>
+      <c r="P36" s="181"/>
+      <c r="Q36" s="181"/>
+      <c r="R36" s="181"/>
+      <c r="S36" s="181"/>
+      <c r="T36" s="181"/>
+      <c r="U36" s="181"/>
+      <c r="V36" s="181"/>
+      <c r="W36" s="181"/>
+      <c r="X36" s="195" t="s">
         <v>569</v>
       </c>
-      <c r="Y36" s="235"/>
-      <c r="Z36" s="235"/>
-      <c r="AA36" s="235"/>
-      <c r="AB36" s="235"/>
-      <c r="AC36" s="235"/>
-      <c r="AD36" s="214"/>
-      <c r="AE36" s="214"/>
-      <c r="AF36" s="214"/>
-      <c r="AG36" s="214"/>
+      <c r="Y36" s="195"/>
+      <c r="Z36" s="195"/>
+      <c r="AA36" s="195"/>
+      <c r="AB36" s="195"/>
+      <c r="AC36" s="195"/>
+      <c r="AD36" s="174"/>
+      <c r="AE36" s="174"/>
+      <c r="AF36" s="174"/>
+      <c r="AG36" s="174"/>
       <c r="AH36" s="2"/>
       <c r="AI36" s="2"/>
       <c r="AJ36" s="2"/>
@@ -12195,46 +12198,46 @@
       <c r="JG36" s="2"/>
       <c r="JH36" s="2"/>
     </row>
-    <row r="37" spans="1:268" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:268" ht="47.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1"/>
       <c r="B37" s="150" t="s">
         <v>720</v>
       </c>
-      <c r="C37" s="217"/>
-      <c r="D37" s="217"/>
-      <c r="E37" s="217"/>
-      <c r="F37" s="217"/>
-      <c r="G37" s="217"/>
-      <c r="H37" s="217"/>
-      <c r="I37" s="217"/>
-      <c r="J37" s="217"/>
-      <c r="K37" s="218"/>
-      <c r="L37" s="218"/>
-      <c r="M37" s="219" t="s">
+      <c r="C37" s="203"/>
+      <c r="D37" s="203"/>
+      <c r="E37" s="203"/>
+      <c r="F37" s="203"/>
+      <c r="G37" s="203"/>
+      <c r="H37" s="203"/>
+      <c r="I37" s="203"/>
+      <c r="J37" s="203"/>
+      <c r="K37" s="204"/>
+      <c r="L37" s="204"/>
+      <c r="M37" s="205" t="s">
         <v>721</v>
       </c>
-      <c r="N37" s="219"/>
-      <c r="O37" s="219"/>
-      <c r="P37" s="219"/>
-      <c r="Q37" s="215"/>
-      <c r="R37" s="215"/>
-      <c r="S37" s="215"/>
-      <c r="T37" s="215"/>
-      <c r="U37" s="215"/>
-      <c r="V37" s="216"/>
-      <c r="W37" s="216"/>
-      <c r="X37" s="187" t="s">
+      <c r="N37" s="205"/>
+      <c r="O37" s="205"/>
+      <c r="P37" s="205"/>
+      <c r="Q37" s="200"/>
+      <c r="R37" s="200"/>
+      <c r="S37" s="200"/>
+      <c r="T37" s="200"/>
+      <c r="U37" s="200"/>
+      <c r="V37" s="201"/>
+      <c r="W37" s="201"/>
+      <c r="X37" s="202" t="s">
         <v>696</v>
       </c>
-      <c r="Y37" s="187"/>
-      <c r="Z37" s="187"/>
-      <c r="AA37" s="187"/>
-      <c r="AB37" s="187"/>
-      <c r="AC37" s="187"/>
-      <c r="AD37" s="185"/>
-      <c r="AE37" s="185"/>
-      <c r="AF37" s="185"/>
-      <c r="AG37" s="185"/>
+      <c r="Y37" s="202"/>
+      <c r="Z37" s="202"/>
+      <c r="AA37" s="202"/>
+      <c r="AB37" s="202"/>
+      <c r="AC37" s="202"/>
+      <c r="AD37" s="232"/>
+      <c r="AE37" s="232"/>
+      <c r="AF37" s="232"/>
+      <c r="AG37" s="232"/>
       <c r="AH37" s="2"/>
       <c r="AI37" s="2"/>
       <c r="AJ37" s="2"/>
@@ -12502,614 +12505,727 @@
       <c r="AG38" s="153"/>
     </row>
     <row r="39" spans="1:268" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="181" t="s">
+      <c r="B39" s="233" t="s">
         <v>574</v>
       </c>
-      <c r="C39" s="181"/>
-      <c r="D39" s="181"/>
-      <c r="E39" s="181"/>
-      <c r="F39" s="181"/>
-      <c r="G39" s="181"/>
-      <c r="H39" s="181"/>
-      <c r="I39" s="181"/>
-      <c r="J39" s="181"/>
-      <c r="K39" s="181"/>
-      <c r="L39" s="181"/>
-      <c r="M39" s="181"/>
-      <c r="N39" s="181"/>
-      <c r="O39" s="181"/>
-      <c r="P39" s="181"/>
-      <c r="Q39" s="181"/>
-      <c r="R39" s="181"/>
-      <c r="S39" s="181"/>
-      <c r="T39" s="181"/>
-      <c r="U39" s="181"/>
-      <c r="V39" s="181"/>
-      <c r="W39" s="181"/>
-      <c r="X39" s="181"/>
-      <c r="Y39" s="181"/>
-      <c r="Z39" s="181"/>
-      <c r="AA39" s="181"/>
-      <c r="AB39" s="181"/>
-      <c r="AC39" s="181"/>
-      <c r="AD39" s="181"/>
-      <c r="AE39" s="181"/>
-      <c r="AF39" s="181"/>
-      <c r="AG39" s="181"/>
+      <c r="C39" s="233"/>
+      <c r="D39" s="233"/>
+      <c r="E39" s="233"/>
+      <c r="F39" s="233"/>
+      <c r="G39" s="233"/>
+      <c r="H39" s="233"/>
+      <c r="I39" s="233"/>
+      <c r="J39" s="233"/>
+      <c r="K39" s="233"/>
+      <c r="L39" s="233"/>
+      <c r="M39" s="233"/>
+      <c r="N39" s="233"/>
+      <c r="O39" s="233"/>
+      <c r="P39" s="233"/>
+      <c r="Q39" s="233"/>
+      <c r="R39" s="233"/>
+      <c r="S39" s="233"/>
+      <c r="T39" s="233"/>
+      <c r="U39" s="233"/>
+      <c r="V39" s="233"/>
+      <c r="W39" s="233"/>
+      <c r="X39" s="233"/>
+      <c r="Y39" s="233"/>
+      <c r="Z39" s="233"/>
+      <c r="AA39" s="233"/>
+      <c r="AB39" s="233"/>
+      <c r="AC39" s="233"/>
+      <c r="AD39" s="233"/>
+      <c r="AE39" s="233"/>
+      <c r="AF39" s="233"/>
+      <c r="AG39" s="233"/>
     </row>
     <row r="40" spans="1:268" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="182" t="s">
+      <c r="B40" s="179" t="s">
         <v>575</v>
       </c>
-      <c r="C40" s="182"/>
-      <c r="D40" s="182"/>
-      <c r="E40" s="182"/>
-      <c r="F40" s="182"/>
-      <c r="G40" s="182"/>
-      <c r="H40" s="182"/>
-      <c r="I40" s="182"/>
-      <c r="J40" s="182"/>
-      <c r="K40" s="182"/>
-      <c r="L40" s="182"/>
-      <c r="M40" s="182"/>
-      <c r="N40" s="182"/>
-      <c r="O40" s="182"/>
-      <c r="P40" s="182"/>
-      <c r="Q40" s="182"/>
-      <c r="R40" s="182"/>
-      <c r="S40" s="182"/>
-      <c r="T40" s="182"/>
-      <c r="U40" s="182"/>
-      <c r="V40" s="182"/>
-      <c r="W40" s="182"/>
-      <c r="X40" s="182"/>
-      <c r="Y40" s="182"/>
-      <c r="Z40" s="182"/>
-      <c r="AA40" s="182"/>
-      <c r="AB40" s="182"/>
-      <c r="AC40" s="182"/>
-      <c r="AD40" s="182"/>
-      <c r="AE40" s="182"/>
-      <c r="AF40" s="182"/>
-      <c r="AG40" s="182"/>
+      <c r="C40" s="179"/>
+      <c r="D40" s="179"/>
+      <c r="E40" s="179"/>
+      <c r="F40" s="179"/>
+      <c r="G40" s="179"/>
+      <c r="H40" s="179"/>
+      <c r="I40" s="179"/>
+      <c r="J40" s="179"/>
+      <c r="K40" s="179"/>
+      <c r="L40" s="179"/>
+      <c r="M40" s="179"/>
+      <c r="N40" s="179"/>
+      <c r="O40" s="179"/>
+      <c r="P40" s="179"/>
+      <c r="Q40" s="179"/>
+      <c r="R40" s="179"/>
+      <c r="S40" s="179"/>
+      <c r="T40" s="179"/>
+      <c r="U40" s="179"/>
+      <c r="V40" s="179"/>
+      <c r="W40" s="179"/>
+      <c r="X40" s="179"/>
+      <c r="Y40" s="179"/>
+      <c r="Z40" s="179"/>
+      <c r="AA40" s="179"/>
+      <c r="AB40" s="179"/>
+      <c r="AC40" s="179"/>
+      <c r="AD40" s="179"/>
+      <c r="AE40" s="179"/>
+      <c r="AF40" s="179"/>
+      <c r="AG40" s="179"/>
     </row>
     <row r="41" spans="1:268" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B41" s="176" t="s">
+      <c r="B41" s="173" t="s">
         <v>570</v>
       </c>
-      <c r="C41" s="176"/>
-      <c r="D41" s="176"/>
-      <c r="E41" s="176"/>
-      <c r="F41" s="176"/>
-      <c r="G41" s="176"/>
-      <c r="H41" s="176"/>
-      <c r="I41" s="176"/>
-      <c r="J41" s="176"/>
-      <c r="K41" s="176"/>
-      <c r="L41" s="176"/>
-      <c r="M41" s="176"/>
-      <c r="N41" s="176"/>
-      <c r="O41" s="176"/>
-      <c r="P41" s="176"/>
-      <c r="Q41" s="176"/>
-      <c r="R41" s="183" t="s">
+      <c r="C41" s="173"/>
+      <c r="D41" s="173"/>
+      <c r="E41" s="173"/>
+      <c r="F41" s="173"/>
+      <c r="G41" s="173"/>
+      <c r="H41" s="173"/>
+      <c r="I41" s="173"/>
+      <c r="J41" s="173"/>
+      <c r="K41" s="173"/>
+      <c r="L41" s="173"/>
+      <c r="M41" s="173"/>
+      <c r="N41" s="173"/>
+      <c r="O41" s="173"/>
+      <c r="P41" s="173"/>
+      <c r="Q41" s="173"/>
+      <c r="R41" s="172" t="s">
         <v>571</v>
       </c>
-      <c r="S41" s="183"/>
-      <c r="T41" s="183"/>
-      <c r="U41" s="183"/>
-      <c r="V41" s="183"/>
-      <c r="W41" s="183"/>
-      <c r="X41" s="183"/>
-      <c r="Y41" s="183"/>
-      <c r="Z41" s="183"/>
-      <c r="AA41" s="183"/>
-      <c r="AB41" s="183"/>
-      <c r="AC41" s="183"/>
-      <c r="AD41" s="183"/>
-      <c r="AE41" s="183"/>
-      <c r="AF41" s="183"/>
-      <c r="AG41" s="183"/>
+      <c r="S41" s="172"/>
+      <c r="T41" s="172"/>
+      <c r="U41" s="172"/>
+      <c r="V41" s="172"/>
+      <c r="W41" s="172"/>
+      <c r="X41" s="172"/>
+      <c r="Y41" s="172"/>
+      <c r="Z41" s="172"/>
+      <c r="AA41" s="172"/>
+      <c r="AB41" s="172"/>
+      <c r="AC41" s="172"/>
+      <c r="AD41" s="172"/>
+      <c r="AE41" s="172"/>
+      <c r="AF41" s="172"/>
+      <c r="AG41" s="172"/>
     </row>
     <row r="42" spans="1:268" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="182" t="s">
+      <c r="B42" s="179" t="s">
         <v>579</v>
       </c>
-      <c r="C42" s="182"/>
-      <c r="D42" s="182"/>
-      <c r="E42" s="182"/>
-      <c r="F42" s="182"/>
-      <c r="G42" s="182"/>
-      <c r="H42" s="182"/>
-      <c r="I42" s="182"/>
-      <c r="J42" s="182"/>
-      <c r="K42" s="182"/>
-      <c r="L42" s="182"/>
-      <c r="M42" s="182"/>
-      <c r="N42" s="182"/>
-      <c r="O42" s="182"/>
-      <c r="P42" s="182"/>
-      <c r="Q42" s="182"/>
-      <c r="R42" s="182"/>
-      <c r="S42" s="182"/>
-      <c r="T42" s="182"/>
-      <c r="U42" s="182"/>
-      <c r="V42" s="182"/>
-      <c r="W42" s="182"/>
-      <c r="X42" s="182"/>
-      <c r="Y42" s="182"/>
-      <c r="Z42" s="182"/>
-      <c r="AA42" s="182"/>
-      <c r="AB42" s="182"/>
-      <c r="AC42" s="182"/>
-      <c r="AD42" s="182"/>
-      <c r="AE42" s="182"/>
-      <c r="AF42" s="182"/>
-      <c r="AG42" s="182"/>
+      <c r="C42" s="179"/>
+      <c r="D42" s="179"/>
+      <c r="E42" s="179"/>
+      <c r="F42" s="179"/>
+      <c r="G42" s="179"/>
+      <c r="H42" s="179"/>
+      <c r="I42" s="179"/>
+      <c r="J42" s="179"/>
+      <c r="K42" s="179"/>
+      <c r="L42" s="179"/>
+      <c r="M42" s="179"/>
+      <c r="N42" s="179"/>
+      <c r="O42" s="179"/>
+      <c r="P42" s="179"/>
+      <c r="Q42" s="179"/>
+      <c r="R42" s="179"/>
+      <c r="S42" s="179"/>
+      <c r="T42" s="179"/>
+      <c r="U42" s="179"/>
+      <c r="V42" s="179"/>
+      <c r="W42" s="179"/>
+      <c r="X42" s="179"/>
+      <c r="Y42" s="179"/>
+      <c r="Z42" s="179"/>
+      <c r="AA42" s="179"/>
+      <c r="AB42" s="179"/>
+      <c r="AC42" s="179"/>
+      <c r="AD42" s="179"/>
+      <c r="AE42" s="179"/>
+      <c r="AF42" s="179"/>
+      <c r="AG42" s="179"/>
     </row>
     <row r="43" spans="1:268" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="176" t="s">
+      <c r="B43" s="173" t="s">
         <v>572</v>
       </c>
-      <c r="C43" s="176"/>
-      <c r="D43" s="176"/>
-      <c r="E43" s="176"/>
-      <c r="F43" s="176"/>
-      <c r="G43" s="176"/>
-      <c r="H43" s="176"/>
-      <c r="I43" s="176"/>
-      <c r="J43" s="176"/>
-      <c r="K43" s="176"/>
-      <c r="L43" s="176"/>
-      <c r="M43" s="176"/>
-      <c r="N43" s="176"/>
-      <c r="O43" s="176"/>
-      <c r="P43" s="176"/>
-      <c r="Q43" s="176"/>
-      <c r="R43" s="183" t="s">
+      <c r="C43" s="173"/>
+      <c r="D43" s="173"/>
+      <c r="E43" s="173"/>
+      <c r="F43" s="173"/>
+      <c r="G43" s="173"/>
+      <c r="H43" s="173"/>
+      <c r="I43" s="173"/>
+      <c r="J43" s="173"/>
+      <c r="K43" s="173"/>
+      <c r="L43" s="173"/>
+      <c r="M43" s="173"/>
+      <c r="N43" s="173"/>
+      <c r="O43" s="173"/>
+      <c r="P43" s="173"/>
+      <c r="Q43" s="173"/>
+      <c r="R43" s="172" t="s">
         <v>571</v>
       </c>
-      <c r="S43" s="183"/>
-      <c r="T43" s="183"/>
-      <c r="U43" s="183"/>
-      <c r="V43" s="183"/>
-      <c r="W43" s="183"/>
-      <c r="X43" s="183"/>
-      <c r="Y43" s="183"/>
-      <c r="Z43" s="183"/>
-      <c r="AA43" s="183"/>
-      <c r="AB43" s="183"/>
-      <c r="AC43" s="183"/>
-      <c r="AD43" s="183"/>
-      <c r="AE43" s="183"/>
-      <c r="AF43" s="183"/>
-      <c r="AG43" s="183"/>
+      <c r="S43" s="172"/>
+      <c r="T43" s="172"/>
+      <c r="U43" s="172"/>
+      <c r="V43" s="172"/>
+      <c r="W43" s="172"/>
+      <c r="X43" s="172"/>
+      <c r="Y43" s="172"/>
+      <c r="Z43" s="172"/>
+      <c r="AA43" s="172"/>
+      <c r="AB43" s="172"/>
+      <c r="AC43" s="172"/>
+      <c r="AD43" s="172"/>
+      <c r="AE43" s="172"/>
+      <c r="AF43" s="172"/>
+      <c r="AG43" s="172"/>
     </row>
     <row r="44" spans="1:268" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B44" s="180" t="s">
+      <c r="B44" s="198" t="s">
         <v>585</v>
       </c>
-      <c r="C44" s="180"/>
-      <c r="D44" s="180"/>
-      <c r="E44" s="180"/>
-      <c r="F44" s="180"/>
-      <c r="G44" s="180"/>
-      <c r="H44" s="180"/>
-      <c r="I44" s="180"/>
-      <c r="J44" s="180"/>
-      <c r="K44" s="180"/>
-      <c r="L44" s="180"/>
-      <c r="M44" s="180"/>
-      <c r="N44" s="180"/>
-      <c r="O44" s="180"/>
-      <c r="P44" s="180"/>
-      <c r="Q44" s="180"/>
-      <c r="R44" s="180"/>
-      <c r="S44" s="180"/>
-      <c r="T44" s="180"/>
-      <c r="U44" s="180"/>
-      <c r="V44" s="180"/>
-      <c r="W44" s="180"/>
-      <c r="X44" s="180"/>
-      <c r="Y44" s="180"/>
-      <c r="Z44" s="180"/>
-      <c r="AA44" s="180"/>
-      <c r="AB44" s="180"/>
-      <c r="AC44" s="180"/>
-      <c r="AD44" s="180"/>
-      <c r="AE44" s="180"/>
-      <c r="AF44" s="180"/>
-      <c r="AG44" s="180"/>
+      <c r="C44" s="198"/>
+      <c r="D44" s="198"/>
+      <c r="E44" s="198"/>
+      <c r="F44" s="198"/>
+      <c r="G44" s="198"/>
+      <c r="H44" s="198"/>
+      <c r="I44" s="198"/>
+      <c r="J44" s="198"/>
+      <c r="K44" s="198"/>
+      <c r="L44" s="198"/>
+      <c r="M44" s="198"/>
+      <c r="N44" s="198"/>
+      <c r="O44" s="198"/>
+      <c r="P44" s="198"/>
+      <c r="Q44" s="198"/>
+      <c r="R44" s="198"/>
+      <c r="S44" s="198"/>
+      <c r="T44" s="198"/>
+      <c r="U44" s="198"/>
+      <c r="V44" s="198"/>
+      <c r="W44" s="198"/>
+      <c r="X44" s="198"/>
+      <c r="Y44" s="198"/>
+      <c r="Z44" s="198"/>
+      <c r="AA44" s="198"/>
+      <c r="AB44" s="198"/>
+      <c r="AC44" s="198"/>
+      <c r="AD44" s="198"/>
+      <c r="AE44" s="198"/>
+      <c r="AF44" s="198"/>
+      <c r="AG44" s="198"/>
     </row>
     <row r="45" spans="1:268" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B45" s="182" t="s">
+      <c r="B45" s="179" t="s">
         <v>584</v>
       </c>
-      <c r="C45" s="182"/>
-      <c r="D45" s="182"/>
-      <c r="E45" s="182"/>
-      <c r="F45" s="182"/>
-      <c r="G45" s="182"/>
-      <c r="H45" s="182"/>
-      <c r="I45" s="182"/>
-      <c r="J45" s="182"/>
-      <c r="K45" s="182"/>
-      <c r="L45" s="182"/>
-      <c r="M45" s="182"/>
-      <c r="N45" s="182"/>
-      <c r="O45" s="182"/>
-      <c r="P45" s="182"/>
-      <c r="Q45" s="182"/>
-      <c r="R45" s="182"/>
-      <c r="S45" s="182"/>
-      <c r="T45" s="182"/>
-      <c r="U45" s="182"/>
-      <c r="V45" s="182"/>
-      <c r="W45" s="182"/>
-      <c r="X45" s="182"/>
-      <c r="Y45" s="182"/>
-      <c r="Z45" s="182"/>
-      <c r="AA45" s="182"/>
-      <c r="AB45" s="182"/>
-      <c r="AC45" s="182"/>
-      <c r="AD45" s="182"/>
-      <c r="AE45" s="182"/>
-      <c r="AF45" s="182"/>
-      <c r="AG45" s="182"/>
+      <c r="C45" s="179"/>
+      <c r="D45" s="179"/>
+      <c r="E45" s="179"/>
+      <c r="F45" s="179"/>
+      <c r="G45" s="179"/>
+      <c r="H45" s="179"/>
+      <c r="I45" s="179"/>
+      <c r="J45" s="179"/>
+      <c r="K45" s="179"/>
+      <c r="L45" s="179"/>
+      <c r="M45" s="179"/>
+      <c r="N45" s="179"/>
+      <c r="O45" s="179"/>
+      <c r="P45" s="179"/>
+      <c r="Q45" s="179"/>
+      <c r="R45" s="179"/>
+      <c r="S45" s="179"/>
+      <c r="T45" s="179"/>
+      <c r="U45" s="179"/>
+      <c r="V45" s="179"/>
+      <c r="W45" s="179"/>
+      <c r="X45" s="179"/>
+      <c r="Y45" s="179"/>
+      <c r="Z45" s="179"/>
+      <c r="AA45" s="179"/>
+      <c r="AB45" s="179"/>
+      <c r="AC45" s="179"/>
+      <c r="AD45" s="179"/>
+      <c r="AE45" s="179"/>
+      <c r="AF45" s="179"/>
+      <c r="AG45" s="179"/>
     </row>
     <row r="46" spans="1:268" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B46" s="176" t="s">
+      <c r="B46" s="173" t="s">
         <v>580</v>
       </c>
-      <c r="C46" s="176"/>
-      <c r="D46" s="176"/>
-      <c r="E46" s="176"/>
-      <c r="F46" s="176"/>
-      <c r="G46" s="176"/>
-      <c r="H46" s="176"/>
-      <c r="I46" s="176"/>
-      <c r="J46" s="176"/>
-      <c r="K46" s="176"/>
-      <c r="L46" s="176"/>
-      <c r="M46" s="176"/>
-      <c r="N46" s="176"/>
-      <c r="O46" s="176"/>
-      <c r="P46" s="176"/>
-      <c r="Q46" s="176"/>
-      <c r="R46" s="176" t="s">
+      <c r="C46" s="173"/>
+      <c r="D46" s="173"/>
+      <c r="E46" s="173"/>
+      <c r="F46" s="173"/>
+      <c r="G46" s="173"/>
+      <c r="H46" s="173"/>
+      <c r="I46" s="173"/>
+      <c r="J46" s="173"/>
+      <c r="K46" s="173"/>
+      <c r="L46" s="173"/>
+      <c r="M46" s="173"/>
+      <c r="N46" s="173"/>
+      <c r="O46" s="173"/>
+      <c r="P46" s="173"/>
+      <c r="Q46" s="173"/>
+      <c r="R46" s="173" t="s">
         <v>581</v>
       </c>
-      <c r="S46" s="176"/>
-      <c r="T46" s="176"/>
-      <c r="U46" s="176"/>
-      <c r="V46" s="232" t="s">
+      <c r="S46" s="173"/>
+      <c r="T46" s="173"/>
+      <c r="U46" s="173"/>
+      <c r="V46" s="176" t="s">
         <v>708</v>
       </c>
-      <c r="W46" s="233"/>
-      <c r="X46" s="233"/>
-      <c r="Y46" s="234"/>
-      <c r="Z46" s="232" t="s">
+      <c r="W46" s="177"/>
+      <c r="X46" s="177"/>
+      <c r="Y46" s="178"/>
+      <c r="Z46" s="176" t="s">
         <v>702</v>
       </c>
-      <c r="AA46" s="233"/>
-      <c r="AB46" s="233"/>
-      <c r="AC46" s="234"/>
-      <c r="AD46" s="183" t="s">
+      <c r="AA46" s="177"/>
+      <c r="AB46" s="177"/>
+      <c r="AC46" s="178"/>
+      <c r="AD46" s="172" t="s">
         <v>5</v>
       </c>
-      <c r="AE46" s="183"/>
-      <c r="AF46" s="183"/>
-      <c r="AG46" s="183"/>
+      <c r="AE46" s="172"/>
+      <c r="AF46" s="172"/>
+      <c r="AG46" s="172"/>
     </row>
     <row r="47" spans="1:268" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B47" s="182" t="s">
+      <c r="B47" s="179" t="s">
         <v>586</v>
       </c>
-      <c r="C47" s="182"/>
-      <c r="D47" s="182"/>
-      <c r="E47" s="182"/>
-      <c r="F47" s="182"/>
-      <c r="G47" s="182"/>
-      <c r="H47" s="182"/>
-      <c r="I47" s="182"/>
-      <c r="J47" s="182"/>
-      <c r="K47" s="182"/>
-      <c r="L47" s="182"/>
-      <c r="M47" s="182"/>
-      <c r="N47" s="182"/>
-      <c r="O47" s="182"/>
-      <c r="P47" s="182"/>
-      <c r="Q47" s="182"/>
-      <c r="R47" s="182"/>
-      <c r="S47" s="182"/>
-      <c r="T47" s="182"/>
-      <c r="U47" s="182"/>
-      <c r="V47" s="182"/>
-      <c r="W47" s="182"/>
-      <c r="X47" s="182"/>
-      <c r="Y47" s="182"/>
-      <c r="Z47" s="182"/>
-      <c r="AA47" s="182"/>
-      <c r="AB47" s="182"/>
-      <c r="AC47" s="182"/>
-      <c r="AD47" s="182"/>
-      <c r="AE47" s="182"/>
-      <c r="AF47" s="182"/>
-      <c r="AG47" s="182"/>
+      <c r="C47" s="179"/>
+      <c r="D47" s="179"/>
+      <c r="E47" s="179"/>
+      <c r="F47" s="179"/>
+      <c r="G47" s="179"/>
+      <c r="H47" s="179"/>
+      <c r="I47" s="179"/>
+      <c r="J47" s="179"/>
+      <c r="K47" s="179"/>
+      <c r="L47" s="179"/>
+      <c r="M47" s="179"/>
+      <c r="N47" s="179"/>
+      <c r="O47" s="179"/>
+      <c r="P47" s="179"/>
+      <c r="Q47" s="179"/>
+      <c r="R47" s="179"/>
+      <c r="S47" s="179"/>
+      <c r="T47" s="179"/>
+      <c r="U47" s="179"/>
+      <c r="V47" s="179"/>
+      <c r="W47" s="179"/>
+      <c r="X47" s="179"/>
+      <c r="Y47" s="179"/>
+      <c r="Z47" s="179"/>
+      <c r="AA47" s="179"/>
+      <c r="AB47" s="179"/>
+      <c r="AC47" s="179"/>
+      <c r="AD47" s="179"/>
+      <c r="AE47" s="179"/>
+      <c r="AF47" s="179"/>
+      <c r="AG47" s="179"/>
     </row>
     <row r="48" spans="1:268" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B48" s="176" t="s">
+      <c r="B48" s="173" t="s">
         <v>582</v>
       </c>
-      <c r="C48" s="176"/>
-      <c r="D48" s="176"/>
-      <c r="E48" s="176"/>
-      <c r="F48" s="176"/>
-      <c r="G48" s="176"/>
-      <c r="H48" s="176"/>
-      <c r="I48" s="176"/>
-      <c r="J48" s="176"/>
-      <c r="K48" s="176"/>
-      <c r="L48" s="176"/>
-      <c r="M48" s="176"/>
-      <c r="N48" s="176"/>
-      <c r="O48" s="176"/>
-      <c r="P48" s="176"/>
-      <c r="Q48" s="176"/>
-      <c r="R48" s="176" t="s">
+      <c r="C48" s="173"/>
+      <c r="D48" s="173"/>
+      <c r="E48" s="173"/>
+      <c r="F48" s="173"/>
+      <c r="G48" s="173"/>
+      <c r="H48" s="173"/>
+      <c r="I48" s="173"/>
+      <c r="J48" s="173"/>
+      <c r="K48" s="173"/>
+      <c r="L48" s="173"/>
+      <c r="M48" s="173"/>
+      <c r="N48" s="173"/>
+      <c r="O48" s="173"/>
+      <c r="P48" s="173"/>
+      <c r="Q48" s="173"/>
+      <c r="R48" s="173" t="s">
         <v>583</v>
       </c>
-      <c r="S48" s="176"/>
-      <c r="T48" s="176"/>
-      <c r="U48" s="176"/>
-      <c r="V48" s="232" t="s">
+      <c r="S48" s="173"/>
+      <c r="T48" s="173"/>
+      <c r="U48" s="173"/>
+      <c r="V48" s="176" t="s">
         <v>708</v>
       </c>
-      <c r="W48" s="233"/>
-      <c r="X48" s="233"/>
-      <c r="Y48" s="234"/>
-      <c r="Z48" s="232" t="s">
+      <c r="W48" s="177"/>
+      <c r="X48" s="177"/>
+      <c r="Y48" s="178"/>
+      <c r="Z48" s="176" t="s">
         <v>702</v>
       </c>
-      <c r="AA48" s="233"/>
-      <c r="AB48" s="233"/>
-      <c r="AC48" s="234"/>
-      <c r="AD48" s="183" t="s">
+      <c r="AA48" s="177"/>
+      <c r="AB48" s="177"/>
+      <c r="AC48" s="178"/>
+      <c r="AD48" s="172" t="s">
         <v>5</v>
       </c>
-      <c r="AE48" s="183"/>
-      <c r="AF48" s="183"/>
-      <c r="AG48" s="183"/>
+      <c r="AE48" s="172"/>
+      <c r="AF48" s="172"/>
+      <c r="AG48" s="172"/>
     </row>
     <row r="49" spans="2:33" x14ac:dyDescent="0.2">
-      <c r="B49" s="229" t="s">
+      <c r="B49" s="191" t="s">
         <v>704</v>
       </c>
-      <c r="C49" s="230"/>
-      <c r="D49" s="230"/>
-      <c r="E49" s="230"/>
-      <c r="F49" s="230"/>
-      <c r="G49" s="230"/>
-      <c r="H49" s="230"/>
-      <c r="I49" s="230"/>
-      <c r="J49" s="230"/>
-      <c r="K49" s="230"/>
-      <c r="L49" s="230"/>
-      <c r="M49" s="230"/>
-      <c r="N49" s="230"/>
-      <c r="O49" s="230"/>
-      <c r="P49" s="230"/>
-      <c r="Q49" s="230"/>
-      <c r="R49" s="230"/>
-      <c r="S49" s="230"/>
-      <c r="T49" s="230"/>
-      <c r="U49" s="230"/>
-      <c r="V49" s="230"/>
-      <c r="W49" s="230"/>
-      <c r="X49" s="230"/>
-      <c r="Y49" s="230"/>
-      <c r="Z49" s="230"/>
-      <c r="AA49" s="230"/>
-      <c r="AB49" s="230"/>
-      <c r="AC49" s="230"/>
-      <c r="AD49" s="230"/>
-      <c r="AE49" s="230"/>
-      <c r="AF49" s="230"/>
-      <c r="AG49" s="231"/>
+      <c r="C49" s="192"/>
+      <c r="D49" s="192"/>
+      <c r="E49" s="192"/>
+      <c r="F49" s="192"/>
+      <c r="G49" s="192"/>
+      <c r="H49" s="192"/>
+      <c r="I49" s="192"/>
+      <c r="J49" s="192"/>
+      <c r="K49" s="192"/>
+      <c r="L49" s="192"/>
+      <c r="M49" s="192"/>
+      <c r="N49" s="192"/>
+      <c r="O49" s="192"/>
+      <c r="P49" s="192"/>
+      <c r="Q49" s="192"/>
+      <c r="R49" s="192"/>
+      <c r="S49" s="192"/>
+      <c r="T49" s="192"/>
+      <c r="U49" s="192"/>
+      <c r="V49" s="192"/>
+      <c r="W49" s="192"/>
+      <c r="X49" s="192"/>
+      <c r="Y49" s="192"/>
+      <c r="Z49" s="192"/>
+      <c r="AA49" s="192"/>
+      <c r="AB49" s="192"/>
+      <c r="AC49" s="192"/>
+      <c r="AD49" s="192"/>
+      <c r="AE49" s="192"/>
+      <c r="AF49" s="192"/>
+      <c r="AG49" s="193"/>
     </row>
     <row r="50" spans="2:33" x14ac:dyDescent="0.2">
-      <c r="B50" s="220" t="s">
+      <c r="B50" s="182" t="s">
         <v>603</v>
       </c>
-      <c r="C50" s="221"/>
-      <c r="D50" s="221"/>
-      <c r="E50" s="221"/>
-      <c r="F50" s="221"/>
-      <c r="G50" s="221"/>
-      <c r="H50" s="221"/>
-      <c r="I50" s="221"/>
-      <c r="J50" s="221"/>
-      <c r="K50" s="221"/>
-      <c r="L50" s="221"/>
-      <c r="M50" s="221"/>
-      <c r="N50" s="221"/>
-      <c r="O50" s="221"/>
-      <c r="P50" s="221"/>
-      <c r="Q50" s="221"/>
-      <c r="R50" s="221"/>
-      <c r="S50" s="221"/>
-      <c r="T50" s="221"/>
-      <c r="U50" s="221"/>
-      <c r="V50" s="221"/>
-      <c r="W50" s="221"/>
-      <c r="X50" s="221"/>
-      <c r="Y50" s="221"/>
-      <c r="Z50" s="221"/>
-      <c r="AA50" s="221"/>
-      <c r="AB50" s="221"/>
-      <c r="AC50" s="221"/>
-      <c r="AD50" s="221"/>
-      <c r="AE50" s="221"/>
-      <c r="AF50" s="221"/>
-      <c r="AG50" s="222"/>
+      <c r="C50" s="183"/>
+      <c r="D50" s="183"/>
+      <c r="E50" s="183"/>
+      <c r="F50" s="183"/>
+      <c r="G50" s="183"/>
+      <c r="H50" s="183"/>
+      <c r="I50" s="183"/>
+      <c r="J50" s="183"/>
+      <c r="K50" s="183"/>
+      <c r="L50" s="183"/>
+      <c r="M50" s="183"/>
+      <c r="N50" s="183"/>
+      <c r="O50" s="183"/>
+      <c r="P50" s="183"/>
+      <c r="Q50" s="183"/>
+      <c r="R50" s="183"/>
+      <c r="S50" s="183"/>
+      <c r="T50" s="183"/>
+      <c r="U50" s="183"/>
+      <c r="V50" s="183"/>
+      <c r="W50" s="183"/>
+      <c r="X50" s="183"/>
+      <c r="Y50" s="183"/>
+      <c r="Z50" s="183"/>
+      <c r="AA50" s="183"/>
+      <c r="AB50" s="183"/>
+      <c r="AC50" s="183"/>
+      <c r="AD50" s="183"/>
+      <c r="AE50" s="183"/>
+      <c r="AF50" s="183"/>
+      <c r="AG50" s="184"/>
     </row>
     <row r="51" spans="2:33" x14ac:dyDescent="0.2">
-      <c r="B51" s="223"/>
-      <c r="C51" s="224"/>
-      <c r="D51" s="224"/>
-      <c r="E51" s="224"/>
-      <c r="F51" s="224"/>
-      <c r="G51" s="224"/>
-      <c r="H51" s="224"/>
-      <c r="I51" s="224"/>
-      <c r="J51" s="224"/>
-      <c r="K51" s="224"/>
-      <c r="L51" s="224"/>
-      <c r="M51" s="224"/>
-      <c r="N51" s="224"/>
-      <c r="O51" s="224"/>
-      <c r="P51" s="224"/>
-      <c r="Q51" s="224"/>
-      <c r="R51" s="224"/>
-      <c r="S51" s="224"/>
-      <c r="T51" s="224"/>
-      <c r="U51" s="224"/>
-      <c r="V51" s="224"/>
-      <c r="W51" s="224"/>
-      <c r="X51" s="224"/>
-      <c r="Y51" s="224"/>
-      <c r="Z51" s="224"/>
-      <c r="AA51" s="224"/>
-      <c r="AB51" s="224"/>
-      <c r="AC51" s="224"/>
-      <c r="AD51" s="224"/>
-      <c r="AE51" s="224"/>
-      <c r="AF51" s="224"/>
-      <c r="AG51" s="225"/>
+      <c r="B51" s="185"/>
+      <c r="C51" s="186"/>
+      <c r="D51" s="186"/>
+      <c r="E51" s="186"/>
+      <c r="F51" s="186"/>
+      <c r="G51" s="186"/>
+      <c r="H51" s="186"/>
+      <c r="I51" s="186"/>
+      <c r="J51" s="186"/>
+      <c r="K51" s="186"/>
+      <c r="L51" s="186"/>
+      <c r="M51" s="186"/>
+      <c r="N51" s="186"/>
+      <c r="O51" s="186"/>
+      <c r="P51" s="186"/>
+      <c r="Q51" s="186"/>
+      <c r="R51" s="186"/>
+      <c r="S51" s="186"/>
+      <c r="T51" s="186"/>
+      <c r="U51" s="186"/>
+      <c r="V51" s="186"/>
+      <c r="W51" s="186"/>
+      <c r="X51" s="186"/>
+      <c r="Y51" s="186"/>
+      <c r="Z51" s="186"/>
+      <c r="AA51" s="186"/>
+      <c r="AB51" s="186"/>
+      <c r="AC51" s="186"/>
+      <c r="AD51" s="186"/>
+      <c r="AE51" s="186"/>
+      <c r="AF51" s="186"/>
+      <c r="AG51" s="187"/>
     </row>
     <row r="52" spans="2:33" x14ac:dyDescent="0.2">
-      <c r="B52" s="226"/>
-      <c r="C52" s="227"/>
-      <c r="D52" s="227"/>
-      <c r="E52" s="227"/>
-      <c r="F52" s="227"/>
-      <c r="G52" s="227"/>
-      <c r="H52" s="227"/>
-      <c r="I52" s="227"/>
-      <c r="J52" s="227"/>
-      <c r="K52" s="227"/>
-      <c r="L52" s="227"/>
-      <c r="M52" s="227"/>
-      <c r="N52" s="227"/>
-      <c r="O52" s="227"/>
-      <c r="P52" s="227"/>
-      <c r="Q52" s="227"/>
-      <c r="R52" s="227"/>
-      <c r="S52" s="227"/>
-      <c r="T52" s="227"/>
-      <c r="U52" s="227"/>
-      <c r="V52" s="227"/>
-      <c r="W52" s="227"/>
-      <c r="X52" s="227"/>
-      <c r="Y52" s="227"/>
-      <c r="Z52" s="227"/>
-      <c r="AA52" s="227"/>
-      <c r="AB52" s="227"/>
-      <c r="AC52" s="227"/>
-      <c r="AD52" s="227"/>
-      <c r="AE52" s="227"/>
-      <c r="AF52" s="227"/>
-      <c r="AG52" s="228"/>
+      <c r="B52" s="188"/>
+      <c r="C52" s="189"/>
+      <c r="D52" s="189"/>
+      <c r="E52" s="189"/>
+      <c r="F52" s="189"/>
+      <c r="G52" s="189"/>
+      <c r="H52" s="189"/>
+      <c r="I52" s="189"/>
+      <c r="J52" s="189"/>
+      <c r="K52" s="189"/>
+      <c r="L52" s="189"/>
+      <c r="M52" s="189"/>
+      <c r="N52" s="189"/>
+      <c r="O52" s="189"/>
+      <c r="P52" s="189"/>
+      <c r="Q52" s="189"/>
+      <c r="R52" s="189"/>
+      <c r="S52" s="189"/>
+      <c r="T52" s="189"/>
+      <c r="U52" s="189"/>
+      <c r="V52" s="189"/>
+      <c r="W52" s="189"/>
+      <c r="X52" s="189"/>
+      <c r="Y52" s="189"/>
+      <c r="Z52" s="189"/>
+      <c r="AA52" s="189"/>
+      <c r="AB52" s="189"/>
+      <c r="AC52" s="189"/>
+      <c r="AD52" s="189"/>
+      <c r="AE52" s="189"/>
+      <c r="AF52" s="189"/>
+      <c r="AG52" s="190"/>
     </row>
     <row r="53" spans="2:33" x14ac:dyDescent="0.2">
-      <c r="B53" s="180" t="s">
+      <c r="B53" s="198" t="s">
         <v>703</v>
       </c>
-      <c r="C53" s="180"/>
-      <c r="D53" s="180"/>
-      <c r="E53" s="180"/>
-      <c r="F53" s="180"/>
-      <c r="G53" s="180"/>
-      <c r="H53" s="180"/>
-      <c r="I53" s="180"/>
-      <c r="J53" s="180"/>
-      <c r="K53" s="180"/>
-      <c r="L53" s="180"/>
-      <c r="M53" s="180"/>
-      <c r="N53" s="180"/>
-      <c r="O53" s="180"/>
-      <c r="P53" s="180"/>
-      <c r="Q53" s="180"/>
-      <c r="R53" s="180"/>
-      <c r="S53" s="180"/>
-      <c r="T53" s="180"/>
-      <c r="U53" s="180"/>
-      <c r="V53" s="180"/>
-      <c r="W53" s="180"/>
-      <c r="X53" s="180"/>
-      <c r="Y53" s="180"/>
-      <c r="Z53" s="180"/>
-      <c r="AA53" s="180"/>
-      <c r="AB53" s="180"/>
-      <c r="AC53" s="180"/>
-      <c r="AD53" s="180"/>
-      <c r="AE53" s="180"/>
-      <c r="AF53" s="180"/>
-      <c r="AG53" s="180"/>
+      <c r="C53" s="198"/>
+      <c r="D53" s="198"/>
+      <c r="E53" s="198"/>
+      <c r="F53" s="198"/>
+      <c r="G53" s="198"/>
+      <c r="H53" s="198"/>
+      <c r="I53" s="198"/>
+      <c r="J53" s="198"/>
+      <c r="K53" s="198"/>
+      <c r="L53" s="198"/>
+      <c r="M53" s="198"/>
+      <c r="N53" s="198"/>
+      <c r="O53" s="198"/>
+      <c r="P53" s="198"/>
+      <c r="Q53" s="198"/>
+      <c r="R53" s="198"/>
+      <c r="S53" s="198"/>
+      <c r="T53" s="198"/>
+      <c r="U53" s="198"/>
+      <c r="V53" s="198"/>
+      <c r="W53" s="198"/>
+      <c r="X53" s="198"/>
+      <c r="Y53" s="198"/>
+      <c r="Z53" s="198"/>
+      <c r="AA53" s="198"/>
+      <c r="AB53" s="198"/>
+      <c r="AC53" s="198"/>
+      <c r="AD53" s="198"/>
+      <c r="AE53" s="198"/>
+      <c r="AF53" s="198"/>
+      <c r="AG53" s="198"/>
     </row>
     <row r="54" spans="2:33" ht="31.35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B54" s="179" t="s">
+      <c r="B54" s="180" t="s">
         <v>602</v>
       </c>
-      <c r="C54" s="179"/>
-      <c r="D54" s="179"/>
-      <c r="E54" s="179"/>
-      <c r="F54" s="179"/>
-      <c r="G54" s="179"/>
-      <c r="H54" s="179"/>
-      <c r="I54" s="179"/>
-      <c r="J54" s="179"/>
-      <c r="K54" s="179"/>
-      <c r="L54" s="179"/>
-      <c r="M54" s="179"/>
-      <c r="N54" s="179"/>
-      <c r="O54" s="179"/>
-      <c r="P54" s="177"/>
-      <c r="Q54" s="177"/>
-      <c r="R54" s="177"/>
-      <c r="S54" s="177"/>
-      <c r="T54" s="177"/>
-      <c r="U54" s="177"/>
-      <c r="V54" s="177"/>
-      <c r="W54" s="177"/>
-      <c r="X54" s="177"/>
-      <c r="Y54" s="177"/>
-      <c r="Z54" s="177"/>
-      <c r="AA54" s="177"/>
-      <c r="AB54" s="177"/>
-      <c r="AC54" s="177"/>
-      <c r="AD54" s="177"/>
-      <c r="AE54" s="177"/>
-      <c r="AF54" s="177"/>
-      <c r="AG54" s="177"/>
+      <c r="C54" s="180"/>
+      <c r="D54" s="180"/>
+      <c r="E54" s="180"/>
+      <c r="F54" s="180"/>
+      <c r="G54" s="180"/>
+      <c r="H54" s="180"/>
+      <c r="I54" s="180"/>
+      <c r="J54" s="180"/>
+      <c r="K54" s="180"/>
+      <c r="L54" s="180"/>
+      <c r="M54" s="180"/>
+      <c r="N54" s="180"/>
+      <c r="O54" s="180"/>
+      <c r="P54" s="217"/>
+      <c r="Q54" s="217"/>
+      <c r="R54" s="217"/>
+      <c r="S54" s="217"/>
+      <c r="T54" s="217"/>
+      <c r="U54" s="217"/>
+      <c r="V54" s="217"/>
+      <c r="W54" s="217"/>
+      <c r="X54" s="217"/>
+      <c r="Y54" s="217"/>
+      <c r="Z54" s="217"/>
+      <c r="AA54" s="217"/>
+      <c r="AB54" s="217"/>
+      <c r="AC54" s="217"/>
+      <c r="AD54" s="217"/>
+      <c r="AE54" s="217"/>
+      <c r="AF54" s="217"/>
+      <c r="AG54" s="217"/>
     </row>
   </sheetData>
   <mergeCells count="167">
-    <mergeCell ref="AD46:AG46"/>
-    <mergeCell ref="R43:AG43"/>
-    <mergeCell ref="B43:Q43"/>
-    <mergeCell ref="F34:H34"/>
-    <mergeCell ref="AD35:AG35"/>
-    <mergeCell ref="V48:Y48"/>
-    <mergeCell ref="Z48:AC48"/>
-    <mergeCell ref="B48:Q48"/>
-    <mergeCell ref="B47:AG47"/>
-    <mergeCell ref="R48:U48"/>
-    <mergeCell ref="AD48:AG48"/>
-    <mergeCell ref="R46:U46"/>
-    <mergeCell ref="C36:H36"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="B10:AG10"/>
+    <mergeCell ref="U12:X12"/>
+    <mergeCell ref="C12:M12"/>
+    <mergeCell ref="B19:AG19"/>
+    <mergeCell ref="B28:AG28"/>
+    <mergeCell ref="T21:W21"/>
+    <mergeCell ref="X21:AA21"/>
+    <mergeCell ref="U15:X15"/>
+    <mergeCell ref="AB21:AG21"/>
+    <mergeCell ref="X23:AA23"/>
+    <mergeCell ref="X20:AG20"/>
+    <mergeCell ref="C21:K21"/>
+    <mergeCell ref="O12:T12"/>
+    <mergeCell ref="Y12:AG12"/>
+    <mergeCell ref="Y13:AG13"/>
+    <mergeCell ref="C23:K23"/>
+    <mergeCell ref="L22:P22"/>
+    <mergeCell ref="Q22:S22"/>
+    <mergeCell ref="T22:W22"/>
+    <mergeCell ref="C26:AG26"/>
+    <mergeCell ref="AA32:AC32"/>
+    <mergeCell ref="AA33:AC33"/>
+    <mergeCell ref="AA34:AC34"/>
+    <mergeCell ref="B54:O54"/>
+    <mergeCell ref="P54:AG54"/>
+    <mergeCell ref="B53:AG53"/>
+    <mergeCell ref="B14:AG14"/>
+    <mergeCell ref="Y15:AG15"/>
+    <mergeCell ref="B39:AG39"/>
+    <mergeCell ref="B40:AG40"/>
+    <mergeCell ref="B41:Q41"/>
+    <mergeCell ref="R41:AG41"/>
+    <mergeCell ref="B18:AG18"/>
+    <mergeCell ref="AD37:AG37"/>
+    <mergeCell ref="L21:P21"/>
+    <mergeCell ref="Q21:S21"/>
+    <mergeCell ref="C20:P20"/>
+    <mergeCell ref="Q20:W20"/>
+    <mergeCell ref="C15:M15"/>
+    <mergeCell ref="O15:T15"/>
+    <mergeCell ref="C16:Q16"/>
+    <mergeCell ref="R16:X16"/>
+    <mergeCell ref="Y16:AG16"/>
+    <mergeCell ref="AE23:AG23"/>
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="C8:Q8"/>
+    <mergeCell ref="R8:X8"/>
+    <mergeCell ref="Y8:AG8"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="Y31:Z31"/>
+    <mergeCell ref="Y32:Z32"/>
+    <mergeCell ref="Q34:U34"/>
+    <mergeCell ref="V34:X34"/>
+    <mergeCell ref="Y33:Z33"/>
+    <mergeCell ref="I34:L34"/>
+    <mergeCell ref="Q32:U32"/>
+    <mergeCell ref="V31:X31"/>
+    <mergeCell ref="Q31:U31"/>
+    <mergeCell ref="Q33:U33"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="M33:N33"/>
+    <mergeCell ref="Y34:Z34"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="C13:Q13"/>
+    <mergeCell ref="R13:X13"/>
+    <mergeCell ref="L23:P23"/>
+    <mergeCell ref="AB23:AD23"/>
+    <mergeCell ref="M3:O3"/>
+    <mergeCell ref="P3:S3"/>
+    <mergeCell ref="O4:S4"/>
+    <mergeCell ref="B11:AG11"/>
+    <mergeCell ref="Y7:AB7"/>
+    <mergeCell ref="AC7:AG7"/>
+    <mergeCell ref="AE22:AG22"/>
+    <mergeCell ref="C22:K22"/>
+    <mergeCell ref="B6:AG6"/>
+    <mergeCell ref="T4:X4"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="E4:L4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="V3:AB3"/>
+    <mergeCell ref="Y4:AB4"/>
+    <mergeCell ref="C2:AB2"/>
+    <mergeCell ref="F3:L3"/>
+    <mergeCell ref="AC2:AG4"/>
+    <mergeCell ref="T7:X7"/>
+    <mergeCell ref="N7:Q7"/>
+    <mergeCell ref="K7:M7"/>
+    <mergeCell ref="AB22:AD22"/>
+    <mergeCell ref="X22:AA22"/>
+    <mergeCell ref="I29:L29"/>
+    <mergeCell ref="T29:W29"/>
+    <mergeCell ref="X29:AC29"/>
+    <mergeCell ref="AD29:AG29"/>
+    <mergeCell ref="C29:H29"/>
+    <mergeCell ref="P29:S29"/>
+    <mergeCell ref="M29:O29"/>
+    <mergeCell ref="Q27:U27"/>
+    <mergeCell ref="AD27:AG27"/>
+    <mergeCell ref="X27:AC27"/>
+    <mergeCell ref="V27:W27"/>
+    <mergeCell ref="C27:P27"/>
+    <mergeCell ref="AD33:AG33"/>
+    <mergeCell ref="V32:X32"/>
+    <mergeCell ref="AD32:AG32"/>
+    <mergeCell ref="AD34:AG34"/>
+    <mergeCell ref="B42:AG42"/>
+    <mergeCell ref="Q23:S23"/>
+    <mergeCell ref="T23:W23"/>
+    <mergeCell ref="C24:AG24"/>
+    <mergeCell ref="B25:AG25"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="M35:P35"/>
+    <mergeCell ref="Q35:U35"/>
+    <mergeCell ref="V35:W35"/>
+    <mergeCell ref="AD31:AG31"/>
+    <mergeCell ref="Q37:U37"/>
+    <mergeCell ref="V37:W37"/>
+    <mergeCell ref="X37:AC37"/>
+    <mergeCell ref="C37:J37"/>
+    <mergeCell ref="K37:L37"/>
+    <mergeCell ref="M37:P37"/>
+    <mergeCell ref="X35:AA35"/>
+    <mergeCell ref="AB35:AC35"/>
+    <mergeCell ref="V33:X33"/>
+    <mergeCell ref="AA31:AC31"/>
     <mergeCell ref="B50:AG52"/>
     <mergeCell ref="B49:AG49"/>
     <mergeCell ref="V46:Y46"/>
@@ -13134,134 +13250,21 @@
     <mergeCell ref="I33:L33"/>
     <mergeCell ref="B44:AG44"/>
     <mergeCell ref="B45:AG45"/>
-    <mergeCell ref="AD33:AG33"/>
-    <mergeCell ref="V32:X32"/>
-    <mergeCell ref="AD32:AG32"/>
-    <mergeCell ref="AD34:AG34"/>
-    <mergeCell ref="B42:AG42"/>
-    <mergeCell ref="Q23:S23"/>
-    <mergeCell ref="T23:W23"/>
-    <mergeCell ref="C24:AG24"/>
-    <mergeCell ref="B25:AG25"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="M35:P35"/>
-    <mergeCell ref="Q35:U35"/>
-    <mergeCell ref="V35:W35"/>
-    <mergeCell ref="AD31:AG31"/>
-    <mergeCell ref="Q37:U37"/>
-    <mergeCell ref="V37:W37"/>
-    <mergeCell ref="X37:AC37"/>
-    <mergeCell ref="C37:J37"/>
-    <mergeCell ref="K37:L37"/>
-    <mergeCell ref="M37:P37"/>
-    <mergeCell ref="X35:AA35"/>
-    <mergeCell ref="AB35:AC35"/>
-    <mergeCell ref="V33:X33"/>
-    <mergeCell ref="AA31:AC31"/>
-    <mergeCell ref="I29:L29"/>
-    <mergeCell ref="T29:W29"/>
-    <mergeCell ref="X29:AC29"/>
-    <mergeCell ref="AD29:AG29"/>
-    <mergeCell ref="C29:H29"/>
-    <mergeCell ref="P29:S29"/>
-    <mergeCell ref="M29:O29"/>
-    <mergeCell ref="Q27:U27"/>
-    <mergeCell ref="AD27:AG27"/>
-    <mergeCell ref="X27:AC27"/>
-    <mergeCell ref="V27:W27"/>
-    <mergeCell ref="C27:P27"/>
-    <mergeCell ref="M3:O3"/>
-    <mergeCell ref="P3:S3"/>
-    <mergeCell ref="O4:S4"/>
-    <mergeCell ref="B11:AG11"/>
-    <mergeCell ref="Y7:AB7"/>
-    <mergeCell ref="AC7:AG7"/>
-    <mergeCell ref="AE22:AG22"/>
-    <mergeCell ref="C22:K22"/>
-    <mergeCell ref="B6:AG6"/>
-    <mergeCell ref="T4:X4"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="E4:L4"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="V3:AB3"/>
-    <mergeCell ref="Y4:AB4"/>
-    <mergeCell ref="C2:AB2"/>
-    <mergeCell ref="F3:L3"/>
-    <mergeCell ref="AC2:AG4"/>
-    <mergeCell ref="T7:X7"/>
-    <mergeCell ref="N7:Q7"/>
-    <mergeCell ref="K7:M7"/>
-    <mergeCell ref="AB22:AD22"/>
-    <mergeCell ref="X22:AA22"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="C8:Q8"/>
-    <mergeCell ref="R8:X8"/>
-    <mergeCell ref="Y8:AG8"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="Y31:Z31"/>
-    <mergeCell ref="Y32:Z32"/>
-    <mergeCell ref="Q34:U34"/>
-    <mergeCell ref="V34:X34"/>
-    <mergeCell ref="Y33:Z33"/>
-    <mergeCell ref="I34:L34"/>
-    <mergeCell ref="Q32:U32"/>
-    <mergeCell ref="V31:X31"/>
-    <mergeCell ref="Q31:U31"/>
-    <mergeCell ref="Q33:U33"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="Y34:Z34"/>
-    <mergeCell ref="O33:P33"/>
-    <mergeCell ref="C13:Q13"/>
-    <mergeCell ref="R13:X13"/>
-    <mergeCell ref="L23:P23"/>
-    <mergeCell ref="AB23:AD23"/>
-    <mergeCell ref="AA32:AC32"/>
-    <mergeCell ref="AA33:AC33"/>
-    <mergeCell ref="AA34:AC34"/>
-    <mergeCell ref="B54:O54"/>
-    <mergeCell ref="P54:AG54"/>
-    <mergeCell ref="B53:AG53"/>
-    <mergeCell ref="B14:AG14"/>
-    <mergeCell ref="Y15:AG15"/>
-    <mergeCell ref="B39:AG39"/>
-    <mergeCell ref="B40:AG40"/>
-    <mergeCell ref="B41:Q41"/>
-    <mergeCell ref="R41:AG41"/>
-    <mergeCell ref="B18:AG18"/>
-    <mergeCell ref="AD37:AG37"/>
-    <mergeCell ref="L21:P21"/>
-    <mergeCell ref="Q21:S21"/>
-    <mergeCell ref="C20:P20"/>
-    <mergeCell ref="Q20:W20"/>
-    <mergeCell ref="C15:M15"/>
-    <mergeCell ref="O15:T15"/>
-    <mergeCell ref="C16:Q16"/>
-    <mergeCell ref="R16:X16"/>
-    <mergeCell ref="Y16:AG16"/>
-    <mergeCell ref="AE23:AG23"/>
-    <mergeCell ref="B10:AG10"/>
-    <mergeCell ref="U12:X12"/>
-    <mergeCell ref="C12:M12"/>
-    <mergeCell ref="B19:AG19"/>
-    <mergeCell ref="B28:AG28"/>
-    <mergeCell ref="T21:W21"/>
-    <mergeCell ref="X21:AA21"/>
-    <mergeCell ref="U15:X15"/>
-    <mergeCell ref="AB21:AG21"/>
-    <mergeCell ref="X23:AA23"/>
-    <mergeCell ref="X20:AG20"/>
-    <mergeCell ref="C21:K21"/>
-    <mergeCell ref="O12:T12"/>
-    <mergeCell ref="Y12:AG12"/>
-    <mergeCell ref="Y13:AG13"/>
-    <mergeCell ref="C23:K23"/>
-    <mergeCell ref="L22:P22"/>
-    <mergeCell ref="Q22:S22"/>
-    <mergeCell ref="T22:W22"/>
-    <mergeCell ref="C26:AG26"/>
+    <mergeCell ref="AD46:AG46"/>
+    <mergeCell ref="R43:AG43"/>
+    <mergeCell ref="B43:Q43"/>
+    <mergeCell ref="F34:H34"/>
+    <mergeCell ref="AD35:AG35"/>
+    <mergeCell ref="V48:Y48"/>
+    <mergeCell ref="Z48:AC48"/>
+    <mergeCell ref="B48:Q48"/>
+    <mergeCell ref="B47:AG47"/>
+    <mergeCell ref="R48:U48"/>
+    <mergeCell ref="AD48:AG48"/>
+    <mergeCell ref="R46:U46"/>
+    <mergeCell ref="C36:H36"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="M34:N34"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -21398,15 +21401,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101001A44C1F890FCF34BA30D378D3367D63B" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="22c88173e6d2a076a971b39a2faa4e23">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="c039d5ce-a415-4a5e-b4fe-9520c78c43c3" xmlns:ns4="fcb16455-6622-4065-81a7-84fea1f9c666" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd62c2bcfd6751c569a4b8d22a7ba344" ns3:_="" ns4:_="">
     <xsd:import namespace="c039d5ce-a415-4a5e-b4fe-9520c78c43c3"/>
@@ -21629,6 +21623,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C2D343A-F610-42B3-83A0-EEB5E4786A2A}">
   <ds:schemaRefs>
@@ -21647,14 +21650,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1BA01D47-E7F6-48AD-8D5C-202680BAB15C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F489C8EF-CFF0-4606-955D-42F7AEA2B205}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21671,4 +21666,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1BA01D47-E7F6-48AD-8D5C-202680BAB15C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>